<commit_message>
Replace level labels with short long grading
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R4bb2ba3077784b02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R3ddea33a460049b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R2e7faac942bd401b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R2761e4f9b18e4adf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R23b78aa8a8934922"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R296f53f9c8ec4d51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R98ee0eb291cf4553"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R99062d4d8ede46b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="Rb07f432cc8594e66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R66cf1f1ee91145f1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -409,7 +409,7 @@
         <x:v>本文量</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>Shortは現Level 3程度、Longは現Level 7程度の長さを目安にする。</x:v>
+        <x:v>Shortは120〜180語程度。Longは300〜450語程度。UIでは旧段階表記を使わない。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -507,7 +507,7 @@
         <x:v>Short / Long</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>Short=現Level 3程度、Long=現Level 7程度</x:v>
+        <x:v>Short=120〜180語程度、Long=300〜450語程度</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1699,7 +1699,7 @@
         <x:v>本文量</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>{Length} で生成する。Shortは現Level 3程度、Longは現Level 7程度。</x:v>
+        <x:v>{Length} で生成する。Shortは120〜180語程度、Longは300〜450語程度。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Limit current ID story choices
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R296f53f9c8ec4d51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R98ee0eb291cf4553"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R99062d4d8ede46b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="Rb07f432cc8594e66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R66cf1f1ee91145f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Re5edc6c366894813"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rc431e28711a449b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R5fce22f7ae214692"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R215e52bda3e34f43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Rf019b09489bf4d1f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -401,7 +401,7 @@
         <x:v>候補表示</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>サイトでは選択したCurrent ID以下の直近10 IDに紐づくコンテンツを表示する。</x:v>
+        <x:v>サイトでは選択したCurrent ID以下の近いIDに紐づくコンテンツを最大3件まで表示する。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Separate short and long ID mappings
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Re5edc6c366894813"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rc431e28711a449b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R5fce22f7ae214692"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R215e52bda3e34f43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Rf019b09489bf4d1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R9bb84a4c52df4b14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R5e8b368a759e495e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R7290b120924347e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="Re4d534de93d24415"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Rfecfba84cb4e421c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -357,18 +357,18 @@
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>Unified Current ID 方針</x:v>
+        <x:v>Unified ID 方針</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>Unified Current ID 方針</x:v>
+        <x:v>Unified ID 方針</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のCurrent IDを一本で指定する。本文量はShortとLongの二段階で選ぶ。</x:v>
+        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のIDを一本で指定する。本文量はShortとLongの二段階で選ぶ。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のCurrent IDを一本で指定する。本文量はShortとLongの二段階で選ぶ。</x:v>
+        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のIDを一本で指定する。本文量はShortとLongの二段階で選ぶ。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -382,10 +382,10 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>Current ID</x:v>
+        <x:v>ID</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>GDMとNHを別々に指定しない。ひとつのCurrent IDだけを指定する。</x:v>
+        <x:v>GDMとNHを別々に指定しない。ひとつのIDだけを指定する。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -401,7 +401,7 @@
         <x:v>候補表示</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>サイトでは選択したCurrent ID以下の近いIDに紐づくコンテンツを最大3件まで表示する。</x:v>
+        <x:v>サイトでは選択したID以下の近いIDに紐づくコンテンツを最大3件まで表示する。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -417,7 +417,7 @@
         <x:v>注意</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>既存本文を新しいID体系へ紐づけ直した表。個別IDの必須語・文法を完全反映する新作本文は今後追加する。</x:v>
+        <x:v>ShortとLongは別IDへ紐づける。個別IDの必須語・文法を完全反映する新作本文は今後追加する。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -455,16 +455,16 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>本文生成時に使う入力欄。Current IDは1つだけ指定し、LengthでShort/Longを選ぶ。</x:v>
+        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、LengthでShort/Longを選ぶ。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>本文生成時に使う入力欄。Current IDは1つだけ指定し、LengthでShort/Longを選ぶ。</x:v>
+        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、LengthでShort/Longを選ぶ。</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>本文生成時に使う入力欄。Current IDは1つだけ指定し、LengthでShort/Longを選ぶ。</x:v>
+        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、LengthでShort/Longを選ぶ。</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>本文生成時に使う入力欄。Current IDは1つだけ指定し、LengthでShort/Longを選ぶ。</x:v>
+        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、LengthでShort/Longを選ぶ。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -484,13 +484,13 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>Current ID</x:v>
+        <x:v>ID</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
         <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>Unified_ProgressのCurrent IDから選ぶ</x:v>
+        <x:v>Unified_ProgressのIDから選ぶ</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
         <x:v>このIDまでのGDM/NH項目を使用可</x:v>
@@ -609,34 +609,34 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Current IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Current IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Current IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Current IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Current IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Current IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
       </x:c>
       <x:c r="G2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Current IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
       </x:c>
       <x:c r="H2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Current IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="16" t="str">
-        <x:v>Current ID</x:v>
+        <x:v>ID</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
         <x:v>Series</x:v>
@@ -1192,13 +1192,11 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="30" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="40" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="40" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="44" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
@@ -1220,64 +1218,46 @@
       <x:c r="F1" s="4" t="str">
         <x:v>Content Map</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
-        <x:v>Content Map</x:v>
-      </x:c>
-      <x:c r="H1" s="4" t="str">
-        <x:v>Content Map</x:v>
-      </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>既存本文を新Current IDへ紐づけ、Short/Longの二段階で選べるようにした表。</x:v>
+        <x:v>既存本文をIDへ紐づけ、Short/Longの二段階で選べるようにした表。ShortとLongは別IDで管理する。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>既存本文を新Current IDへ紐づけ、Short/Longの二段階で選べるようにした表。</x:v>
+        <x:v>既存本文をIDへ紐づけ、Short/Longの二段階で選べるようにした表。ShortとLongは別IDで管理する。</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>既存本文を新Current IDへ紐づけ、Short/Longの二段階で選べるようにした表。</x:v>
+        <x:v>既存本文をIDへ紐づけ、Short/Longの二段階で選べるようにした表。ShortとLongは別IDで管理する。</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>既存本文を新Current IDへ紐づけ、Short/Longの二段階で選べるようにした表。</x:v>
+        <x:v>既存本文をIDへ紐づけ、Short/Longの二段階で選べるようにした表。ShortとLongは別IDで管理する。</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>既存本文を新Current IDへ紐づけ、Short/Longの二段階で選べるようにした表。</x:v>
+        <x:v>既存本文をIDへ紐づけ、Short/Longの二段階で選べるようにした表。ShortとLongは別IDで管理する。</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
-        <x:v>既存本文を新Current IDへ紐づけ、Short/Longの二段階で選べるようにした表。</x:v>
-      </x:c>
-      <x:c r="G2" s="7" t="str">
-        <x:v>既存本文を新Current IDへ紐づけ、Short/Longの二段階で選べるようにした表。</x:v>
-      </x:c>
-      <x:c r="H2" s="7" t="str">
-        <x:v>既存本文を新Current IDへ紐づけ、Short/Longの二段階で選べるようにした表。</x:v>
+        <x:v>既存本文をIDへ紐づけ、Short/Longの二段階で選べるようにした表。ShortとLongは別IDで管理する。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="16" t="str">
-        <x:v>Current ID</x:v>
+        <x:v>ID</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
+        <x:v>Length</x:v>
+      </x:c>
+      <x:c r="C4" s="16" t="str">
         <x:v>Genre</x:v>
       </x:c>
-      <x:c r="C4" s="16" t="str">
+      <x:c r="D4" s="16" t="str">
         <x:v>Title</x:v>
       </x:c>
-      <x:c r="D4" s="16" t="str">
+      <x:c r="E4" s="16" t="str">
         <x:v>Slug</x:v>
       </x:c>
-      <x:c r="E4" s="16" t="str">
-        <x:v>Short Label</x:v>
-      </x:c>
       <x:c r="F4" s="16" t="str">
-        <x:v>Short Text</x:v>
-      </x:c>
-      <x:c r="G4" s="16" t="str">
-        <x:v>Long Label</x:v>
-      </x:c>
-      <x:c r="H4" s="16" t="str">
-        <x:v>Long Text</x:v>
+        <x:v>Text</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -1285,25 +1265,19 @@
         <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="str">
         <x:v>Mystery</x:v>
       </x:c>
-      <x:c r="C5" s="12" t="str">
+      <x:c r="D5" s="12" t="str">
         <x:v>The Little Door</x:v>
       </x:c>
-      <x:c r="D5" s="12" t="str">
+      <x:c r="E5" s="12" t="str">
         <x:v>graded-story</x:v>
-      </x:c>
-      <x:c r="E5" s="12" t="str">
-        <x:v>Short</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
         <x:v>lessons/graded-story/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G5" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H5" s="12" t="str">
-        <x:v>lessons/graded-story/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1311,25 +1285,19 @@
         <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="str">
         <x:v>Human Drama</x:v>
       </x:c>
-      <x:c r="C6" s="12" t="str">
+      <x:c r="D6" s="12" t="str">
         <x:v>The Quiet Bread Shop</x:v>
       </x:c>
-      <x:c r="D6" s="12" t="str">
+      <x:c r="E6" s="12" t="str">
         <x:v>bread-shop</x:v>
-      </x:c>
-      <x:c r="E6" s="12" t="str">
-        <x:v>Short</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
         <x:v>lessons/bread-shop/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G6" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H6" s="12" t="str">
-        <x:v>lessons/bread-shop/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1337,25 +1305,19 @@
         <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C7" s="12" t="str">
         <x:v>SF</x:v>
       </x:c>
-      <x:c r="C7" s="12" t="str">
+      <x:c r="D7" s="12" t="str">
         <x:v>The Star Bus</x:v>
       </x:c>
-      <x:c r="D7" s="12" t="str">
+      <x:c r="E7" s="12" t="str">
         <x:v>star-bus</x:v>
-      </x:c>
-      <x:c r="E7" s="12" t="str">
-        <x:v>Short</x:v>
       </x:c>
       <x:c r="F7" s="12" t="str">
         <x:v>lessons/star-bus/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G7" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H7" s="12" t="str">
-        <x:v>lessons/star-bus/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -1363,25 +1325,19 @@
         <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C8" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
-      <x:c r="C8" s="12" t="str">
+      <x:c r="D8" s="12" t="str">
         <x:v>The Wrong Robot</x:v>
       </x:c>
-      <x:c r="D8" s="12" t="str">
+      <x:c r="E8" s="12" t="str">
         <x:v>wrong-robot</x:v>
-      </x:c>
-      <x:c r="E8" s="12" t="str">
-        <x:v>Short</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
         <x:v>lessons/wrong-robot/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G8" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H8" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1389,25 +1345,19 @@
         <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="str">
         <x:v>Fantasy</x:v>
       </x:c>
-      <x:c r="C9" s="12" t="str">
+      <x:c r="D9" s="12" t="str">
         <x:v>The Moon Cup</x:v>
       </x:c>
-      <x:c r="D9" s="12" t="str">
+      <x:c r="E9" s="12" t="str">
         <x:v>moon-cup</x:v>
-      </x:c>
-      <x:c r="E9" s="12" t="str">
-        <x:v>Short</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
         <x:v>lessons/moon-cup/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G9" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H9" s="12" t="str">
-        <x:v>lessons/moon-cup/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1415,24 +1365,18 @@
         <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C10" s="12" t="str">
         <x:v>Human Drama</x:v>
       </x:c>
-      <x:c r="C10" s="12" t="str">
+      <x:c r="D10" s="12" t="str">
         <x:v>The Quiet Bread Shop</x:v>
       </x:c>
-      <x:c r="D10" s="12" t="str">
+      <x:c r="E10" s="12" t="str">
         <x:v>bread-shop</x:v>
       </x:c>
-      <x:c r="E10" s="12" t="str">
-        <x:v>Short</x:v>
-      </x:c>
       <x:c r="F10" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G10" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H10" s="12" t="str">
         <x:v>lessons/bread-shop/level-7.txt</x:v>
       </x:c>
     </x:row>
@@ -1441,24 +1385,18 @@
         <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C11" s="12" t="str">
         <x:v>Mystery</x:v>
       </x:c>
-      <x:c r="C11" s="12" t="str">
+      <x:c r="D11" s="12" t="str">
         <x:v>The Little Door</x:v>
       </x:c>
-      <x:c r="D11" s="12" t="str">
+      <x:c r="E11" s="12" t="str">
         <x:v>graded-story</x:v>
       </x:c>
-      <x:c r="E11" s="12" t="str">
-        <x:v>Short</x:v>
-      </x:c>
       <x:c r="F11" s="12" t="str">
-        <x:v>lessons/graded-story/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G11" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H11" s="12" t="str">
         <x:v>lessons/graded-story/level-7.txt</x:v>
       </x:c>
     </x:row>
@@ -1467,25 +1405,19 @@
         <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C12" s="12" t="str">
         <x:v>Human Drama</x:v>
       </x:c>
-      <x:c r="C12" s="12" t="str">
+      <x:c r="D12" s="12" t="str">
         <x:v>The Quiet Bread Shop</x:v>
       </x:c>
-      <x:c r="D12" s="12" t="str">
+      <x:c r="E12" s="12" t="str">
         <x:v>bread-shop</x:v>
-      </x:c>
-      <x:c r="E12" s="12" t="str">
-        <x:v>Short</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
         <x:v>lessons/bread-shop/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G12" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H12" s="12" t="str">
-        <x:v>lessons/bread-shop/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -1493,25 +1425,19 @@
         <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C13" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
-      <x:c r="C13" s="12" t="str">
+      <x:c r="D13" s="12" t="str">
         <x:v>The Wrong Robot</x:v>
       </x:c>
-      <x:c r="D13" s="12" t="str">
+      <x:c r="E13" s="12" t="str">
         <x:v>wrong-robot</x:v>
-      </x:c>
-      <x:c r="E13" s="12" t="str">
-        <x:v>Short</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
         <x:v>lessons/wrong-robot/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G13" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H13" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -1519,24 +1445,18 @@
         <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="str">
         <x:v>SF</x:v>
       </x:c>
-      <x:c r="C14" s="12" t="str">
+      <x:c r="D14" s="12" t="str">
         <x:v>The Star Bus</x:v>
       </x:c>
-      <x:c r="D14" s="12" t="str">
+      <x:c r="E14" s="12" t="str">
         <x:v>star-bus</x:v>
       </x:c>
-      <x:c r="E14" s="12" t="str">
-        <x:v>Short</x:v>
-      </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>lessons/star-bus/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G14" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H14" s="12" t="str">
         <x:v>lessons/star-bus/level-7.txt</x:v>
       </x:c>
     </x:row>
@@ -1545,24 +1465,18 @@
         <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="str">
         <x:v>Mystery</x:v>
       </x:c>
-      <x:c r="C15" s="12" t="str">
+      <x:c r="D15" s="12" t="str">
         <x:v>The Little Door</x:v>
       </x:c>
-      <x:c r="D15" s="12" t="str">
+      <x:c r="E15" s="12" t="str">
         <x:v>graded-story</x:v>
       </x:c>
-      <x:c r="E15" s="12" t="str">
-        <x:v>Short</x:v>
-      </x:c>
       <x:c r="F15" s="12" t="str">
-        <x:v>lessons/graded-story/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G15" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H15" s="12" t="str">
         <x:v>lessons/graded-story/level-7.txt</x:v>
       </x:c>
     </x:row>
@@ -1571,25 +1485,19 @@
         <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="str">
         <x:v>Fantasy</x:v>
       </x:c>
-      <x:c r="C16" s="12" t="str">
+      <x:c r="D16" s="12" t="str">
         <x:v>The Moon Cup</x:v>
       </x:c>
-      <x:c r="D16" s="12" t="str">
+      <x:c r="E16" s="12" t="str">
         <x:v>moon-cup</x:v>
-      </x:c>
-      <x:c r="E16" s="12" t="str">
-        <x:v>Short</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
         <x:v>lessons/moon-cup/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G16" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H16" s="12" t="str">
-        <x:v>lessons/moon-cup/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -1597,25 +1505,19 @@
         <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C17" s="12" t="str">
         <x:v>Human Drama</x:v>
       </x:c>
-      <x:c r="C17" s="12" t="str">
+      <x:c r="D17" s="12" t="str">
         <x:v>The Quiet Bread Shop</x:v>
       </x:c>
-      <x:c r="D17" s="12" t="str">
+      <x:c r="E17" s="12" t="str">
         <x:v>bread-shop</x:v>
-      </x:c>
-      <x:c r="E17" s="12" t="str">
-        <x:v>Short</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
         <x:v>lessons/bread-shop/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G17" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H17" s="12" t="str">
-        <x:v>lessons/bread-shop/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -1623,31 +1525,25 @@
         <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C18" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
-      <x:c r="C18" s="12" t="str">
+      <x:c r="D18" s="12" t="str">
         <x:v>The Wrong Robot</x:v>
       </x:c>
-      <x:c r="D18" s="12" t="str">
+      <x:c r="E18" s="12" t="str">
         <x:v>wrong-robot</x:v>
       </x:c>
-      <x:c r="E18" s="12" t="str">
-        <x:v>Short</x:v>
-      </x:c>
       <x:c r="F18" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-3.txt</x:v>
-      </x:c>
-      <x:c r="G18" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="H18" s="12" t="str">
         <x:v>lessons/wrong-robot/level-7.txt</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1671,10 +1567,10 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>生成時はCurrent IDを1つだけ使い、本文量をShort/Longで指定する。</x:v>
+        <x:v>生成時はIDを1つだけ使い、本文量をShort/Longで指定する。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>生成時はCurrent IDを1つだけ使い、本文量をShort/Longで指定する。</x:v>
+        <x:v>生成時はIDを1つだけ使い、本文量をShort/Longで指定する。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -1691,7 +1587,7 @@
         <x:v>生成指示</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>Current IDは {Current ID}。GDM-41-10まではGDMを使い、以降はNH1/NH2の進行順に沿って、このIDまでの語彙・文法を使用する。</x:v>
+        <x:v>IDは {ID}。GDM-41-10まではGDMを使い、以降はNH1/NH2の進行順に沿って、このIDまでの語彙・文法を使用する。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1707,7 +1603,7 @@
         <x:v>必須項目</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>指定されたCurrent IDそのものの導入語・文法は本文に必ず自然に入れる。</x:v>
+        <x:v>指定されたIDそのものの導入語・文法は本文に必ず自然に入れる。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -1723,7 +1619,7 @@
         <x:v>出力</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Title / Current ID / Length / Genre / English text / used target items memo</x:v>
+        <x:v>Title / ID / Length / Genre / English text / used target items memo</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add targeted ID reading stories
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R9bb84a4c52df4b14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R5e8b368a759e495e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R7290b120924347e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="Re4d534de93d24415"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Rfecfba84cb4e421c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Rccdff05856cd4fc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rc79f0606aa1341de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R1761c59f93c34b5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="Rb1680888fa404e98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Rd38a19bd4d77481e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1262,7 +1262,7 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
         <x:v>Short</x:v>
@@ -1271,273 +1271,473 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>The Little Door</x:v>
+        <x:v>The Red Pin</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>graded-story</x:v>
+        <x:v>red-pin</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
-        <x:v>lessons/graded-story/level-3.txt</x:v>
+        <x:v>lessons/red-pin/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>GDM-10</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Book Under the Hat</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>book-under-hat</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/book-under-hat/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>GDM-22</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>The Star Bus</x:v>
+        <x:v>The Water Pen Trick</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
-        <x:v>star-bus</x:v>
+        <x:v>water-pen-trick</x:v>
       </x:c>
       <x:c r="F7" s="12" t="str">
-        <x:v>lessons/star-bus/level-3.txt</x:v>
+        <x:v>lessons/water-pen-trick/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>GDM-37-4</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
+        <x:v>Where Is the Bell?</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>wrong-robot</x:v>
+        <x:v>where-is-the-bell</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-3.txt</x:v>
+        <x:v>lessons/where-is-the-bell/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
-        <x:v>The Moon Cup</x:v>
+        <x:v>The Little Door</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>moon-cup</x:v>
+        <x:v>graded-story</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
-        <x:v>lessons/moon-cup/level-3.txt</x:v>
+        <x:v>lessons/graded-story/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH1-0-FAMILY</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C10" s="12" t="str">
         <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>Rina's Brother</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>rina-brother</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
-        <x:v>lessons/bread-shop/level-7.txt</x:v>
+        <x:v>lessons/rina-brother/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>The Little Door</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>graded-story</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
-        <x:v>lessons/graded-story/level-7.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
         <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Rainy Club Map</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>rainy-club-map</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
+        <x:v>The Star Bus</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>wrong-robot</x:v>
+        <x:v>star-bus</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-3.txt</x:v>
+        <x:v>lessons/star-bus/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C14" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>The Star Bus</x:v>
+        <x:v>Can the Clock Sing?</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
-        <x:v>star-bus</x:v>
+        <x:v>can-clock-sing</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>lessons/star-bus/level-7.txt</x:v>
+        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C15" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>The Little Door</x:v>
+        <x:v>The Wrong Robot</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>graded-story</x:v>
+        <x:v>wrong-robot</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
-        <x:v>lessons/graded-story/level-7.txt</x:v>
+        <x:v>lessons/wrong-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>The Moon Cup</x:v>
+        <x:v>Don't Be a Hero</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>moon-cup</x:v>
+        <x:v>dont-be-a-hero</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>lessons/moon-cup/level-3.txt</x:v>
+        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Window Note</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>window-note</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/window-note/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
+        <x:v>NH1-1-8-3-WHY</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C18" s="12" t="str">
+        <x:v>Fantasy</x:v>
+      </x:c>
+      <x:c r="D18" s="12" t="str">
+        <x:v>The Moon Cup</x:v>
+      </x:c>
+      <x:c r="E18" s="12" t="str">
+        <x:v>moon-cup</x:v>
+      </x:c>
+      <x:c r="F18" s="12" t="str">
+        <x:v>lessons/moon-cup/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="12" t="str">
+        <x:v>NH1-1-10-V</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C19" s="12" t="str">
+        <x:v>Human Drama</x:v>
+      </x:c>
+      <x:c r="D19" s="12" t="str">
+        <x:v>The Rainy Club Map</x:v>
+      </x:c>
+      <x:c r="E19" s="12" t="str">
+        <x:v>rainy-club-map</x:v>
+      </x:c>
+      <x:c r="F19" s="12" t="str">
+        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="12" t="str">
+        <x:v>NH1-1-11-1-MAYBE</x:v>
+      </x:c>
+      <x:c r="B20" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C20" s="12" t="str">
+        <x:v>Fantasy</x:v>
+      </x:c>
+      <x:c r="D20" s="12" t="str">
+        <x:v>Can the Clock Sing?</x:v>
+      </x:c>
+      <x:c r="E20" s="12" t="str">
+        <x:v>can-clock-sing</x:v>
+      </x:c>
+      <x:c r="F20" s="12" t="str">
+        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="12" t="str">
+        <x:v>NH2-2-1-3-SVOO</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C21" s="12" t="str">
+        <x:v>Human Drama</x:v>
+      </x:c>
+      <x:c r="D21" s="12" t="str">
+        <x:v>The Quiet Bread Shop</x:v>
+      </x:c>
+      <x:c r="E21" s="12" t="str">
+        <x:v>bread-shop</x:v>
+      </x:c>
+      <x:c r="F21" s="12" t="str">
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="12" t="str">
+        <x:v>NH2-2-1-3-SVOO</x:v>
+      </x:c>
+      <x:c r="B22" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C22" s="12" t="str">
+        <x:v>Comedy</x:v>
+      </x:c>
+      <x:c r="D22" s="12" t="str">
+        <x:v>The Gift Lesson</x:v>
+      </x:c>
+      <x:c r="E22" s="12" t="str">
+        <x:v>gift-lesson</x:v>
+      </x:c>
+      <x:c r="F22" s="12" t="str">
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="12" t="str">
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
+      </x:c>
+      <x:c r="B23" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C23" s="12" t="str">
+        <x:v>Comedy</x:v>
+      </x:c>
+      <x:c r="D23" s="12" t="str">
+        <x:v>The Wrong Robot</x:v>
+      </x:c>
+      <x:c r="E23" s="12" t="str">
+        <x:v>wrong-robot</x:v>
+      </x:c>
+      <x:c r="F23" s="12" t="str">
+        <x:v>lessons/wrong-robot/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="12" t="str">
+        <x:v>NH2-2-3-1-SHOULD</x:v>
+      </x:c>
+      <x:c r="B24" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C24" s="12" t="str">
+        <x:v>Human Drama</x:v>
+      </x:c>
+      <x:c r="D24" s="12" t="str">
+        <x:v>Don't Be a Hero</x:v>
+      </x:c>
+      <x:c r="E24" s="12" t="str">
+        <x:v>dont-be-a-hero</x:v>
+      </x:c>
+      <x:c r="F24" s="12" t="str">
+        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="12" t="str">
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+      </x:c>
+      <x:c r="B25" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C25" s="12" t="str">
+        <x:v>Comedy</x:v>
+      </x:c>
+      <x:c r="D25" s="12" t="str">
+        <x:v>The Gift Lesson</x:v>
+      </x:c>
+      <x:c r="E25" s="12" t="str">
+        <x:v>gift-lesson</x:v>
+      </x:c>
+      <x:c r="F25" s="12" t="str">
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="12" t="str">
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
+      </x:c>
+      <x:c r="B26" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C26" s="12" t="str">
+        <x:v>Fantasy</x:v>
+      </x:c>
+      <x:c r="D26" s="12" t="str">
+        <x:v>The Moon Cup</x:v>
+      </x:c>
+      <x:c r="E26" s="12" t="str">
+        <x:v>moon-cup</x:v>
+      </x:c>
+      <x:c r="F26" s="12" t="str">
+        <x:v>lessons/moon-cup/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="12" t="str">
+        <x:v>NH2-2-6-MORE-THAN</x:v>
+      </x:c>
+      <x:c r="B27" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C27" s="12" t="str">
+        <x:v>Human Drama</x:v>
+      </x:c>
+      <x:c r="D27" s="12" t="str">
+        <x:v>The Quiet Bread Shop</x:v>
+      </x:c>
+      <x:c r="E27" s="12" t="str">
+        <x:v>bread-shop</x:v>
+      </x:c>
+      <x:c r="F27" s="12" t="str">
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="12" t="str">
         <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
-      <x:c r="B18" s="12" t="str">
+      <x:c r="B28" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
-      <x:c r="C18" s="12" t="str">
+      <x:c r="C28" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
-      <x:c r="D18" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
-      </x:c>
-      <x:c r="E18" s="12" t="str">
-        <x:v>wrong-robot</x:v>
-      </x:c>
-      <x:c r="F18" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-7.txt</x:v>
+      <x:c r="D28" s="12" t="str">
+        <x:v>The Gift Lesson</x:v>
+      </x:c>
+      <x:c r="E28" s="12" t="str">
+        <x:v>gift-lesson</x:v>
+      </x:c>
+      <x:c r="F28" s="12" t="str">
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add missing ID reading stories
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Rccdff05856cd4fc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rc79f0606aa1341de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R1761c59f93c34b5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="Rb1680888fa404e98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Rd38a19bd4d77481e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R99e59abc4ccc498e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R0d3a920a5fe24f6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R8c57e277dd734d6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R0423358a94894fc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R5f832522382d4889"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1740,6 +1740,406 @@
         <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="12" t="str">
+        <x:v>GDM-1</x:v>
+      </x:c>
+      <x:c r="B29" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C29" s="12" t="str">
+        <x:v>Comedy</x:v>
+      </x:c>
+      <x:c r="D29" s="12" t="str">
+        <x:v>The Red Pin Parade</x:v>
+      </x:c>
+      <x:c r="E29" s="12" t="str">
+        <x:v>red-pin-parade</x:v>
+      </x:c>
+      <x:c r="F29" s="12" t="str">
+        <x:v>lessons/red-pin-parade/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="12" t="str">
+        <x:v>GDM-10</x:v>
+      </x:c>
+      <x:c r="B30" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C30" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D30" s="12" t="str">
+        <x:v>The Old Book Signal</x:v>
+      </x:c>
+      <x:c r="E30" s="12" t="str">
+        <x:v>old-book-signal</x:v>
+      </x:c>
+      <x:c r="F30" s="12" t="str">
+        <x:v>lessons/old-book-signal/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="A31" s="12" t="str">
+        <x:v>GDM-22</x:v>
+      </x:c>
+      <x:c r="B31" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C31" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D31" s="12" t="str">
+        <x:v>The Pens in the Water</x:v>
+      </x:c>
+      <x:c r="E31" s="12" t="str">
+        <x:v>pens-in-water</x:v>
+      </x:c>
+      <x:c r="F31" s="12" t="str">
+        <x:v>lessons/pens-in-water/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" s="12" t="str">
+        <x:v>GDM-37-4</x:v>
+      </x:c>
+      <x:c r="B32" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C32" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D32" s="12" t="str">
+        <x:v>The Map Under the Stage</x:v>
+      </x:c>
+      <x:c r="E32" s="12" t="str">
+        <x:v>map-under-stage</x:v>
+      </x:c>
+      <x:c r="F32" s="12" t="str">
+        <x:v>lessons/map-under-stage/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="12" t="str">
+        <x:v>GDM-41-10</x:v>
+      </x:c>
+      <x:c r="B33" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C33" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D33" s="12" t="str">
+        <x:v>The Door Under the Stage</x:v>
+      </x:c>
+      <x:c r="E33" s="12" t="str">
+        <x:v>door-under-stage</x:v>
+      </x:c>
+      <x:c r="F33" s="12" t="str">
+        <x:v>lessons/door-under-stage/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="A34" s="12" t="str">
+        <x:v>NH1-0-FAMILY</x:v>
+      </x:c>
+      <x:c r="B34" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C34" s="12" t="str">
+        <x:v>Human Drama</x:v>
+      </x:c>
+      <x:c r="D34" s="12" t="str">
+        <x:v>Family Photo Day</x:v>
+      </x:c>
+      <x:c r="E34" s="12" t="str">
+        <x:v>family-photo-day</x:v>
+      </x:c>
+      <x:c r="F34" s="12" t="str">
+        <x:v>lessons/family-photo-day/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="15" hidden="0" customHeight="1">
+      <x:c r="A35" s="12" t="str">
+        <x:v>NH1-1-6-V</x:v>
+      </x:c>
+      <x:c r="B35" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C35" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D35" s="12" t="str">
+        <x:v>The Letter Under the Door</x:v>
+      </x:c>
+      <x:c r="E35" s="12" t="str">
+        <x:v>letter-under-door</x:v>
+      </x:c>
+      <x:c r="F35" s="12" t="str">
+        <x:v>lessons/letter-under-door/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
+      <x:c r="A36" s="12" t="str">
+        <x:v>NH1-1-8-3-WHY</x:v>
+      </x:c>
+      <x:c r="B36" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C36" s="12" t="str">
+        <x:v>SF</x:v>
+      </x:c>
+      <x:c r="D36" s="12" t="str">
+        <x:v>Why the Lights Blink</x:v>
+      </x:c>
+      <x:c r="E36" s="12" t="str">
+        <x:v>why-lights-blink</x:v>
+      </x:c>
+      <x:c r="F36" s="12" t="str">
+        <x:v>lessons/why-lights-blink/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="A37" s="12" t="str">
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
+      </x:c>
+      <x:c r="B37" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C37" s="12" t="str">
+        <x:v>Comedy</x:v>
+      </x:c>
+      <x:c r="D37" s="12" t="str">
+        <x:v>Because of the Soup</x:v>
+      </x:c>
+      <x:c r="E37" s="12" t="str">
+        <x:v>because-of-soup</x:v>
+      </x:c>
+      <x:c r="F37" s="12" t="str">
+        <x:v>lessons/because-of-soup/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
+      <x:c r="A38" s="12" t="str">
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
+      </x:c>
+      <x:c r="B38" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C38" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D38" s="12" t="str">
+        <x:v>How to Open the Box</x:v>
+      </x:c>
+      <x:c r="E38" s="12" t="str">
+        <x:v>open-the-box</x:v>
+      </x:c>
+      <x:c r="F38" s="12" t="str">
+        <x:v>lessons/open-the-box/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="15" hidden="0" customHeight="1">
+      <x:c r="A39" s="12" t="str">
+        <x:v>NH2-2-6-MORE-THAN</x:v>
+      </x:c>
+      <x:c r="B39" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C39" s="12" t="str">
+        <x:v>Human Drama</x:v>
+      </x:c>
+      <x:c r="D39" s="12" t="str">
+        <x:v>More Than Half</x:v>
+      </x:c>
+      <x:c r="E39" s="12" t="str">
+        <x:v>more-than-half</x:v>
+      </x:c>
+      <x:c r="F39" s="12" t="str">
+        <x:v>lessons/more-than-half/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="15" hidden="0" customHeight="1">
+      <x:c r="A40" s="12" t="str">
+        <x:v>NH1-1-10-V</x:v>
+      </x:c>
+      <x:c r="B40" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C40" s="12" t="str">
+        <x:v>Human Drama</x:v>
+      </x:c>
+      <x:c r="D40" s="12" t="str">
+        <x:v>The Travel Ticket</x:v>
+      </x:c>
+      <x:c r="E40" s="12" t="str">
+        <x:v>travel-ticket</x:v>
+      </x:c>
+      <x:c r="F40" s="12" t="str">
+        <x:v>lessons/travel-ticket/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="15" hidden="0" customHeight="1">
+      <x:c r="A41" s="12" t="str">
+        <x:v>NH1-1-11-1-MAYBE</x:v>
+      </x:c>
+      <x:c r="B41" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C41" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D41" s="12" t="str">
+        <x:v>Maybe at the Window</x:v>
+      </x:c>
+      <x:c r="E41" s="12" t="str">
+        <x:v>maybe-window</x:v>
+      </x:c>
+      <x:c r="F41" s="12" t="str">
+        <x:v>lessons/maybe-window/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="15" hidden="0" customHeight="1">
+      <x:c r="A42" s="12" t="str">
+        <x:v>NH2-2-3-1-SHOULD</x:v>
+      </x:c>
+      <x:c r="B42" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C42" s="12" t="str">
+        <x:v>Comedy</x:v>
+      </x:c>
+      <x:c r="D42" s="12" t="str">
+        <x:v>The Should Sign</x:v>
+      </x:c>
+      <x:c r="E42" s="12" t="str">
+        <x:v>should-sign</x:v>
+      </x:c>
+      <x:c r="F42" s="12" t="str">
+        <x:v>lessons/should-sign/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="15" hidden="0" customHeight="1">
+      <x:c r="A43" s="12" t="str">
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+      </x:c>
+      <x:c r="B43" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C43" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D43" s="12" t="str">
+        <x:v>The Have-To Key</x:v>
+      </x:c>
+      <x:c r="E43" s="12" t="str">
+        <x:v>have-to-key</x:v>
+      </x:c>
+      <x:c r="F43" s="12" t="str">
+        <x:v>lessons/have-to-key/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="15" hidden="0" customHeight="1">
+      <x:c r="A44" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B44" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C44" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D44" s="12" t="str">
+        <x:v>The Poster Was Moved</x:v>
+      </x:c>
+      <x:c r="E44" s="12" t="str">
+        <x:v>passive-poster</x:v>
+      </x:c>
+      <x:c r="F44" s="12" t="str">
+        <x:v>lessons/passive-poster/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="15" hidden="0" customHeight="1">
+      <x:c r="A45" s="12" t="str">
+        <x:v>NH1-1-1-V</x:v>
+      </x:c>
+      <x:c r="B45" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C45" s="12" t="str">
+        <x:v>Comedy</x:v>
+      </x:c>
+      <x:c r="D45" s="12" t="str">
+        <x:v>The Drink and Read Race</x:v>
+      </x:c>
+      <x:c r="E45" s="12" t="str">
+        <x:v>drink-read-race</x:v>
+      </x:c>
+      <x:c r="F45" s="12" t="str">
+        <x:v>lessons/drink-read-race/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="15" hidden="0" customHeight="1">
+      <x:c r="A46" s="12" t="str">
+        <x:v>NH1-1-3-CAN-Q</x:v>
+      </x:c>
+      <x:c r="B46" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C46" s="12" t="str">
+        <x:v>Fantasy</x:v>
+      </x:c>
+      <x:c r="D46" s="12" t="str">
+        <x:v>Can the Lantern Fly?</x:v>
+      </x:c>
+      <x:c r="E46" s="12" t="str">
+        <x:v>can-lantern</x:v>
+      </x:c>
+      <x:c r="F46" s="12" t="str">
+        <x:v>lessons/can-lantern/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="15" hidden="0" customHeight="1">
+      <x:c r="A47" s="12" t="str">
+        <x:v>NH1-1-5-2-DONTBE</x:v>
+      </x:c>
+      <x:c r="B47" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C47" s="12" t="str">
+        <x:v>Human Drama</x:v>
+      </x:c>
+      <x:c r="D47" s="12" t="str">
+        <x:v>Don't Be Late</x:v>
+      </x:c>
+      <x:c r="E47" s="12" t="str">
+        <x:v>dont-be-late</x:v>
+      </x:c>
+      <x:c r="F47" s="12" t="str">
+        <x:v>lessons/dont-be-late/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="15" hidden="0" customHeight="1">
+      <x:c r="A48" s="12" t="str">
+        <x:v>NH2-2-1-3-SVOO</x:v>
+      </x:c>
+      <x:c r="B48" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C48" s="12" t="str">
+        <x:v>Comedy</x:v>
+      </x:c>
+      <x:c r="D48" s="12" t="str">
+        <x:v>Show Me the Seat</x:v>
+      </x:c>
+      <x:c r="E48" s="12" t="str">
+        <x:v>show-me-the-seat</x:v>
+      </x:c>
+      <x:c r="F48" s="12" t="str">
+        <x:v>lessons/show-me-the-seat/level-7.txt</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Add adventure genre coverage
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R99e59abc4ccc498e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R0d3a920a5fe24f6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R8c57e277dd734d6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R0423358a94894fc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R5f832522382d4889"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R8e17d541179642ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Ra1da358f21314ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="Rc025d71215f0459e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R1fe445edce4e4455"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R689d278dbf8a4649"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1748,7 +1748,7 @@
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
         <x:v>The Red Pin Parade</x:v>
@@ -1768,7 +1768,7 @@
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
         <x:v>The Old Book Signal</x:v>
@@ -1788,7 +1788,7 @@
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C31" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
         <x:v>The Pens in the Water</x:v>
@@ -1808,7 +1808,7 @@
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C32" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
         <x:v>The Map Under the Stage</x:v>
@@ -1828,7 +1828,7 @@
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C33" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D33" s="12" t="str">
         <x:v>The Door Under the Stage</x:v>
@@ -1848,7 +1848,7 @@
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C34" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
         <x:v>Family Photo Day</x:v>
@@ -1868,7 +1868,7 @@
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C35" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
         <x:v>The Letter Under the Door</x:v>
@@ -1888,7 +1888,7 @@
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C36" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
         <x:v>Why the Lights Blink</x:v>
@@ -1908,7 +1908,7 @@
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C37" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
         <x:v>Because of the Soup</x:v>
@@ -1928,7 +1928,7 @@
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C38" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
         <x:v>How to Open the Box</x:v>
@@ -1948,7 +1948,7 @@
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C39" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
         <x:v>More Than Half</x:v>
@@ -1968,7 +1968,7 @@
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C40" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
         <x:v>The Travel Ticket</x:v>
@@ -1988,7 +1988,7 @@
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C41" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
         <x:v>Maybe at the Window</x:v>
@@ -2008,7 +2008,7 @@
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C42" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
         <x:v>The Should Sign</x:v>
@@ -2028,7 +2028,7 @@
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C43" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
         <x:v>The Have-To Key</x:v>
@@ -2048,7 +2048,7 @@
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C44" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D44" s="12" t="str">
         <x:v>The Poster Was Moved</x:v>
@@ -2068,7 +2068,7 @@
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C45" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
         <x:v>The Drink and Read Race</x:v>
@@ -2088,7 +2088,7 @@
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C46" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
         <x:v>Can the Lantern Fly?</x:v>
@@ -2108,7 +2108,7 @@
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C47" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
         <x:v>Don't Be Late</x:v>
@@ -2128,7 +2128,7 @@
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C48" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
         <x:v>Show Me the Seat</x:v>

</xml_diff>

<commit_message>
Add five SF reading stories
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R8e17d541179642ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Ra1da358f21314ec5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="Rc025d71215f0459e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R1fe445edce4e4455"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R689d278dbf8a4649"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R67c24fa1a04d4416"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rc2dbed25defc4db5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R9777d663d18b4bf5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R4680476142674d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R7897c9c79e62402e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2140,6 +2140,106 @@
         <x:v>lessons/show-me-the-seat/level-7.txt</x:v>
       </x:c>
     </x:row>
+    <x:row r="49" ht="15" hidden="0" customHeight="1">
+      <x:c r="A49" s="12" t="str">
+        <x:v>GDM-22</x:v>
+      </x:c>
+      <x:c r="B49" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C49" s="12" t="str">
+        <x:v>SF</x:v>
+      </x:c>
+      <x:c r="D49" s="12" t="str">
+        <x:v>The Signal Under Water</x:v>
+      </x:c>
+      <x:c r="E49" s="12" t="str">
+        <x:v>signal-under-water</x:v>
+      </x:c>
+      <x:c r="F49" s="12" t="str">
+        <x:v>lessons/signal-under-water/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="15" hidden="0" customHeight="1">
+      <x:c r="A50" s="12" t="str">
+        <x:v>NH1-1-6-V</x:v>
+      </x:c>
+      <x:c r="B50" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C50" s="12" t="str">
+        <x:v>SF</x:v>
+      </x:c>
+      <x:c r="D50" s="12" t="str">
+        <x:v>The Orbit Note</x:v>
+      </x:c>
+      <x:c r="E50" s="12" t="str">
+        <x:v>orbit-note</x:v>
+      </x:c>
+      <x:c r="F50" s="12" t="str">
+        <x:v>lessons/orbit-note/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="15" hidden="0" customHeight="1">
+      <x:c r="A51" s="12" t="str">
+        <x:v>NH1-1-8-3-WHY</x:v>
+      </x:c>
+      <x:c r="B51" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C51" s="12" t="str">
+        <x:v>SF</x:v>
+      </x:c>
+      <x:c r="D51" s="12" t="str">
+        <x:v>Why the Moon Robot Stops</x:v>
+      </x:c>
+      <x:c r="E51" s="12" t="str">
+        <x:v>why-moon-robot</x:v>
+      </x:c>
+      <x:c r="F51" s="12" t="str">
+        <x:v>lessons/why-moon-robot/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="15" hidden="0" customHeight="1">
+      <x:c r="A52" s="12" t="str">
+        <x:v>NH1-1-11-1-MAYBE</x:v>
+      </x:c>
+      <x:c r="B52" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C52" s="12" t="str">
+        <x:v>SF</x:v>
+      </x:c>
+      <x:c r="D52" s="12" t="str">
+        <x:v>Maybe at the Mars Window</x:v>
+      </x:c>
+      <x:c r="E52" s="12" t="str">
+        <x:v>maybe-mars-window</x:v>
+      </x:c>
+      <x:c r="F52" s="12" t="str">
+        <x:v>lessons/maybe-mars-window/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="15" hidden="0" customHeight="1">
+      <x:c r="A53" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B53" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C53" s="12" t="str">
+        <x:v>SF</x:v>
+      </x:c>
+      <x:c r="D53" s="12" t="str">
+        <x:v>The Station Was Moved</x:v>
+      </x:c>
+      <x:c r="E53" s="12" t="str">
+        <x:v>station-was-moved</x:v>
+      </x:c>
+      <x:c r="F53" s="12" t="str">
+        <x:v>lessons/station-was-moved/level-7.txt</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Add five long mystery readings
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R67c24fa1a04d4416"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rc2dbed25defc4db5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R9777d663d18b4bf5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R4680476142674d6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R7897c9c79e62402e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R80ea6fe03eb74083"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R268f28e18bd045ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R2bf0896b9de3484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R6275c49f0dd34f4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R785af35ce8524cb5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2240,6 +2240,106 @@
         <x:v>lessons/station-was-moved/level-7.txt</x:v>
       </x:c>
     </x:row>
+    <x:row r="54" ht="15" hidden="0" customHeight="1">
+      <x:c r="A54" s="12" t="str">
+        <x:v>GDM-37-4</x:v>
+      </x:c>
+      <x:c r="B54" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C54" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D54" s="12" t="str">
+        <x:v>Where the Roof Door Opens</x:v>
+      </x:c>
+      <x:c r="E54" s="12" t="str">
+        <x:v>where-the-roof-door</x:v>
+      </x:c>
+      <x:c r="F54" s="12" t="str">
+        <x:v>lessons/where-the-roof-door/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="15" hidden="0" customHeight="1">
+      <x:c r="A55" s="12" t="str">
+        <x:v>NH1-1-10-V</x:v>
+      </x:c>
+      <x:c r="B55" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C55" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D55" s="12" t="str">
+        <x:v>The Traveling Shadow Ticket</x:v>
+      </x:c>
+      <x:c r="E55" s="12" t="str">
+        <x:v>traveling-shadow-ticket</x:v>
+      </x:c>
+      <x:c r="F55" s="12" t="str">
+        <x:v>lessons/traveling-shadow-ticket/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="24" hidden="0" customHeight="1">
+      <x:c r="A56" s="12" t="str">
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
+      </x:c>
+      <x:c r="B56" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C56" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D56" s="12" t="str">
+        <x:v>Because the Wall Listened</x:v>
+      </x:c>
+      <x:c r="E56" s="12" t="str">
+        <x:v>because-the-wall-listened</x:v>
+      </x:c>
+      <x:c r="F56" s="12" t="str">
+        <x:v>lessons/because-the-wall-listened/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="15" hidden="0" customHeight="1">
+      <x:c r="A57" s="12" t="str">
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
+      </x:c>
+      <x:c r="B57" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C57" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D57" s="12" t="str">
+        <x:v>How to Read the Stone</x:v>
+      </x:c>
+      <x:c r="E57" s="12" t="str">
+        <x:v>how-to-read-the-stone</x:v>
+      </x:c>
+      <x:c r="F57" s="12" t="str">
+        <x:v>lessons/how-to-read-the-stone/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="15" hidden="0" customHeight="1">
+      <x:c r="A58" s="12" t="str">
+        <x:v>NH2-2-6-MORE-THAN</x:v>
+      </x:c>
+      <x:c r="B58" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C58" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D58" s="12" t="str">
+        <x:v>More Than One Moon</x:v>
+      </x:c>
+      <x:c r="E58" s="12" t="str">
+        <x:v>more-than-one-moon</x:v>
+      </x:c>
+      <x:c r="F58" s="12" t="str">
+        <x:v>lessons/more-than-one-moon/level-7.txt</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Add very short and very long readings
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R80ea6fe03eb74083"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R268f28e18bd045ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R2bf0896b9de3484a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R6275c49f0dd34f4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R785af35ce8524cb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Rc1cebf0037454a22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rb10d647d399e46a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R36e46d12f7f447ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R8d95ff92a14b4d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R4b71513115af4cd0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -365,10 +365,10 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のIDを一本で指定する。本文量はShortとLongの二段階で選ぶ。</x:v>
+        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のIDを一本で指定する。本文量はVery Short / Short / Long / Very Longから選ぶ。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のIDを一本で指定する。本文量はShortとLongの二段階で選ぶ。</x:v>
+        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のIDを一本で指定する。本文量はVery Short / Short / Long / Very Longから選ぶ。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -409,7 +409,7 @@
         <x:v>本文量</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>Shortは120〜180語程度。Longは300〜450語程度。UIでは旧段階表記を使わない。</x:v>
+        <x:v>Very Shortはごく短い導入用。Shortは120〜180語程度。Longは300〜450語程度。Very Longは650〜900語程度。UIでは旧段階表記を使わない。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -417,7 +417,7 @@
         <x:v>注意</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>ShortとLongは別IDへ紐づける。個別IDの必須語・文法を完全反映する新作本文は今後追加する。</x:v>
+        <x:v>各Lengthは別IDへ紐づける。個別IDの必須語・文法を完全反映する新作本文は今後追加する。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -455,16 +455,16 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、LengthでShort/Longを選ぶ。</x:v>
+        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、Lengthで本文量を選ぶ。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、LengthでShort/Longを選ぶ。</x:v>
+        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、Lengthで本文量を選ぶ。</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、LengthでShort/Longを選ぶ。</x:v>
+        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、Lengthで本文量を選ぶ。</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、LengthでShort/Longを選ぶ。</x:v>
+        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、Lengthで本文量を選ぶ。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -496,7 +496,7 @@
         <x:v>このIDまでのGDM/NH項目を使用可</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+    <x:row r="6" ht="24" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
         <x:v>Length</x:v>
       </x:c>
@@ -504,10 +504,10 @@
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>Short / Long</x:v>
+        <x:v>Very Short / Short / Long / Very Long</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>Short=120〜180語程度、Long=300〜450語程度</x:v>
+        <x:v>Very Short=ごく短い導入、Short=120〜180語程度、Long=300〜450語程度、Very Long=650〜900語程度</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1221,22 +1221,22 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>既存本文をIDへ紐づけ、Short/Longの二段階で選べるようにした表。ShortとLongは別IDで管理する。</x:v>
+        <x:v>既存本文をIDへ紐づけ、Length別に選べるようにした表。LengthごとにIDで管理する。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>既存本文をIDへ紐づけ、Short/Longの二段階で選べるようにした表。ShortとLongは別IDで管理する。</x:v>
+        <x:v>既存本文をIDへ紐づけ、Length別に選べるようにした表。LengthごとにIDで管理する。</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>既存本文をIDへ紐づけ、Short/Longの二段階で選べるようにした表。ShortとLongは別IDで管理する。</x:v>
+        <x:v>既存本文をIDへ紐づけ、Length別に選べるようにした表。LengthごとにIDで管理する。</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>既存本文をIDへ紐づけ、Short/Longの二段階で選べるようにした表。ShortとLongは別IDで管理する。</x:v>
+        <x:v>既存本文をIDへ紐づけ、Length別に選べるようにした表。LengthごとにIDで管理する。</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>既存本文をIDへ紐づけ、Short/Longの二段階で選べるようにした表。ShortとLongは別IDで管理する。</x:v>
+        <x:v>既存本文をIDへ紐づけ、Length別に選べるようにした表。LengthごとにIDで管理する。</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
-        <x:v>既存本文をIDへ紐づけ、Short/Longの二段階で選べるようにした表。ShortとLongは別IDで管理する。</x:v>
+        <x:v>既存本文をIDへ紐づけ、Length別に選べるようにした表。LengthごとにIDで管理する。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -1265,384 +1265,384 @@
         <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Very Short</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>The Red Pin</x:v>
+        <x:v>The Little Door</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>red-pin</x:v>
+        <x:v>graded-story</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
-        <x:v>lessons/red-pin/level-3.txt</x:v>
+        <x:v>lessons/graded-story/level-1.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
-        <x:v>GDM-10</x:v>
+        <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Very Short</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>The Book Under the Hat</x:v>
+        <x:v>The Blue Lunch Box</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
-        <x:v>book-under-hat</x:v>
+        <x:v>blue-lunch-box</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
-        <x:v>lessons/book-under-hat/level-3.txt</x:v>
+        <x:v>lessons/blue-lunch-box/level-1.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Very Short</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>The Water Pen Trick</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
-        <x:v>water-pen-trick</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F7" s="12" t="str">
-        <x:v>lessons/water-pen-trick/level-3.txt</x:v>
+        <x:v>lessons/bread-shop/level-1.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Very Short</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>Where Is the Bell?</x:v>
+        <x:v>The Star Bus</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>where-is-the-bell</x:v>
+        <x:v>star-bus</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
-        <x:v>lessons/where-is-the-bell/level-3.txt</x:v>
+        <x:v>lessons/star-bus/level-1.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Very Short</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
-        <x:v>The Little Door</x:v>
+        <x:v>The Wrong Robot</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>graded-story</x:v>
+        <x:v>wrong-robot</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
-        <x:v>lessons/graded-story/level-3.txt</x:v>
+        <x:v>lessons/wrong-robot/level-1.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
-        <x:v>NH1-0-FAMILY</x:v>
+        <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C10" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>Rina's Brother</x:v>
+        <x:v>The Red Pin</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>rina-brother</x:v>
+        <x:v>red-pin</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
-        <x:v>lessons/rina-brother/level-3.txt</x:v>
+        <x:v>lessons/red-pin/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>GDM-10</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Book Under the Hat</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>book-under-hat</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/book-under-hat/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>GDM-22</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>The Rainy Club Map</x:v>
+        <x:v>The Water Pen Trick</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>rainy-club-map</x:v>
+        <x:v>water-pen-trick</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
-        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
+        <x:v>lessons/water-pen-trick/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>GDM-37-4</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>The Star Bus</x:v>
+        <x:v>Where Is the Bell?</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>star-bus</x:v>
+        <x:v>where-is-the-bell</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
-        <x:v>lessons/star-bus/level-3.txt</x:v>
+        <x:v>lessons/where-is-the-bell/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C14" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>Can the Clock Sing?</x:v>
+        <x:v>The Little Door</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
-        <x:v>can-clock-sing</x:v>
+        <x:v>graded-story</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
+        <x:v>lessons/graded-story/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH1-0-FAMILY</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C15" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
+        <x:v>Rina's Brother</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>wrong-robot</x:v>
+        <x:v>rina-brother</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-3.txt</x:v>
+        <x:v>lessons/rina-brother/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str">
         <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>Don't Be a Hero</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>dont-be-a-hero</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>The Window Note</x:v>
+        <x:v>The Rainy Club Map</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
-        <x:v>window-note</x:v>
+        <x:v>rainy-club-map</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
-        <x:v>lessons/window-note/level-3.txt</x:v>
+        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
-        <x:v>The Moon Cup</x:v>
+        <x:v>The Star Bus</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>moon-cup</x:v>
+        <x:v>star-bus</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
-        <x:v>lessons/moon-cup/level-3.txt</x:v>
+        <x:v>lessons/star-bus/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C19" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
-        <x:v>The Rainy Club Map</x:v>
+        <x:v>Can the Clock Sing?</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>rainy-club-map</x:v>
+        <x:v>can-clock-sing</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
-        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
+        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C20" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
-        <x:v>Can the Clock Sing?</x:v>
+        <x:v>The Wrong Robot</x:v>
       </x:c>
       <x:c r="E20" s="12" t="str">
-        <x:v>can-clock-sing</x:v>
+        <x:v>wrong-robot</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
-        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
+        <x:v>lessons/wrong-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C21" s="12" t="str">
         <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D21" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>Don't Be a Hero</x:v>
       </x:c>
       <x:c r="E21" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>dont-be-a-hero</x:v>
       </x:c>
       <x:c r="F21" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C22" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>The Window Note</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>window-note</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/window-note/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C23" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
+        <x:v>The Moon Cup</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>wrong-robot</x:v>
+        <x:v>moon-cup</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-3.txt</x:v>
+        <x:v>lessons/moon-cup/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
         <x:v>Long</x:v>
@@ -1651,198 +1651,198 @@
         <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>Don't Be a Hero</x:v>
+        <x:v>The Rainy Club Map</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
-        <x:v>dont-be-a-hero</x:v>
+        <x:v>rainy-club-map</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
-        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
+        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>Can the Clock Sing?</x:v>
       </x:c>
       <x:c r="E25" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>can-clock-sing</x:v>
       </x:c>
       <x:c r="F25" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C26" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D26" s="12" t="str">
-        <x:v>The Moon Cup</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E26" s="12" t="str">
-        <x:v>moon-cup</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
-        <x:v>lessons/moon-cup/level-3.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C27" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D27" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E27" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F27" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>The Wrong Robot</x:v>
       </x:c>
       <x:c r="E28" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>wrong-robot</x:v>
       </x:c>
       <x:c r="F28" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/wrong-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
-        <x:v>The Red Pin Parade</x:v>
+        <x:v>Don't Be a Hero</x:v>
       </x:c>
       <x:c r="E29" s="12" t="str">
-        <x:v>red-pin-parade</x:v>
+        <x:v>dont-be-a-hero</x:v>
       </x:c>
       <x:c r="F29" s="12" t="str">
-        <x:v>lessons/red-pin-parade/level-7.txt</x:v>
+        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="12" t="str">
-        <x:v>GDM-10</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>The Old Book Signal</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>old-book-signal</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
-        <x:v>lessons/old-book-signal/level-7.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C31" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>The Pens in the Water</x:v>
+        <x:v>The Moon Cup</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
-        <x:v>pens-in-water</x:v>
+        <x:v>moon-cup</x:v>
       </x:c>
       <x:c r="F31" s="12" t="str">
-        <x:v>lessons/pens-in-water/level-7.txt</x:v>
+        <x:v>lessons/moon-cup/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B32" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C32" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
-        <x:v>The Map Under the Stage</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
-        <x:v>map-under-stage</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F32" s="12" t="str">
-        <x:v>lessons/map-under-stage/level-7.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B33" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C33" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D33" s="12" t="str">
-        <x:v>The Door Under the Stage</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E33" s="12" t="str">
-        <x:v>door-under-stage</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F33" s="12" t="str">
-        <x:v>lessons/door-under-stage/level-7.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="12" t="str">
-        <x:v>NH1-0-FAMILY</x:v>
+        <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B34" s="12" t="str">
         <x:v>Long</x:v>
@@ -1851,18 +1851,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
-        <x:v>Family Photo Day</x:v>
+        <x:v>The Red Pin Parade</x:v>
       </x:c>
       <x:c r="E34" s="12" t="str">
-        <x:v>family-photo-day</x:v>
+        <x:v>red-pin-parade</x:v>
       </x:c>
       <x:c r="F34" s="12" t="str">
-        <x:v>lessons/family-photo-day/level-7.txt</x:v>
+        <x:v>lessons/red-pin-parade/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>GDM-10</x:v>
       </x:c>
       <x:c r="B35" s="12" t="str">
         <x:v>Long</x:v>
@@ -1871,18 +1871,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
-        <x:v>The Letter Under the Door</x:v>
+        <x:v>The Old Book Signal</x:v>
       </x:c>
       <x:c r="E35" s="12" t="str">
-        <x:v>letter-under-door</x:v>
+        <x:v>old-book-signal</x:v>
       </x:c>
       <x:c r="F35" s="12" t="str">
-        <x:v>lessons/letter-under-door/level-7.txt</x:v>
+        <x:v>lessons/old-book-signal/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>GDM-22</x:v>
       </x:c>
       <x:c r="B36" s="12" t="str">
         <x:v>Long</x:v>
@@ -1891,18 +1891,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>Why the Lights Blink</x:v>
+        <x:v>The Pens in the Water</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
-        <x:v>why-lights-blink</x:v>
+        <x:v>pens-in-water</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
-        <x:v>lessons/why-lights-blink/level-7.txt</x:v>
+        <x:v>lessons/pens-in-water/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>GDM-37-4</x:v>
       </x:c>
       <x:c r="B37" s="12" t="str">
         <x:v>Long</x:v>
@@ -1911,18 +1911,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
-        <x:v>Because of the Soup</x:v>
+        <x:v>The Map Under the Stage</x:v>
       </x:c>
       <x:c r="E37" s="12" t="str">
-        <x:v>because-of-soup</x:v>
+        <x:v>map-under-stage</x:v>
       </x:c>
       <x:c r="F37" s="12" t="str">
-        <x:v>lessons/because-of-soup/level-7.txt</x:v>
+        <x:v>lessons/map-under-stage/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B38" s="12" t="str">
         <x:v>Long</x:v>
@@ -1931,18 +1931,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>How to Open the Box</x:v>
+        <x:v>The Door Under the Stage</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>open-the-box</x:v>
+        <x:v>door-under-stage</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
-        <x:v>lessons/open-the-box/level-7.txt</x:v>
+        <x:v>lessons/door-under-stage/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH1-0-FAMILY</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
         <x:v>Long</x:v>
@@ -1951,118 +1951,118 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>More Than Half</x:v>
+        <x:v>Family Photo Day</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
-        <x:v>more-than-half</x:v>
+        <x:v>family-photo-day</x:v>
       </x:c>
       <x:c r="F39" s="12" t="str">
-        <x:v>lessons/more-than-half/level-7.txt</x:v>
+        <x:v>lessons/family-photo-day/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B40" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C40" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>The Travel Ticket</x:v>
+        <x:v>The Letter Under the Door</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
-        <x:v>travel-ticket</x:v>
+        <x:v>letter-under-door</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
-        <x:v>lessons/travel-ticket/level-3.txt</x:v>
+        <x:v>lessons/letter-under-door/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B41" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C41" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
-        <x:v>Maybe at the Window</x:v>
+        <x:v>Why the Lights Blink</x:v>
       </x:c>
       <x:c r="E41" s="12" t="str">
-        <x:v>maybe-window</x:v>
+        <x:v>why-lights-blink</x:v>
       </x:c>
       <x:c r="F41" s="12" t="str">
-        <x:v>lessons/maybe-window/level-3.txt</x:v>
+        <x:v>lessons/why-lights-blink/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B42" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C42" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
-        <x:v>The Should Sign</x:v>
+        <x:v>Because of the Soup</x:v>
       </x:c>
       <x:c r="E42" s="12" t="str">
-        <x:v>should-sign</x:v>
+        <x:v>because-of-soup</x:v>
       </x:c>
       <x:c r="F42" s="12" t="str">
-        <x:v>lessons/should-sign/level-3.txt</x:v>
+        <x:v>lessons/because-of-soup/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B43" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C43" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
-        <x:v>The Have-To Key</x:v>
+        <x:v>How to Open the Box</x:v>
       </x:c>
       <x:c r="E43" s="12" t="str">
-        <x:v>have-to-key</x:v>
+        <x:v>open-the-box</x:v>
       </x:c>
       <x:c r="F43" s="12" t="str">
-        <x:v>lessons/have-to-key/level-3.txt</x:v>
+        <x:v>lessons/open-the-box/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B44" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C44" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D44" s="12" t="str">
-        <x:v>The Poster Was Moved</x:v>
+        <x:v>More Than Half</x:v>
       </x:c>
       <x:c r="E44" s="12" t="str">
-        <x:v>passive-poster</x:v>
+        <x:v>more-than-half</x:v>
       </x:c>
       <x:c r="F44" s="12" t="str">
-        <x:v>lessons/passive-poster/level-3.txt</x:v>
+        <x:v>lessons/more-than-half/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B45" s="12" t="str">
         <x:v>Short</x:v>
@@ -2071,18 +2071,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
-        <x:v>The Drink and Read Race</x:v>
+        <x:v>The Travel Ticket</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
-        <x:v>drink-read-race</x:v>
+        <x:v>travel-ticket</x:v>
       </x:c>
       <x:c r="F45" s="12" t="str">
-        <x:v>lessons/drink-read-race/level-3.txt</x:v>
+        <x:v>lessons/travel-ticket/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B46" s="12" t="str">
         <x:v>Short</x:v>
@@ -2091,18 +2091,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
-        <x:v>Can the Lantern Fly?</x:v>
+        <x:v>Maybe at the Window</x:v>
       </x:c>
       <x:c r="E46" s="12" t="str">
-        <x:v>can-lantern</x:v>
+        <x:v>maybe-window</x:v>
       </x:c>
       <x:c r="F46" s="12" t="str">
-        <x:v>lessons/can-lantern/level-3.txt</x:v>
+        <x:v>lessons/maybe-window/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B47" s="12" t="str">
         <x:v>Short</x:v>
@@ -2111,233 +2111,353 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
-        <x:v>Don't Be Late</x:v>
+        <x:v>The Should Sign</x:v>
       </x:c>
       <x:c r="E47" s="12" t="str">
-        <x:v>dont-be-late</x:v>
+        <x:v>should-sign</x:v>
       </x:c>
       <x:c r="F47" s="12" t="str">
-        <x:v>lessons/dont-be-late/level-3.txt</x:v>
+        <x:v>lessons/should-sign/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B48" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C48" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
-        <x:v>Show Me the Seat</x:v>
+        <x:v>The Have-To Key</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
-        <x:v>show-me-the-seat</x:v>
+        <x:v>have-to-key</x:v>
       </x:c>
       <x:c r="F48" s="12" t="str">
-        <x:v>lessons/show-me-the-seat/level-7.txt</x:v>
+        <x:v>lessons/have-to-key/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B49" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C49" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D49" s="12" t="str">
-        <x:v>The Signal Under Water</x:v>
+        <x:v>The Poster Was Moved</x:v>
       </x:c>
       <x:c r="E49" s="12" t="str">
-        <x:v>signal-under-water</x:v>
+        <x:v>passive-poster</x:v>
       </x:c>
       <x:c r="F49" s="12" t="str">
-        <x:v>lessons/signal-under-water/level-3.txt</x:v>
+        <x:v>lessons/passive-poster/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B50" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C50" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
-        <x:v>The Orbit Note</x:v>
+        <x:v>The Drink and Read Race</x:v>
       </x:c>
       <x:c r="E50" s="12" t="str">
-        <x:v>orbit-note</x:v>
+        <x:v>drink-read-race</x:v>
       </x:c>
       <x:c r="F50" s="12" t="str">
-        <x:v>lessons/orbit-note/level-3.txt</x:v>
+        <x:v>lessons/drink-read-race/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B51" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C51" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D51" s="12" t="str">
-        <x:v>Why the Moon Robot Stops</x:v>
+        <x:v>Can the Lantern Fly?</x:v>
       </x:c>
       <x:c r="E51" s="12" t="str">
-        <x:v>why-moon-robot</x:v>
+        <x:v>can-lantern</x:v>
       </x:c>
       <x:c r="F51" s="12" t="str">
-        <x:v>lessons/why-moon-robot/level-3.txt</x:v>
+        <x:v>lessons/can-lantern/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B52" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C52" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D52" s="12" t="str">
-        <x:v>Maybe at the Mars Window</x:v>
+        <x:v>Don't Be Late</x:v>
       </x:c>
       <x:c r="E52" s="12" t="str">
-        <x:v>maybe-mars-window</x:v>
+        <x:v>dont-be-late</x:v>
       </x:c>
       <x:c r="F52" s="12" t="str">
-        <x:v>lessons/maybe-mars-window/level-3.txt</x:v>
+        <x:v>lessons/dont-be-late/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B53" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C53" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
-        <x:v>The Station Was Moved</x:v>
+        <x:v>Show Me the Seat</x:v>
       </x:c>
       <x:c r="E53" s="12" t="str">
-        <x:v>station-was-moved</x:v>
+        <x:v>show-me-the-seat</x:v>
       </x:c>
       <x:c r="F53" s="12" t="str">
-        <x:v>lessons/station-was-moved/level-7.txt</x:v>
+        <x:v>lessons/show-me-the-seat/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>GDM-22</x:v>
       </x:c>
       <x:c r="B54" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C54" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D54" s="12" t="str">
-        <x:v>Where the Roof Door Opens</x:v>
+        <x:v>The Signal Under Water</x:v>
       </x:c>
       <x:c r="E54" s="12" t="str">
-        <x:v>where-the-roof-door</x:v>
+        <x:v>signal-under-water</x:v>
       </x:c>
       <x:c r="F54" s="12" t="str">
-        <x:v>lessons/where-the-roof-door/level-7.txt</x:v>
+        <x:v>lessons/signal-under-water/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B55" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C55" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
-        <x:v>The Traveling Shadow Ticket</x:v>
+        <x:v>The Orbit Note</x:v>
       </x:c>
       <x:c r="E55" s="12" t="str">
-        <x:v>traveling-shadow-ticket</x:v>
+        <x:v>orbit-note</x:v>
       </x:c>
       <x:c r="F55" s="12" t="str">
-        <x:v>lessons/traveling-shadow-ticket/level-7.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56" ht="24" hidden="0" customHeight="1">
+        <x:v>lessons/orbit-note/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B56" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C56" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D56" s="12" t="str">
-        <x:v>Because the Wall Listened</x:v>
+        <x:v>Why the Moon Robot Stops</x:v>
       </x:c>
       <x:c r="E56" s="12" t="str">
-        <x:v>because-the-wall-listened</x:v>
+        <x:v>why-moon-robot</x:v>
       </x:c>
       <x:c r="F56" s="12" t="str">
-        <x:v>lessons/because-the-wall-listened/level-7.txt</x:v>
+        <x:v>lessons/why-moon-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B57" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C57" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D57" s="12" t="str">
-        <x:v>How to Read the Stone</x:v>
+        <x:v>Maybe at the Mars Window</x:v>
       </x:c>
       <x:c r="E57" s="12" t="str">
-        <x:v>how-to-read-the-stone</x:v>
+        <x:v>maybe-mars-window</x:v>
       </x:c>
       <x:c r="F57" s="12" t="str">
-        <x:v>lessons/how-to-read-the-stone/level-7.txt</x:v>
+        <x:v>lessons/maybe-mars-window/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B58" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C58" s="12" t="str">
+        <x:v>SF</x:v>
+      </x:c>
+      <x:c r="D58" s="12" t="str">
+        <x:v>The Station Was Moved</x:v>
+      </x:c>
+      <x:c r="E58" s="12" t="str">
+        <x:v>station-was-moved</x:v>
+      </x:c>
+      <x:c r="F58" s="12" t="str">
+        <x:v>lessons/station-was-moved/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="15" hidden="0" customHeight="1">
+      <x:c r="A59" s="12" t="str">
+        <x:v>GDM-37-4</x:v>
+      </x:c>
+      <x:c r="B59" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C59" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D59" s="12" t="str">
+        <x:v>Where the Roof Door Opens</x:v>
+      </x:c>
+      <x:c r="E59" s="12" t="str">
+        <x:v>where-the-roof-door</x:v>
+      </x:c>
+      <x:c r="F59" s="12" t="str">
+        <x:v>lessons/where-the-roof-door/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="15" hidden="0" customHeight="1">
+      <x:c r="A60" s="12" t="str">
+        <x:v>NH1-1-10-V</x:v>
+      </x:c>
+      <x:c r="B60" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C60" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D60" s="12" t="str">
+        <x:v>The Traveling Shadow Ticket</x:v>
+      </x:c>
+      <x:c r="E60" s="12" t="str">
+        <x:v>traveling-shadow-ticket</x:v>
+      </x:c>
+      <x:c r="F60" s="12" t="str">
+        <x:v>lessons/traveling-shadow-ticket/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="24" hidden="0" customHeight="1">
+      <x:c r="A61" s="12" t="str">
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
+      </x:c>
+      <x:c r="B61" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C61" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D61" s="12" t="str">
+        <x:v>Because the Wall Listened</x:v>
+      </x:c>
+      <x:c r="E61" s="12" t="str">
+        <x:v>because-the-wall-listened</x:v>
+      </x:c>
+      <x:c r="F61" s="12" t="str">
+        <x:v>lessons/because-the-wall-listened/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="15" hidden="0" customHeight="1">
+      <x:c r="A62" s="12" t="str">
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
+      </x:c>
+      <x:c r="B62" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C62" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D62" s="12" t="str">
+        <x:v>How to Read the Stone</x:v>
+      </x:c>
+      <x:c r="E62" s="12" t="str">
+        <x:v>how-to-read-the-stone</x:v>
+      </x:c>
+      <x:c r="F62" s="12" t="str">
+        <x:v>lessons/how-to-read-the-stone/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="15" hidden="0" customHeight="1">
+      <x:c r="A63" s="12" t="str">
         <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
-      <x:c r="B58" s="12" t="str">
-        <x:v>Long</x:v>
-      </x:c>
-      <x:c r="C58" s="12" t="str">
+      <x:c r="B63" s="12" t="str">
+        <x:v>Long</x:v>
+      </x:c>
+      <x:c r="C63" s="12" t="str">
         <x:v>Mystery</x:v>
       </x:c>
-      <x:c r="D58" s="12" t="str">
+      <x:c r="D63" s="12" t="str">
         <x:v>More Than One Moon</x:v>
       </x:c>
-      <x:c r="E58" s="12" t="str">
+      <x:c r="E63" s="12" t="str">
         <x:v>more-than-one-moon</x:v>
       </x:c>
-      <x:c r="F58" s="12" t="str">
+      <x:c r="F63" s="12" t="str">
         <x:v>lessons/more-than-one-moon/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="15" hidden="0" customHeight="1">
+      <x:c r="A64" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B64" s="12" t="str">
+        <x:v>Very Long</x:v>
+      </x:c>
+      <x:c r="C64" s="12" t="str">
+        <x:v>Comedy</x:v>
+      </x:c>
+      <x:c r="D64" s="12" t="str">
+        <x:v>The Pudding Case</x:v>
+      </x:c>
+      <x:c r="E64" s="12" t="str">
+        <x:v>jaio-pudding-case</x:v>
+      </x:c>
+      <x:c r="F64" s="12" t="str">
+        <x:v>lessons/jaio-pudding-case/level-8.txt</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2367,10 +2487,10 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>生成時はIDを1つだけ使い、本文量をShort/Longで指定する。</x:v>
+        <x:v>生成時はIDを1つだけ使い、本文量をLengthで指定する。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>生成時はIDを1つだけ使い、本文量をShort/Longで指定する。</x:v>
+        <x:v>生成時はIDを1つだけ使い、本文量をLengthで指定する。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -2395,7 +2515,7 @@
         <x:v>本文量</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>{Length} で生成する。Shortは120〜180語程度、Longは300〜450語程度。</x:v>
+        <x:v>{Length} で生成する。Very Shortはごく短い導入、Shortは120〜180語程度、Longは300〜450語程度、Very Longは650〜900語程度。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Add very long readings for all genres
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Rc1cebf0037454a22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rb10d647d399e46a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R36e46d12f7f447ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R8d95ff92a14b4d92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R4b71513115af4cd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Rcb78d983bc0341b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R1b6be33b67664369"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="Rfdc1054a8b7e4d1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R37db3907867c4172"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Ra2147b5579274c32"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2448,15 +2448,115 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C64" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D64" s="12" t="str">
+        <x:v>The Locked Umbrella Room</x:v>
+      </x:c>
+      <x:c r="E64" s="12" t="str">
+        <x:v>locked-umbrella-room</x:v>
+      </x:c>
+      <x:c r="F64" s="12" t="str">
+        <x:v>lessons/locked-umbrella-room/level-8.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="15" hidden="0" customHeight="1">
+      <x:c r="A65" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B65" s="12" t="str">
+        <x:v>Very Long</x:v>
+      </x:c>
+      <x:c r="C65" s="12" t="str">
+        <x:v>Human Drama</x:v>
+      </x:c>
+      <x:c r="D65" s="12" t="str">
+        <x:v>The Last Seat at the Table</x:v>
+      </x:c>
+      <x:c r="E65" s="12" t="str">
+        <x:v>last-seat-table</x:v>
+      </x:c>
+      <x:c r="F65" s="12" t="str">
+        <x:v>lessons/last-seat-table/level-8.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="15" hidden="0" customHeight="1">
+      <x:c r="A66" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B66" s="12" t="str">
+        <x:v>Very Long</x:v>
+      </x:c>
+      <x:c r="C66" s="12" t="str">
+        <x:v>SF</x:v>
+      </x:c>
+      <x:c r="D66" s="12" t="str">
+        <x:v>The Library That Was Moved</x:v>
+      </x:c>
+      <x:c r="E66" s="12" t="str">
+        <x:v>library-moved</x:v>
+      </x:c>
+      <x:c r="F66" s="12" t="str">
+        <x:v>lessons/library-moved/level-8.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="15" hidden="0" customHeight="1">
+      <x:c r="A67" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B67" s="12" t="str">
+        <x:v>Very Long</x:v>
+      </x:c>
+      <x:c r="C67" s="12" t="str">
+        <x:v>Fantasy</x:v>
+      </x:c>
+      <x:c r="D67" s="12" t="str">
+        <x:v>The Moon Lantern Path</x:v>
+      </x:c>
+      <x:c r="E67" s="12" t="str">
+        <x:v>moon-lantern-path</x:v>
+      </x:c>
+      <x:c r="F67" s="12" t="str">
+        <x:v>lessons/moon-lantern-path/level-8.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="15" hidden="0" customHeight="1">
+      <x:c r="A68" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B68" s="12" t="str">
+        <x:v>Very Long</x:v>
+      </x:c>
+      <x:c r="C68" s="12" t="str">
+        <x:v>Adventure</x:v>
+      </x:c>
+      <x:c r="D68" s="12" t="str">
+        <x:v>The Folded Map Race</x:v>
+      </x:c>
+      <x:c r="E68" s="12" t="str">
+        <x:v>folded-map-race</x:v>
+      </x:c>
+      <x:c r="F68" s="12" t="str">
+        <x:v>lessons/folded-map-race/level-8.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="15" hidden="0" customHeight="1">
+      <x:c r="A69" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B69" s="12" t="str">
+        <x:v>Very Long</x:v>
+      </x:c>
+      <x:c r="C69" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
-      <x:c r="D64" s="12" t="str">
+      <x:c r="D69" s="12" t="str">
         <x:v>The Pudding Case</x:v>
       </x:c>
-      <x:c r="E64" s="12" t="str">
+      <x:c r="E69" s="12" t="str">
         <x:v>jaio-pudding-case</x:v>
       </x:c>
-      <x:c r="F64" s="12" t="str">
+      <x:c r="F69" s="12" t="str">
         <x:v>lessons/jaio-pudding-case/level-8.txt</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add missing very short genre readings
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Rcb78d983bc0341b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R1b6be33b67664369"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="Rfdc1054a8b7e4d1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R37db3907867c4172"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Ra2147b5579274c32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R55a7b17a9e974eac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R1b8cbbd4f3774a42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R77b7db81f5774da8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R37f33c371d6f4b51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Rafa9053897ec40d0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1348,16 +1348,16 @@
         <x:v>Very Short</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
+        <x:v>The Silver Stone</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>wrong-robot</x:v>
+        <x:v>silver-stone</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-1.txt</x:v>
+        <x:v>lessons/silver-stone/level-1.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1365,44 +1365,44 @@
         <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Very Short</x:v>
       </x:c>
       <x:c r="C10" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>The Red Pin</x:v>
+        <x:v>The Red Bag Path</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>red-pin</x:v>
+        <x:v>red-bag-path</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
-        <x:v>lessons/red-pin/level-3.txt</x:v>
+        <x:v>lessons/red-bag-path/level-1.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>GDM-10</x:v>
+        <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Very Short</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>The Book Under the Hat</x:v>
+        <x:v>The Wrong Robot</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>book-under-hat</x:v>
+        <x:v>wrong-robot</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
-        <x:v>lessons/book-under-hat/level-3.txt</x:v>
+        <x:v>lessons/wrong-robot/level-1.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
         <x:v>Short</x:v>
@@ -1411,38 +1411,38 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>The Water Pen Trick</x:v>
+        <x:v>The Red Pin</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>water-pen-trick</x:v>
+        <x:v>red-pin</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
-        <x:v>lessons/water-pen-trick/level-3.txt</x:v>
+        <x:v>lessons/red-pin/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>GDM-10</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>Where Is the Bell?</x:v>
+        <x:v>The Book Under the Hat</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>where-is-the-bell</x:v>
+        <x:v>book-under-hat</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
-        <x:v>lessons/where-is-the-bell/level-3.txt</x:v>
+        <x:v>lessons/book-under-hat/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>GDM-22</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
         <x:v>Short</x:v>
@@ -1451,438 +1451,438 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>The Little Door</x:v>
+        <x:v>The Water Pen Trick</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
-        <x:v>graded-story</x:v>
+        <x:v>water-pen-trick</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>lessons/graded-story/level-3.txt</x:v>
+        <x:v>lessons/water-pen-trick/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>NH1-0-FAMILY</x:v>
+        <x:v>GDM-37-4</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C15" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>Rina's Brother</x:v>
+        <x:v>Where Is the Bell?</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>rina-brother</x:v>
+        <x:v>where-is-the-bell</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
-        <x:v>lessons/rina-brother/level-3.txt</x:v>
+        <x:v>lessons/where-is-the-bell/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Little Door</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>graded-story</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/graded-story/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>NH1-0-FAMILY</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str">
         <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>The Rainy Club Map</x:v>
+        <x:v>Rina's Brother</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
-        <x:v>rainy-club-map</x:v>
+        <x:v>rina-brother</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
-        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
+        <x:v>lessons/rina-brother/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
-        <x:v>The Star Bus</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>star-bus</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
-        <x:v>lessons/star-bus/level-3.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C19" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
-        <x:v>Can the Clock Sing?</x:v>
+        <x:v>The Rainy Club Map</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>can-clock-sing</x:v>
+        <x:v>rainy-club-map</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
-        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
+        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C20" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
+        <x:v>The Star Bus</x:v>
       </x:c>
       <x:c r="E20" s="12" t="str">
-        <x:v>wrong-robot</x:v>
+        <x:v>star-bus</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-3.txt</x:v>
+        <x:v>lessons/star-bus/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C21" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D21" s="12" t="str">
-        <x:v>Don't Be a Hero</x:v>
+        <x:v>Can the Clock Sing?</x:v>
       </x:c>
       <x:c r="E21" s="12" t="str">
-        <x:v>dont-be-a-hero</x:v>
+        <x:v>can-clock-sing</x:v>
       </x:c>
       <x:c r="F21" s="12" t="str">
-        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
+        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C22" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>The Window Note</x:v>
+        <x:v>The Wrong Robot</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>window-note</x:v>
+        <x:v>wrong-robot</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
-        <x:v>lessons/window-note/level-3.txt</x:v>
+        <x:v>lessons/wrong-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C23" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>The Moon Cup</x:v>
+        <x:v>Don't Be a Hero</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>moon-cup</x:v>
+        <x:v>dont-be-a-hero</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
-        <x:v>lessons/moon-cup/level-3.txt</x:v>
+        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C24" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>The Rainy Club Map</x:v>
+        <x:v>The Window Note</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
-        <x:v>rainy-club-map</x:v>
+        <x:v>window-note</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
-        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
+        <x:v>lessons/window-note/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str">
         <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
-        <x:v>Can the Clock Sing?</x:v>
+        <x:v>The Moon Cup</x:v>
       </x:c>
       <x:c r="E25" s="12" t="str">
-        <x:v>can-clock-sing</x:v>
+        <x:v>moon-cup</x:v>
       </x:c>
       <x:c r="F25" s="12" t="str">
-        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
+        <x:v>lessons/moon-cup/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C26" s="12" t="str">
         <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D26" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Rainy Club Map</x:v>
       </x:c>
       <x:c r="E26" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>rainy-club-map</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C27" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D27" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>Can the Clock Sing?</x:v>
       </x:c>
       <x:c r="E27" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>can-clock-sing</x:v>
       </x:c>
       <x:c r="F27" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E28" s="12" t="str">
-        <x:v>wrong-robot</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F28" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-3.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
-        <x:v>Don't Be a Hero</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E29" s="12" t="str">
-        <x:v>dont-be-a-hero</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F29" s="12" t="str">
-        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>The Wrong Robot</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>wrong-robot</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/wrong-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C31" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>The Moon Cup</x:v>
+        <x:v>Don't Be a Hero</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
-        <x:v>moon-cup</x:v>
+        <x:v>dont-be-a-hero</x:v>
       </x:c>
       <x:c r="F31" s="12" t="str">
-        <x:v>lessons/moon-cup/level-3.txt</x:v>
+        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B32" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C32" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F32" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B33" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C33" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D33" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>The Moon Cup</x:v>
       </x:c>
       <x:c r="E33" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>moon-cup</x:v>
       </x:c>
       <x:c r="F33" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/moon-cup/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B34" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C34" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
-        <x:v>The Red Pin Parade</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E34" s="12" t="str">
-        <x:v>red-pin-parade</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F34" s="12" t="str">
-        <x:v>lessons/red-pin-parade/level-7.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="12" t="str">
-        <x:v>GDM-10</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B35" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C35" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
-        <x:v>The Old Book Signal</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E35" s="12" t="str">
-        <x:v>old-book-signal</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F35" s="12" t="str">
-        <x:v>lessons/old-book-signal/level-7.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B36" s="12" t="str">
         <x:v>Long</x:v>
@@ -1891,18 +1891,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>The Pens in the Water</x:v>
+        <x:v>The Red Pin Parade</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
-        <x:v>pens-in-water</x:v>
+        <x:v>red-pin-parade</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
-        <x:v>lessons/pens-in-water/level-7.txt</x:v>
+        <x:v>lessons/red-pin-parade/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>GDM-10</x:v>
       </x:c>
       <x:c r="B37" s="12" t="str">
         <x:v>Long</x:v>
@@ -1911,18 +1911,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
-        <x:v>The Map Under the Stage</x:v>
+        <x:v>The Old Book Signal</x:v>
       </x:c>
       <x:c r="E37" s="12" t="str">
-        <x:v>map-under-stage</x:v>
+        <x:v>old-book-signal</x:v>
       </x:c>
       <x:c r="F37" s="12" t="str">
-        <x:v>lessons/map-under-stage/level-7.txt</x:v>
+        <x:v>lessons/old-book-signal/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>GDM-22</x:v>
       </x:c>
       <x:c r="B38" s="12" t="str">
         <x:v>Long</x:v>
@@ -1931,18 +1931,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>The Door Under the Stage</x:v>
+        <x:v>The Pens in the Water</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>door-under-stage</x:v>
+        <x:v>pens-in-water</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
-        <x:v>lessons/door-under-stage/level-7.txt</x:v>
+        <x:v>lessons/pens-in-water/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="12" t="str">
-        <x:v>NH1-0-FAMILY</x:v>
+        <x:v>GDM-37-4</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
         <x:v>Long</x:v>
@@ -1951,18 +1951,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>Family Photo Day</x:v>
+        <x:v>The Map Under the Stage</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
-        <x:v>family-photo-day</x:v>
+        <x:v>map-under-stage</x:v>
       </x:c>
       <x:c r="F39" s="12" t="str">
-        <x:v>lessons/family-photo-day/level-7.txt</x:v>
+        <x:v>lessons/map-under-stage/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B40" s="12" t="str">
         <x:v>Long</x:v>
@@ -1971,18 +1971,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>The Letter Under the Door</x:v>
+        <x:v>The Door Under the Stage</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
-        <x:v>letter-under-door</x:v>
+        <x:v>door-under-stage</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
-        <x:v>lessons/letter-under-door/level-7.txt</x:v>
+        <x:v>lessons/door-under-stage/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH1-0-FAMILY</x:v>
       </x:c>
       <x:c r="B41" s="12" t="str">
         <x:v>Long</x:v>
@@ -1991,18 +1991,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
-        <x:v>Why the Lights Blink</x:v>
+        <x:v>Family Photo Day</x:v>
       </x:c>
       <x:c r="E41" s="12" t="str">
-        <x:v>why-lights-blink</x:v>
+        <x:v>family-photo-day</x:v>
       </x:c>
       <x:c r="F41" s="12" t="str">
-        <x:v>lessons/why-lights-blink/level-7.txt</x:v>
+        <x:v>lessons/family-photo-day/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B42" s="12" t="str">
         <x:v>Long</x:v>
@@ -2011,18 +2011,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
-        <x:v>Because of the Soup</x:v>
+        <x:v>The Letter Under the Door</x:v>
       </x:c>
       <x:c r="E42" s="12" t="str">
-        <x:v>because-of-soup</x:v>
+        <x:v>letter-under-door</x:v>
       </x:c>
       <x:c r="F42" s="12" t="str">
-        <x:v>lessons/because-of-soup/level-7.txt</x:v>
+        <x:v>lessons/letter-under-door/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B43" s="12" t="str">
         <x:v>Long</x:v>
@@ -2031,18 +2031,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
-        <x:v>How to Open the Box</x:v>
+        <x:v>Why the Lights Blink</x:v>
       </x:c>
       <x:c r="E43" s="12" t="str">
-        <x:v>open-the-box</x:v>
+        <x:v>why-lights-blink</x:v>
       </x:c>
       <x:c r="F43" s="12" t="str">
-        <x:v>lessons/open-the-box/level-7.txt</x:v>
+        <x:v>lessons/why-lights-blink/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B44" s="12" t="str">
         <x:v>Long</x:v>
@@ -2051,58 +2051,58 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D44" s="12" t="str">
-        <x:v>More Than Half</x:v>
+        <x:v>Because of the Soup</x:v>
       </x:c>
       <x:c r="E44" s="12" t="str">
-        <x:v>more-than-half</x:v>
+        <x:v>because-of-soup</x:v>
       </x:c>
       <x:c r="F44" s="12" t="str">
-        <x:v>lessons/more-than-half/level-7.txt</x:v>
+        <x:v>lessons/because-of-soup/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B45" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C45" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
-        <x:v>The Travel Ticket</x:v>
+        <x:v>How to Open the Box</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
-        <x:v>travel-ticket</x:v>
+        <x:v>open-the-box</x:v>
       </x:c>
       <x:c r="F45" s="12" t="str">
-        <x:v>lessons/travel-ticket/level-3.txt</x:v>
+        <x:v>lessons/open-the-box/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B46" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C46" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
-        <x:v>Maybe at the Window</x:v>
+        <x:v>More Than Half</x:v>
       </x:c>
       <x:c r="E46" s="12" t="str">
-        <x:v>maybe-window</x:v>
+        <x:v>more-than-half</x:v>
       </x:c>
       <x:c r="F46" s="12" t="str">
-        <x:v>lessons/maybe-window/level-3.txt</x:v>
+        <x:v>lessons/more-than-half/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B47" s="12" t="str">
         <x:v>Short</x:v>
@@ -2111,18 +2111,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
-        <x:v>The Should Sign</x:v>
+        <x:v>The Travel Ticket</x:v>
       </x:c>
       <x:c r="E47" s="12" t="str">
-        <x:v>should-sign</x:v>
+        <x:v>travel-ticket</x:v>
       </x:c>
       <x:c r="F47" s="12" t="str">
-        <x:v>lessons/should-sign/level-3.txt</x:v>
+        <x:v>lessons/travel-ticket/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B48" s="12" t="str">
         <x:v>Short</x:v>
@@ -2131,18 +2131,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
-        <x:v>The Have-To Key</x:v>
+        <x:v>Maybe at the Window</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
-        <x:v>have-to-key</x:v>
+        <x:v>maybe-window</x:v>
       </x:c>
       <x:c r="F48" s="12" t="str">
-        <x:v>lessons/have-to-key/level-3.txt</x:v>
+        <x:v>lessons/maybe-window/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B49" s="12" t="str">
         <x:v>Short</x:v>
@@ -2151,18 +2151,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D49" s="12" t="str">
-        <x:v>The Poster Was Moved</x:v>
+        <x:v>The Should Sign</x:v>
       </x:c>
       <x:c r="E49" s="12" t="str">
-        <x:v>passive-poster</x:v>
+        <x:v>should-sign</x:v>
       </x:c>
       <x:c r="F49" s="12" t="str">
-        <x:v>lessons/passive-poster/level-3.txt</x:v>
+        <x:v>lessons/should-sign/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B50" s="12" t="str">
         <x:v>Short</x:v>
@@ -2171,18 +2171,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
-        <x:v>The Drink and Read Race</x:v>
+        <x:v>The Have-To Key</x:v>
       </x:c>
       <x:c r="E50" s="12" t="str">
-        <x:v>drink-read-race</x:v>
+        <x:v>have-to-key</x:v>
       </x:c>
       <x:c r="F50" s="12" t="str">
-        <x:v>lessons/drink-read-race/level-3.txt</x:v>
+        <x:v>lessons/have-to-key/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B51" s="12" t="str">
         <x:v>Short</x:v>
@@ -2191,18 +2191,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D51" s="12" t="str">
-        <x:v>Can the Lantern Fly?</x:v>
+        <x:v>The Poster Was Moved</x:v>
       </x:c>
       <x:c r="E51" s="12" t="str">
-        <x:v>can-lantern</x:v>
+        <x:v>passive-poster</x:v>
       </x:c>
       <x:c r="F51" s="12" t="str">
-        <x:v>lessons/can-lantern/level-3.txt</x:v>
+        <x:v>lessons/passive-poster/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B52" s="12" t="str">
         <x:v>Short</x:v>
@@ -2211,78 +2211,78 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D52" s="12" t="str">
-        <x:v>Don't Be Late</x:v>
+        <x:v>The Drink and Read Race</x:v>
       </x:c>
       <x:c r="E52" s="12" t="str">
-        <x:v>dont-be-late</x:v>
+        <x:v>drink-read-race</x:v>
       </x:c>
       <x:c r="F52" s="12" t="str">
-        <x:v>lessons/dont-be-late/level-3.txt</x:v>
+        <x:v>lessons/drink-read-race/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B53" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C53" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
-        <x:v>Show Me the Seat</x:v>
+        <x:v>Can the Lantern Fly?</x:v>
       </x:c>
       <x:c r="E53" s="12" t="str">
-        <x:v>show-me-the-seat</x:v>
+        <x:v>can-lantern</x:v>
       </x:c>
       <x:c r="F53" s="12" t="str">
-        <x:v>lessons/show-me-the-seat/level-7.txt</x:v>
+        <x:v>lessons/can-lantern/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B54" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C54" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D54" s="12" t="str">
-        <x:v>The Signal Under Water</x:v>
+        <x:v>Don't Be Late</x:v>
       </x:c>
       <x:c r="E54" s="12" t="str">
-        <x:v>signal-under-water</x:v>
+        <x:v>dont-be-late</x:v>
       </x:c>
       <x:c r="F54" s="12" t="str">
-        <x:v>lessons/signal-under-water/level-3.txt</x:v>
+        <x:v>lessons/dont-be-late/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B55" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C55" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
-        <x:v>The Orbit Note</x:v>
+        <x:v>Show Me the Seat</x:v>
       </x:c>
       <x:c r="E55" s="12" t="str">
-        <x:v>orbit-note</x:v>
+        <x:v>show-me-the-seat</x:v>
       </x:c>
       <x:c r="F55" s="12" t="str">
-        <x:v>lessons/orbit-note/level-3.txt</x:v>
+        <x:v>lessons/show-me-the-seat/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>GDM-22</x:v>
       </x:c>
       <x:c r="B56" s="12" t="str">
         <x:v>Short</x:v>
@@ -2291,18 +2291,18 @@
         <x:v>SF</x:v>
       </x:c>
       <x:c r="D56" s="12" t="str">
-        <x:v>Why the Moon Robot Stops</x:v>
+        <x:v>The Signal Under Water</x:v>
       </x:c>
       <x:c r="E56" s="12" t="str">
-        <x:v>why-moon-robot</x:v>
+        <x:v>signal-under-water</x:v>
       </x:c>
       <x:c r="F56" s="12" t="str">
-        <x:v>lessons/why-moon-robot/level-3.txt</x:v>
+        <x:v>lessons/signal-under-water/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B57" s="12" t="str">
         <x:v>Short</x:v>
@@ -2311,78 +2311,78 @@
         <x:v>SF</x:v>
       </x:c>
       <x:c r="D57" s="12" t="str">
-        <x:v>Maybe at the Mars Window</x:v>
+        <x:v>The Orbit Note</x:v>
       </x:c>
       <x:c r="E57" s="12" t="str">
-        <x:v>maybe-mars-window</x:v>
+        <x:v>orbit-note</x:v>
       </x:c>
       <x:c r="F57" s="12" t="str">
-        <x:v>lessons/maybe-mars-window/level-3.txt</x:v>
+        <x:v>lessons/orbit-note/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B58" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C58" s="12" t="str">
         <x:v>SF</x:v>
       </x:c>
       <x:c r="D58" s="12" t="str">
-        <x:v>The Station Was Moved</x:v>
+        <x:v>Why the Moon Robot Stops</x:v>
       </x:c>
       <x:c r="E58" s="12" t="str">
-        <x:v>station-was-moved</x:v>
+        <x:v>why-moon-robot</x:v>
       </x:c>
       <x:c r="F58" s="12" t="str">
-        <x:v>lessons/station-was-moved/level-7.txt</x:v>
+        <x:v>lessons/why-moon-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B59" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C59" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D59" s="12" t="str">
-        <x:v>Where the Roof Door Opens</x:v>
+        <x:v>Maybe at the Mars Window</x:v>
       </x:c>
       <x:c r="E59" s="12" t="str">
-        <x:v>where-the-roof-door</x:v>
+        <x:v>maybe-mars-window</x:v>
       </x:c>
       <x:c r="F59" s="12" t="str">
-        <x:v>lessons/where-the-roof-door/level-7.txt</x:v>
+        <x:v>lessons/maybe-mars-window/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
       <x:c r="A60" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B60" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C60" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D60" s="12" t="str">
-        <x:v>The Traveling Shadow Ticket</x:v>
+        <x:v>The Station Was Moved</x:v>
       </x:c>
       <x:c r="E60" s="12" t="str">
-        <x:v>traveling-shadow-ticket</x:v>
+        <x:v>station-was-moved</x:v>
       </x:c>
       <x:c r="F60" s="12" t="str">
-        <x:v>lessons/traveling-shadow-ticket/level-7.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61" ht="24" hidden="0" customHeight="1">
+        <x:v>lessons/station-was-moved/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>GDM-37-4</x:v>
       </x:c>
       <x:c r="B61" s="12" t="str">
         <x:v>Long</x:v>
@@ -2391,18 +2391,18 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D61" s="12" t="str">
-        <x:v>Because the Wall Listened</x:v>
+        <x:v>Where the Roof Door Opens</x:v>
       </x:c>
       <x:c r="E61" s="12" t="str">
-        <x:v>because-the-wall-listened</x:v>
+        <x:v>where-the-roof-door</x:v>
       </x:c>
       <x:c r="F61" s="12" t="str">
-        <x:v>lessons/because-the-wall-listened/level-7.txt</x:v>
+        <x:v>lessons/where-the-roof-door/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
       <x:c r="A62" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B62" s="12" t="str">
         <x:v>Long</x:v>
@@ -2411,18 +2411,18 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D62" s="12" t="str">
-        <x:v>How to Read the Stone</x:v>
+        <x:v>The Traveling Shadow Ticket</x:v>
       </x:c>
       <x:c r="E62" s="12" t="str">
-        <x:v>how-to-read-the-stone</x:v>
+        <x:v>traveling-shadow-ticket</x:v>
       </x:c>
       <x:c r="F62" s="12" t="str">
-        <x:v>lessons/how-to-read-the-stone/level-7.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="15" hidden="0" customHeight="1">
+        <x:v>lessons/traveling-shadow-ticket/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="24" hidden="0" customHeight="1">
       <x:c r="A63" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B63" s="12" t="str">
         <x:v>Long</x:v>
@@ -2431,53 +2431,53 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D63" s="12" t="str">
-        <x:v>More Than One Moon</x:v>
+        <x:v>Because the Wall Listened</x:v>
       </x:c>
       <x:c r="E63" s="12" t="str">
-        <x:v>more-than-one-moon</x:v>
+        <x:v>because-the-wall-listened</x:v>
       </x:c>
       <x:c r="F63" s="12" t="str">
-        <x:v>lessons/more-than-one-moon/level-7.txt</x:v>
+        <x:v>lessons/because-the-wall-listened/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
       <x:c r="A64" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B64" s="12" t="str">
-        <x:v>Very Long</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C64" s="12" t="str">
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D64" s="12" t="str">
-        <x:v>The Locked Umbrella Room</x:v>
+        <x:v>How to Read the Stone</x:v>
       </x:c>
       <x:c r="E64" s="12" t="str">
-        <x:v>locked-umbrella-room</x:v>
+        <x:v>how-to-read-the-stone</x:v>
       </x:c>
       <x:c r="F64" s="12" t="str">
-        <x:v>lessons/locked-umbrella-room/level-8.txt</x:v>
+        <x:v>lessons/how-to-read-the-stone/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
       <x:c r="A65" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B65" s="12" t="str">
-        <x:v>Very Long</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C65" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D65" s="12" t="str">
-        <x:v>The Last Seat at the Table</x:v>
+        <x:v>More Than One Moon</x:v>
       </x:c>
       <x:c r="E65" s="12" t="str">
-        <x:v>last-seat-table</x:v>
+        <x:v>more-than-one-moon</x:v>
       </x:c>
       <x:c r="F65" s="12" t="str">
-        <x:v>lessons/last-seat-table/level-8.txt</x:v>
+        <x:v>lessons/more-than-one-moon/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
@@ -2488,16 +2488,16 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C66" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D66" s="12" t="str">
-        <x:v>The Library That Was Moved</x:v>
+        <x:v>The Locked Umbrella Room</x:v>
       </x:c>
       <x:c r="E66" s="12" t="str">
-        <x:v>library-moved</x:v>
+        <x:v>locked-umbrella-room</x:v>
       </x:c>
       <x:c r="F66" s="12" t="str">
-        <x:v>lessons/library-moved/level-8.txt</x:v>
+        <x:v>lessons/locked-umbrella-room/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
@@ -2508,16 +2508,16 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C67" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D67" s="12" t="str">
-        <x:v>The Moon Lantern Path</x:v>
+        <x:v>The Last Seat at the Table</x:v>
       </x:c>
       <x:c r="E67" s="12" t="str">
-        <x:v>moon-lantern-path</x:v>
+        <x:v>last-seat-table</x:v>
       </x:c>
       <x:c r="F67" s="12" t="str">
-        <x:v>lessons/moon-lantern-path/level-8.txt</x:v>
+        <x:v>lessons/last-seat-table/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
@@ -2528,16 +2528,16 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C68" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D68" s="12" t="str">
-        <x:v>The Folded Map Race</x:v>
+        <x:v>The Library That Was Moved</x:v>
       </x:c>
       <x:c r="E68" s="12" t="str">
-        <x:v>folded-map-race</x:v>
+        <x:v>library-moved</x:v>
       </x:c>
       <x:c r="F68" s="12" t="str">
-        <x:v>lessons/folded-map-race/level-8.txt</x:v>
+        <x:v>lessons/library-moved/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
@@ -2548,15 +2548,55 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C69" s="12" t="str">
+        <x:v>Fantasy</x:v>
+      </x:c>
+      <x:c r="D69" s="12" t="str">
+        <x:v>The Moon Lantern Path</x:v>
+      </x:c>
+      <x:c r="E69" s="12" t="str">
+        <x:v>moon-lantern-path</x:v>
+      </x:c>
+      <x:c r="F69" s="12" t="str">
+        <x:v>lessons/moon-lantern-path/level-8.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="15" hidden="0" customHeight="1">
+      <x:c r="A70" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B70" s="12" t="str">
+        <x:v>Very Long</x:v>
+      </x:c>
+      <x:c r="C70" s="12" t="str">
+        <x:v>Adventure</x:v>
+      </x:c>
+      <x:c r="D70" s="12" t="str">
+        <x:v>The Folded Map Race</x:v>
+      </x:c>
+      <x:c r="E70" s="12" t="str">
+        <x:v>folded-map-race</x:v>
+      </x:c>
+      <x:c r="F70" s="12" t="str">
+        <x:v>lessons/folded-map-race/level-8.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="15" hidden="0" customHeight="1">
+      <x:c r="A71" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B71" s="12" t="str">
+        <x:v>Very Long</x:v>
+      </x:c>
+      <x:c r="C71" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
-      <x:c r="D69" s="12" t="str">
+      <x:c r="D71" s="12" t="str">
         <x:v>The Pudding Case</x:v>
       </x:c>
-      <x:c r="E69" s="12" t="str">
+      <x:c r="E71" s="12" t="str">
         <x:v>jaio-pudding-case</x:v>
       </x:c>
-      <x:c r="F69" s="12" t="str">
+      <x:c r="F71" s="12" t="str">
         <x:v>lessons/jaio-pudding-case/level-8.txt</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add three long comedy readings
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R55a7b17a9e974eac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R1b8cbbd4f3774a42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R77b7db81f5774da8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R37f33c371d6f4b51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Rafa9053897ec40d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R412d19f74af44710"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R09a920fbc9a148b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="Rbcfa5fd0a8a249d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R4bddbd0fa9454779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Ra76d17e3452d44f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1602,22 +1602,22 @@
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C22" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
+        <x:v>Can the Principal Dance?</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>wrong-robot</x:v>
+        <x:v>principal-dance</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-3.txt</x:v>
+        <x:v>lessons/principal-dance/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
@@ -1625,119 +1625,119 @@
         <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C23" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>Don't Be a Hero</x:v>
+        <x:v>The Wrong Robot</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>dont-be-a-hero</x:v>
+        <x:v>wrong-robot</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
-        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
+        <x:v>lessons/wrong-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C24" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>The Window Note</x:v>
+        <x:v>Don't Be a Hero</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
-        <x:v>window-note</x:v>
+        <x:v>dont-be-a-hero</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
-        <x:v>lessons/window-note/level-3.txt</x:v>
+        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
-        <x:v>The Moon Cup</x:v>
+        <x:v>The Window Note</x:v>
       </x:c>
       <x:c r="E25" s="12" t="str">
-        <x:v>moon-cup</x:v>
+        <x:v>window-note</x:v>
       </x:c>
       <x:c r="F25" s="12" t="str">
-        <x:v>lessons/moon-cup/level-3.txt</x:v>
+        <x:v>lessons/window-note/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C26" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D26" s="12" t="str">
-        <x:v>The Rainy Club Map</x:v>
+        <x:v>The Moon Cup</x:v>
       </x:c>
       <x:c r="E26" s="12" t="str">
-        <x:v>rainy-club-map</x:v>
+        <x:v>moon-cup</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
-        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
+        <x:v>lessons/moon-cup/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C27" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D27" s="12" t="str">
-        <x:v>Can the Clock Sing?</x:v>
+        <x:v>The Rainy Club Map</x:v>
       </x:c>
       <x:c r="E27" s="12" t="str">
-        <x:v>can-clock-sing</x:v>
+        <x:v>rainy-club-map</x:v>
       </x:c>
       <x:c r="F27" s="12" t="str">
-        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
+        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>Can the Clock Sing?</x:v>
       </x:c>
       <x:c r="E28" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>can-clock-sing</x:v>
       </x:c>
       <x:c r="F28" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
@@ -1745,64 +1745,64 @@
         <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E29" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F29" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>wrong-robot</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-3.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C31" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>Don't Be a Hero</x:v>
+        <x:v>The Wrong Robot</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
-        <x:v>dont-be-a-hero</x:v>
+        <x:v>wrong-robot</x:v>
       </x:c>
       <x:c r="F31" s="12" t="str">
-        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
+        <x:v>lessons/wrong-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B32" s="12" t="str">
         <x:v>Long</x:v>
@@ -1811,138 +1811,138 @@
         <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>Because the Hat Said No</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>hat-said-no</x:v>
       </x:c>
       <x:c r="F32" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/hat-said-no/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B33" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C33" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D33" s="12" t="str">
-        <x:v>The Moon Cup</x:v>
+        <x:v>Don't Be a Hero</x:v>
       </x:c>
       <x:c r="E33" s="12" t="str">
-        <x:v>moon-cup</x:v>
+        <x:v>dont-be-a-hero</x:v>
       </x:c>
       <x:c r="F33" s="12" t="str">
-        <x:v>lessons/moon-cup/level-3.txt</x:v>
+        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B34" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C34" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E34" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F34" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B35" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C35" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>The Moon Cup</x:v>
       </x:c>
       <x:c r="E35" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>moon-cup</x:v>
       </x:c>
       <x:c r="F35" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/moon-cup/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B36" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C36" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>The Red Pin Parade</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
-        <x:v>red-pin-parade</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
-        <x:v>lessons/red-pin-parade/level-7.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
-        <x:v>GDM-10</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B37" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C37" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
-        <x:v>The Old Book Signal</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E37" s="12" t="str">
-        <x:v>old-book-signal</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F37" s="12" t="str">
-        <x:v>lessons/old-book-signal/level-7.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B38" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C38" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>The Pens in the Water</x:v>
+        <x:v>The Cake Was Moved</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>pens-in-water</x:v>
+        <x:v>cake-was-moved</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
-        <x:v>lessons/pens-in-water/level-7.txt</x:v>
+        <x:v>lessons/cake-was-moved/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
         <x:v>Long</x:v>
@@ -1951,18 +1951,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>The Map Under the Stage</x:v>
+        <x:v>The Red Pin Parade</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
-        <x:v>map-under-stage</x:v>
+        <x:v>red-pin-parade</x:v>
       </x:c>
       <x:c r="F39" s="12" t="str">
-        <x:v>lessons/map-under-stage/level-7.txt</x:v>
+        <x:v>lessons/red-pin-parade/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>GDM-10</x:v>
       </x:c>
       <x:c r="B40" s="12" t="str">
         <x:v>Long</x:v>
@@ -1971,18 +1971,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>The Door Under the Stage</x:v>
+        <x:v>The Old Book Signal</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
-        <x:v>door-under-stage</x:v>
+        <x:v>old-book-signal</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
-        <x:v>lessons/door-under-stage/level-7.txt</x:v>
+        <x:v>lessons/old-book-signal/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="12" t="str">
-        <x:v>NH1-0-FAMILY</x:v>
+        <x:v>GDM-22</x:v>
       </x:c>
       <x:c r="B41" s="12" t="str">
         <x:v>Long</x:v>
@@ -1991,18 +1991,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
-        <x:v>Family Photo Day</x:v>
+        <x:v>The Pens in the Water</x:v>
       </x:c>
       <x:c r="E41" s="12" t="str">
-        <x:v>family-photo-day</x:v>
+        <x:v>pens-in-water</x:v>
       </x:c>
       <x:c r="F41" s="12" t="str">
-        <x:v>lessons/family-photo-day/level-7.txt</x:v>
+        <x:v>lessons/pens-in-water/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>GDM-37-4</x:v>
       </x:c>
       <x:c r="B42" s="12" t="str">
         <x:v>Long</x:v>
@@ -2011,18 +2011,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
-        <x:v>The Letter Under the Door</x:v>
+        <x:v>The Map Under the Stage</x:v>
       </x:c>
       <x:c r="E42" s="12" t="str">
-        <x:v>letter-under-door</x:v>
+        <x:v>map-under-stage</x:v>
       </x:c>
       <x:c r="F42" s="12" t="str">
-        <x:v>lessons/letter-under-door/level-7.txt</x:v>
+        <x:v>lessons/map-under-stage/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B43" s="12" t="str">
         <x:v>Long</x:v>
@@ -2031,18 +2031,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
-        <x:v>Why the Lights Blink</x:v>
+        <x:v>The Door Under the Stage</x:v>
       </x:c>
       <x:c r="E43" s="12" t="str">
-        <x:v>why-lights-blink</x:v>
+        <x:v>door-under-stage</x:v>
       </x:c>
       <x:c r="F43" s="12" t="str">
-        <x:v>lessons/why-lights-blink/level-7.txt</x:v>
+        <x:v>lessons/door-under-stage/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH1-0-FAMILY</x:v>
       </x:c>
       <x:c r="B44" s="12" t="str">
         <x:v>Long</x:v>
@@ -2051,18 +2051,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D44" s="12" t="str">
-        <x:v>Because of the Soup</x:v>
+        <x:v>Family Photo Day</x:v>
       </x:c>
       <x:c r="E44" s="12" t="str">
-        <x:v>because-of-soup</x:v>
+        <x:v>family-photo-day</x:v>
       </x:c>
       <x:c r="F44" s="12" t="str">
-        <x:v>lessons/because-of-soup/level-7.txt</x:v>
+        <x:v>lessons/family-photo-day/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B45" s="12" t="str">
         <x:v>Long</x:v>
@@ -2071,18 +2071,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
-        <x:v>How to Open the Box</x:v>
+        <x:v>The Letter Under the Door</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
-        <x:v>open-the-box</x:v>
+        <x:v>letter-under-door</x:v>
       </x:c>
       <x:c r="F45" s="12" t="str">
-        <x:v>lessons/open-the-box/level-7.txt</x:v>
+        <x:v>lessons/letter-under-door/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B46" s="12" t="str">
         <x:v>Long</x:v>
@@ -2091,78 +2091,78 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
-        <x:v>More Than Half</x:v>
+        <x:v>Why the Lights Blink</x:v>
       </x:c>
       <x:c r="E46" s="12" t="str">
-        <x:v>more-than-half</x:v>
+        <x:v>why-lights-blink</x:v>
       </x:c>
       <x:c r="F46" s="12" t="str">
-        <x:v>lessons/more-than-half/level-7.txt</x:v>
+        <x:v>lessons/why-lights-blink/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B47" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C47" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
-        <x:v>The Travel Ticket</x:v>
+        <x:v>Because of the Soup</x:v>
       </x:c>
       <x:c r="E47" s="12" t="str">
-        <x:v>travel-ticket</x:v>
+        <x:v>because-of-soup</x:v>
       </x:c>
       <x:c r="F47" s="12" t="str">
-        <x:v>lessons/travel-ticket/level-3.txt</x:v>
+        <x:v>lessons/because-of-soup/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B48" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C48" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
-        <x:v>Maybe at the Window</x:v>
+        <x:v>How to Open the Box</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
-        <x:v>maybe-window</x:v>
+        <x:v>open-the-box</x:v>
       </x:c>
       <x:c r="F48" s="12" t="str">
-        <x:v>lessons/maybe-window/level-3.txt</x:v>
+        <x:v>lessons/open-the-box/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B49" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C49" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D49" s="12" t="str">
-        <x:v>The Should Sign</x:v>
+        <x:v>More Than Half</x:v>
       </x:c>
       <x:c r="E49" s="12" t="str">
-        <x:v>should-sign</x:v>
+        <x:v>more-than-half</x:v>
       </x:c>
       <x:c r="F49" s="12" t="str">
-        <x:v>lessons/should-sign/level-3.txt</x:v>
+        <x:v>lessons/more-than-half/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B50" s="12" t="str">
         <x:v>Short</x:v>
@@ -2171,18 +2171,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
-        <x:v>The Have-To Key</x:v>
+        <x:v>The Travel Ticket</x:v>
       </x:c>
       <x:c r="E50" s="12" t="str">
-        <x:v>have-to-key</x:v>
+        <x:v>travel-ticket</x:v>
       </x:c>
       <x:c r="F50" s="12" t="str">
-        <x:v>lessons/have-to-key/level-3.txt</x:v>
+        <x:v>lessons/travel-ticket/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B51" s="12" t="str">
         <x:v>Short</x:v>
@@ -2191,18 +2191,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D51" s="12" t="str">
-        <x:v>The Poster Was Moved</x:v>
+        <x:v>Maybe at the Window</x:v>
       </x:c>
       <x:c r="E51" s="12" t="str">
-        <x:v>passive-poster</x:v>
+        <x:v>maybe-window</x:v>
       </x:c>
       <x:c r="F51" s="12" t="str">
-        <x:v>lessons/passive-poster/level-3.txt</x:v>
+        <x:v>lessons/maybe-window/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B52" s="12" t="str">
         <x:v>Short</x:v>
@@ -2211,18 +2211,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D52" s="12" t="str">
-        <x:v>The Drink and Read Race</x:v>
+        <x:v>The Should Sign</x:v>
       </x:c>
       <x:c r="E52" s="12" t="str">
-        <x:v>drink-read-race</x:v>
+        <x:v>should-sign</x:v>
       </x:c>
       <x:c r="F52" s="12" t="str">
-        <x:v>lessons/drink-read-race/level-3.txt</x:v>
+        <x:v>lessons/should-sign/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B53" s="12" t="str">
         <x:v>Short</x:v>
@@ -2231,18 +2231,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
-        <x:v>Can the Lantern Fly?</x:v>
+        <x:v>The Have-To Key</x:v>
       </x:c>
       <x:c r="E53" s="12" t="str">
-        <x:v>can-lantern</x:v>
+        <x:v>have-to-key</x:v>
       </x:c>
       <x:c r="F53" s="12" t="str">
-        <x:v>lessons/can-lantern/level-3.txt</x:v>
+        <x:v>lessons/have-to-key/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B54" s="12" t="str">
         <x:v>Short</x:v>
@@ -2251,98 +2251,98 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D54" s="12" t="str">
-        <x:v>Don't Be Late</x:v>
+        <x:v>The Poster Was Moved</x:v>
       </x:c>
       <x:c r="E54" s="12" t="str">
-        <x:v>dont-be-late</x:v>
+        <x:v>passive-poster</x:v>
       </x:c>
       <x:c r="F54" s="12" t="str">
-        <x:v>lessons/dont-be-late/level-3.txt</x:v>
+        <x:v>lessons/passive-poster/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B55" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C55" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
-        <x:v>Show Me the Seat</x:v>
+        <x:v>The Drink and Read Race</x:v>
       </x:c>
       <x:c r="E55" s="12" t="str">
-        <x:v>show-me-the-seat</x:v>
+        <x:v>drink-read-race</x:v>
       </x:c>
       <x:c r="F55" s="12" t="str">
-        <x:v>lessons/show-me-the-seat/level-7.txt</x:v>
+        <x:v>lessons/drink-read-race/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B56" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C56" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D56" s="12" t="str">
-        <x:v>The Signal Under Water</x:v>
+        <x:v>Can the Lantern Fly?</x:v>
       </x:c>
       <x:c r="E56" s="12" t="str">
-        <x:v>signal-under-water</x:v>
+        <x:v>can-lantern</x:v>
       </x:c>
       <x:c r="F56" s="12" t="str">
-        <x:v>lessons/signal-under-water/level-3.txt</x:v>
+        <x:v>lessons/can-lantern/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B57" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C57" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D57" s="12" t="str">
-        <x:v>The Orbit Note</x:v>
+        <x:v>Don't Be Late</x:v>
       </x:c>
       <x:c r="E57" s="12" t="str">
-        <x:v>orbit-note</x:v>
+        <x:v>dont-be-late</x:v>
       </x:c>
       <x:c r="F57" s="12" t="str">
-        <x:v>lessons/orbit-note/level-3.txt</x:v>
+        <x:v>lessons/dont-be-late/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B58" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C58" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D58" s="12" t="str">
-        <x:v>Why the Moon Robot Stops</x:v>
+        <x:v>Show Me the Seat</x:v>
       </x:c>
       <x:c r="E58" s="12" t="str">
-        <x:v>why-moon-robot</x:v>
+        <x:v>show-me-the-seat</x:v>
       </x:c>
       <x:c r="F58" s="12" t="str">
-        <x:v>lessons/why-moon-robot/level-3.txt</x:v>
+        <x:v>lessons/show-me-the-seat/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>GDM-22</x:v>
       </x:c>
       <x:c r="B59" s="12" t="str">
         <x:v>Short</x:v>
@@ -2351,98 +2351,98 @@
         <x:v>SF</x:v>
       </x:c>
       <x:c r="D59" s="12" t="str">
-        <x:v>Maybe at the Mars Window</x:v>
+        <x:v>The Signal Under Water</x:v>
       </x:c>
       <x:c r="E59" s="12" t="str">
-        <x:v>maybe-mars-window</x:v>
+        <x:v>signal-under-water</x:v>
       </x:c>
       <x:c r="F59" s="12" t="str">
-        <x:v>lessons/maybe-mars-window/level-3.txt</x:v>
+        <x:v>lessons/signal-under-water/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
       <x:c r="A60" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B60" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C60" s="12" t="str">
         <x:v>SF</x:v>
       </x:c>
       <x:c r="D60" s="12" t="str">
-        <x:v>The Station Was Moved</x:v>
+        <x:v>The Orbit Note</x:v>
       </x:c>
       <x:c r="E60" s="12" t="str">
-        <x:v>station-was-moved</x:v>
+        <x:v>orbit-note</x:v>
       </x:c>
       <x:c r="F60" s="12" t="str">
-        <x:v>lessons/station-was-moved/level-7.txt</x:v>
+        <x:v>lessons/orbit-note/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B61" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C61" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D61" s="12" t="str">
-        <x:v>Where the Roof Door Opens</x:v>
+        <x:v>Why the Moon Robot Stops</x:v>
       </x:c>
       <x:c r="E61" s="12" t="str">
-        <x:v>where-the-roof-door</x:v>
+        <x:v>why-moon-robot</x:v>
       </x:c>
       <x:c r="F61" s="12" t="str">
-        <x:v>lessons/where-the-roof-door/level-7.txt</x:v>
+        <x:v>lessons/why-moon-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
       <x:c r="A62" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B62" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C62" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D62" s="12" t="str">
-        <x:v>The Traveling Shadow Ticket</x:v>
+        <x:v>Maybe at the Mars Window</x:v>
       </x:c>
       <x:c r="E62" s="12" t="str">
-        <x:v>traveling-shadow-ticket</x:v>
+        <x:v>maybe-mars-window</x:v>
       </x:c>
       <x:c r="F62" s="12" t="str">
-        <x:v>lessons/traveling-shadow-ticket/level-7.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63" ht="24" hidden="0" customHeight="1">
+        <x:v>lessons/maybe-mars-window/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="15" hidden="0" customHeight="1">
       <x:c r="A63" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B63" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C63" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D63" s="12" t="str">
-        <x:v>Because the Wall Listened</x:v>
+        <x:v>The Station Was Moved</x:v>
       </x:c>
       <x:c r="E63" s="12" t="str">
-        <x:v>because-the-wall-listened</x:v>
+        <x:v>station-was-moved</x:v>
       </x:c>
       <x:c r="F63" s="12" t="str">
-        <x:v>lessons/because-the-wall-listened/level-7.txt</x:v>
+        <x:v>lessons/station-was-moved/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
       <x:c r="A64" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>GDM-37-4</x:v>
       </x:c>
       <x:c r="B64" s="12" t="str">
         <x:v>Long</x:v>
@@ -2451,18 +2451,18 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D64" s="12" t="str">
-        <x:v>How to Read the Stone</x:v>
+        <x:v>Where the Roof Door Opens</x:v>
       </x:c>
       <x:c r="E64" s="12" t="str">
-        <x:v>how-to-read-the-stone</x:v>
+        <x:v>where-the-roof-door</x:v>
       </x:c>
       <x:c r="F64" s="12" t="str">
-        <x:v>lessons/how-to-read-the-stone/level-7.txt</x:v>
+        <x:v>lessons/where-the-roof-door/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
       <x:c r="A65" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B65" s="12" t="str">
         <x:v>Long</x:v>
@@ -2471,73 +2471,73 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D65" s="12" t="str">
-        <x:v>More Than One Moon</x:v>
+        <x:v>The Traveling Shadow Ticket</x:v>
       </x:c>
       <x:c r="E65" s="12" t="str">
-        <x:v>more-than-one-moon</x:v>
+        <x:v>traveling-shadow-ticket</x:v>
       </x:c>
       <x:c r="F65" s="12" t="str">
-        <x:v>lessons/more-than-one-moon/level-7.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66" ht="15" hidden="0" customHeight="1">
+        <x:v>lessons/traveling-shadow-ticket/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="24" hidden="0" customHeight="1">
       <x:c r="A66" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B66" s="12" t="str">
-        <x:v>Very Long</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C66" s="12" t="str">
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D66" s="12" t="str">
-        <x:v>The Locked Umbrella Room</x:v>
+        <x:v>Because the Wall Listened</x:v>
       </x:c>
       <x:c r="E66" s="12" t="str">
-        <x:v>locked-umbrella-room</x:v>
+        <x:v>because-the-wall-listened</x:v>
       </x:c>
       <x:c r="F66" s="12" t="str">
-        <x:v>lessons/locked-umbrella-room/level-8.txt</x:v>
+        <x:v>lessons/because-the-wall-listened/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
       <x:c r="A67" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B67" s="12" t="str">
-        <x:v>Very Long</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C67" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D67" s="12" t="str">
-        <x:v>The Last Seat at the Table</x:v>
+        <x:v>How to Read the Stone</x:v>
       </x:c>
       <x:c r="E67" s="12" t="str">
-        <x:v>last-seat-table</x:v>
+        <x:v>how-to-read-the-stone</x:v>
       </x:c>
       <x:c r="F67" s="12" t="str">
-        <x:v>lessons/last-seat-table/level-8.txt</x:v>
+        <x:v>lessons/how-to-read-the-stone/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
       <x:c r="A68" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B68" s="12" t="str">
-        <x:v>Very Long</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C68" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D68" s="12" t="str">
-        <x:v>The Library That Was Moved</x:v>
+        <x:v>More Than One Moon</x:v>
       </x:c>
       <x:c r="E68" s="12" t="str">
-        <x:v>library-moved</x:v>
+        <x:v>more-than-one-moon</x:v>
       </x:c>
       <x:c r="F68" s="12" t="str">
-        <x:v>lessons/library-moved/level-8.txt</x:v>
+        <x:v>lessons/more-than-one-moon/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
@@ -2548,16 +2548,16 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C69" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D69" s="12" t="str">
-        <x:v>The Moon Lantern Path</x:v>
+        <x:v>The Locked Umbrella Room</x:v>
       </x:c>
       <x:c r="E69" s="12" t="str">
-        <x:v>moon-lantern-path</x:v>
+        <x:v>locked-umbrella-room</x:v>
       </x:c>
       <x:c r="F69" s="12" t="str">
-        <x:v>lessons/moon-lantern-path/level-8.txt</x:v>
+        <x:v>lessons/locked-umbrella-room/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
@@ -2568,16 +2568,16 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C70" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D70" s="12" t="str">
-        <x:v>The Folded Map Race</x:v>
+        <x:v>The Last Seat at the Table</x:v>
       </x:c>
       <x:c r="E70" s="12" t="str">
-        <x:v>folded-map-race</x:v>
+        <x:v>last-seat-table</x:v>
       </x:c>
       <x:c r="F70" s="12" t="str">
-        <x:v>lessons/folded-map-race/level-8.txt</x:v>
+        <x:v>lessons/last-seat-table/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="15" hidden="0" customHeight="1">
@@ -2588,15 +2588,75 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C71" s="12" t="str">
+        <x:v>SF</x:v>
+      </x:c>
+      <x:c r="D71" s="12" t="str">
+        <x:v>The Library That Was Moved</x:v>
+      </x:c>
+      <x:c r="E71" s="12" t="str">
+        <x:v>library-moved</x:v>
+      </x:c>
+      <x:c r="F71" s="12" t="str">
+        <x:v>lessons/library-moved/level-8.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="15" hidden="0" customHeight="1">
+      <x:c r="A72" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B72" s="12" t="str">
+        <x:v>Very Long</x:v>
+      </x:c>
+      <x:c r="C72" s="12" t="str">
+        <x:v>Fantasy</x:v>
+      </x:c>
+      <x:c r="D72" s="12" t="str">
+        <x:v>The Moon Lantern Path</x:v>
+      </x:c>
+      <x:c r="E72" s="12" t="str">
+        <x:v>moon-lantern-path</x:v>
+      </x:c>
+      <x:c r="F72" s="12" t="str">
+        <x:v>lessons/moon-lantern-path/level-8.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="15" hidden="0" customHeight="1">
+      <x:c r="A73" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B73" s="12" t="str">
+        <x:v>Very Long</x:v>
+      </x:c>
+      <x:c r="C73" s="12" t="str">
+        <x:v>Adventure</x:v>
+      </x:c>
+      <x:c r="D73" s="12" t="str">
+        <x:v>The Folded Map Race</x:v>
+      </x:c>
+      <x:c r="E73" s="12" t="str">
+        <x:v>folded-map-race</x:v>
+      </x:c>
+      <x:c r="F73" s="12" t="str">
+        <x:v>lessons/folded-map-race/level-8.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="15" hidden="0" customHeight="1">
+      <x:c r="A74" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B74" s="12" t="str">
+        <x:v>Very Long</x:v>
+      </x:c>
+      <x:c r="C74" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
-      <x:c r="D71" s="12" t="str">
+      <x:c r="D74" s="12" t="str">
         <x:v>The Pudding Case</x:v>
       </x:c>
-      <x:c r="E71" s="12" t="str">
+      <x:c r="E74" s="12" t="str">
         <x:v>jaio-pudding-case</x:v>
       </x:c>
-      <x:c r="F71" s="12" t="str">
+      <x:c r="F74" s="12" t="str">
         <x:v>lessons/jaio-pudding-case/level-8.txt</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add cross-genre fantasy adventure reading
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R412d19f74af44710"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R09a920fbc9a148b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="Rbcfa5fd0a8a249d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R4bddbd0fa9454779"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Ra76d17e3452d44f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Rcf972c212868411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R69ada2d3f23145de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R873d23f339e74af0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R18c6969c95f54d99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Rce026c2334ca4e23"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1882,42 +1882,42 @@
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B36" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C36" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Fantasy / Adventure</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Dice Gate</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>dice-gate</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/dice-gate/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B37" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C37" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E37" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F37" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
@@ -1931,38 +1931,38 @@
         <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>The Cake Was Moved</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>cake-was-moved</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
-        <x:v>lessons/cake-was-moved/level-7.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C39" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>The Red Pin Parade</x:v>
+        <x:v>The Cake Was Moved</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
-        <x:v>red-pin-parade</x:v>
+        <x:v>cake-was-moved</x:v>
       </x:c>
       <x:c r="F39" s="12" t="str">
-        <x:v>lessons/red-pin-parade/level-7.txt</x:v>
+        <x:v>lessons/cake-was-moved/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="12" t="str">
-        <x:v>GDM-10</x:v>
+        <x:v>GDM-1</x:v>
       </x:c>
       <x:c r="B40" s="12" t="str">
         <x:v>Long</x:v>
@@ -1971,18 +1971,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>The Old Book Signal</x:v>
+        <x:v>The Red Pin Parade</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
-        <x:v>old-book-signal</x:v>
+        <x:v>red-pin-parade</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
-        <x:v>lessons/old-book-signal/level-7.txt</x:v>
+        <x:v>lessons/red-pin-parade/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>GDM-10</x:v>
       </x:c>
       <x:c r="B41" s="12" t="str">
         <x:v>Long</x:v>
@@ -1991,18 +1991,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
-        <x:v>The Pens in the Water</x:v>
+        <x:v>The Old Book Signal</x:v>
       </x:c>
       <x:c r="E41" s="12" t="str">
-        <x:v>pens-in-water</x:v>
+        <x:v>old-book-signal</x:v>
       </x:c>
       <x:c r="F41" s="12" t="str">
-        <x:v>lessons/pens-in-water/level-7.txt</x:v>
+        <x:v>lessons/old-book-signal/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>GDM-22</x:v>
       </x:c>
       <x:c r="B42" s="12" t="str">
         <x:v>Long</x:v>
@@ -2011,18 +2011,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
-        <x:v>The Map Under the Stage</x:v>
+        <x:v>The Pens in the Water</x:v>
       </x:c>
       <x:c r="E42" s="12" t="str">
-        <x:v>map-under-stage</x:v>
+        <x:v>pens-in-water</x:v>
       </x:c>
       <x:c r="F42" s="12" t="str">
-        <x:v>lessons/map-under-stage/level-7.txt</x:v>
+        <x:v>lessons/pens-in-water/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>GDM-37-4</x:v>
       </x:c>
       <x:c r="B43" s="12" t="str">
         <x:v>Long</x:v>
@@ -2031,18 +2031,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
-        <x:v>The Door Under the Stage</x:v>
+        <x:v>The Map Under the Stage</x:v>
       </x:c>
       <x:c r="E43" s="12" t="str">
-        <x:v>door-under-stage</x:v>
+        <x:v>map-under-stage</x:v>
       </x:c>
       <x:c r="F43" s="12" t="str">
-        <x:v>lessons/door-under-stage/level-7.txt</x:v>
+        <x:v>lessons/map-under-stage/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="12" t="str">
-        <x:v>NH1-0-FAMILY</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B44" s="12" t="str">
         <x:v>Long</x:v>
@@ -2051,18 +2051,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D44" s="12" t="str">
-        <x:v>Family Photo Day</x:v>
+        <x:v>The Door Under the Stage</x:v>
       </x:c>
       <x:c r="E44" s="12" t="str">
-        <x:v>family-photo-day</x:v>
+        <x:v>door-under-stage</x:v>
       </x:c>
       <x:c r="F44" s="12" t="str">
-        <x:v>lessons/family-photo-day/level-7.txt</x:v>
+        <x:v>lessons/door-under-stage/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>NH1-0-FAMILY</x:v>
       </x:c>
       <x:c r="B45" s="12" t="str">
         <x:v>Long</x:v>
@@ -2071,18 +2071,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
-        <x:v>The Letter Under the Door</x:v>
+        <x:v>Family Photo Day</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
-        <x:v>letter-under-door</x:v>
+        <x:v>family-photo-day</x:v>
       </x:c>
       <x:c r="F45" s="12" t="str">
-        <x:v>lessons/letter-under-door/level-7.txt</x:v>
+        <x:v>lessons/family-photo-day/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B46" s="12" t="str">
         <x:v>Long</x:v>
@@ -2091,18 +2091,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
-        <x:v>Why the Lights Blink</x:v>
+        <x:v>The Letter Under the Door</x:v>
       </x:c>
       <x:c r="E46" s="12" t="str">
-        <x:v>why-lights-blink</x:v>
+        <x:v>letter-under-door</x:v>
       </x:c>
       <x:c r="F46" s="12" t="str">
-        <x:v>lessons/why-lights-blink/level-7.txt</x:v>
+        <x:v>lessons/letter-under-door/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B47" s="12" t="str">
         <x:v>Long</x:v>
@@ -2111,18 +2111,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
-        <x:v>Because of the Soup</x:v>
+        <x:v>Why the Lights Blink</x:v>
       </x:c>
       <x:c r="E47" s="12" t="str">
-        <x:v>because-of-soup</x:v>
+        <x:v>why-lights-blink</x:v>
       </x:c>
       <x:c r="F47" s="12" t="str">
-        <x:v>lessons/because-of-soup/level-7.txt</x:v>
+        <x:v>lessons/why-lights-blink/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B48" s="12" t="str">
         <x:v>Long</x:v>
@@ -2131,18 +2131,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
-        <x:v>How to Open the Box</x:v>
+        <x:v>Because of the Soup</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
-        <x:v>open-the-box</x:v>
+        <x:v>because-of-soup</x:v>
       </x:c>
       <x:c r="F48" s="12" t="str">
-        <x:v>lessons/open-the-box/level-7.txt</x:v>
+        <x:v>lessons/because-of-soup/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B49" s="12" t="str">
         <x:v>Long</x:v>
@@ -2151,38 +2151,38 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D49" s="12" t="str">
-        <x:v>More Than Half</x:v>
+        <x:v>How to Open the Box</x:v>
       </x:c>
       <x:c r="E49" s="12" t="str">
-        <x:v>more-than-half</x:v>
+        <x:v>open-the-box</x:v>
       </x:c>
       <x:c r="F49" s="12" t="str">
-        <x:v>lessons/more-than-half/level-7.txt</x:v>
+        <x:v>lessons/open-the-box/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B50" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C50" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
-        <x:v>The Travel Ticket</x:v>
+        <x:v>More Than Half</x:v>
       </x:c>
       <x:c r="E50" s="12" t="str">
-        <x:v>travel-ticket</x:v>
+        <x:v>more-than-half</x:v>
       </x:c>
       <x:c r="F50" s="12" t="str">
-        <x:v>lessons/travel-ticket/level-3.txt</x:v>
+        <x:v>lessons/more-than-half/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B51" s="12" t="str">
         <x:v>Short</x:v>
@@ -2191,18 +2191,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D51" s="12" t="str">
-        <x:v>Maybe at the Window</x:v>
+        <x:v>The Travel Ticket</x:v>
       </x:c>
       <x:c r="E51" s="12" t="str">
-        <x:v>maybe-window</x:v>
+        <x:v>travel-ticket</x:v>
       </x:c>
       <x:c r="F51" s="12" t="str">
-        <x:v>lessons/maybe-window/level-3.txt</x:v>
+        <x:v>lessons/travel-ticket/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B52" s="12" t="str">
         <x:v>Short</x:v>
@@ -2211,18 +2211,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D52" s="12" t="str">
-        <x:v>The Should Sign</x:v>
+        <x:v>Maybe at the Window</x:v>
       </x:c>
       <x:c r="E52" s="12" t="str">
-        <x:v>should-sign</x:v>
+        <x:v>maybe-window</x:v>
       </x:c>
       <x:c r="F52" s="12" t="str">
-        <x:v>lessons/should-sign/level-3.txt</x:v>
+        <x:v>lessons/maybe-window/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B53" s="12" t="str">
         <x:v>Short</x:v>
@@ -2231,18 +2231,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
-        <x:v>The Have-To Key</x:v>
+        <x:v>The Should Sign</x:v>
       </x:c>
       <x:c r="E53" s="12" t="str">
-        <x:v>have-to-key</x:v>
+        <x:v>should-sign</x:v>
       </x:c>
       <x:c r="F53" s="12" t="str">
-        <x:v>lessons/have-to-key/level-3.txt</x:v>
+        <x:v>lessons/should-sign/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B54" s="12" t="str">
         <x:v>Short</x:v>
@@ -2251,18 +2251,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D54" s="12" t="str">
-        <x:v>The Poster Was Moved</x:v>
+        <x:v>The Have-To Key</x:v>
       </x:c>
       <x:c r="E54" s="12" t="str">
-        <x:v>passive-poster</x:v>
+        <x:v>have-to-key</x:v>
       </x:c>
       <x:c r="F54" s="12" t="str">
-        <x:v>lessons/passive-poster/level-3.txt</x:v>
+        <x:v>lessons/have-to-key/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B55" s="12" t="str">
         <x:v>Short</x:v>
@@ -2271,18 +2271,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
-        <x:v>The Drink and Read Race</x:v>
+        <x:v>The Poster Was Moved</x:v>
       </x:c>
       <x:c r="E55" s="12" t="str">
-        <x:v>drink-read-race</x:v>
+        <x:v>passive-poster</x:v>
       </x:c>
       <x:c r="F55" s="12" t="str">
-        <x:v>lessons/drink-read-race/level-3.txt</x:v>
+        <x:v>lessons/passive-poster/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B56" s="12" t="str">
         <x:v>Short</x:v>
@@ -2291,18 +2291,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D56" s="12" t="str">
-        <x:v>Can the Lantern Fly?</x:v>
+        <x:v>The Drink and Read Race</x:v>
       </x:c>
       <x:c r="E56" s="12" t="str">
-        <x:v>can-lantern</x:v>
+        <x:v>drink-read-race</x:v>
       </x:c>
       <x:c r="F56" s="12" t="str">
-        <x:v>lessons/can-lantern/level-3.txt</x:v>
+        <x:v>lessons/drink-read-race/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B57" s="12" t="str">
         <x:v>Short</x:v>
@@ -2311,58 +2311,58 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D57" s="12" t="str">
-        <x:v>Don't Be Late</x:v>
+        <x:v>Can the Lantern Fly?</x:v>
       </x:c>
       <x:c r="E57" s="12" t="str">
-        <x:v>dont-be-late</x:v>
+        <x:v>can-lantern</x:v>
       </x:c>
       <x:c r="F57" s="12" t="str">
-        <x:v>lessons/dont-be-late/level-3.txt</x:v>
+        <x:v>lessons/can-lantern/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH1-1-5-2-DONTBE</x:v>
       </x:c>
       <x:c r="B58" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C58" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D58" s="12" t="str">
-        <x:v>Show Me the Seat</x:v>
+        <x:v>Don't Be Late</x:v>
       </x:c>
       <x:c r="E58" s="12" t="str">
-        <x:v>show-me-the-seat</x:v>
+        <x:v>dont-be-late</x:v>
       </x:c>
       <x:c r="F58" s="12" t="str">
-        <x:v>lessons/show-me-the-seat/level-7.txt</x:v>
+        <x:v>lessons/dont-be-late/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B59" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C59" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D59" s="12" t="str">
-        <x:v>The Signal Under Water</x:v>
+        <x:v>Show Me the Seat</x:v>
       </x:c>
       <x:c r="E59" s="12" t="str">
-        <x:v>signal-under-water</x:v>
+        <x:v>show-me-the-seat</x:v>
       </x:c>
       <x:c r="F59" s="12" t="str">
-        <x:v>lessons/signal-under-water/level-3.txt</x:v>
+        <x:v>lessons/show-me-the-seat/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
       <x:c r="A60" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>GDM-22</x:v>
       </x:c>
       <x:c r="B60" s="12" t="str">
         <x:v>Short</x:v>
@@ -2371,18 +2371,18 @@
         <x:v>SF</x:v>
       </x:c>
       <x:c r="D60" s="12" t="str">
-        <x:v>The Orbit Note</x:v>
+        <x:v>The Signal Under Water</x:v>
       </x:c>
       <x:c r="E60" s="12" t="str">
-        <x:v>orbit-note</x:v>
+        <x:v>signal-under-water</x:v>
       </x:c>
       <x:c r="F60" s="12" t="str">
-        <x:v>lessons/orbit-note/level-3.txt</x:v>
+        <x:v>lessons/signal-under-water/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B61" s="12" t="str">
         <x:v>Short</x:v>
@@ -2391,18 +2391,18 @@
         <x:v>SF</x:v>
       </x:c>
       <x:c r="D61" s="12" t="str">
-        <x:v>Why the Moon Robot Stops</x:v>
+        <x:v>The Orbit Note</x:v>
       </x:c>
       <x:c r="E61" s="12" t="str">
-        <x:v>why-moon-robot</x:v>
+        <x:v>orbit-note</x:v>
       </x:c>
       <x:c r="F61" s="12" t="str">
-        <x:v>lessons/why-moon-robot/level-3.txt</x:v>
+        <x:v>lessons/orbit-note/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
       <x:c r="A62" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B62" s="12" t="str">
         <x:v>Short</x:v>
@@ -2411,58 +2411,58 @@
         <x:v>SF</x:v>
       </x:c>
       <x:c r="D62" s="12" t="str">
-        <x:v>Maybe at the Mars Window</x:v>
+        <x:v>Why the Moon Robot Stops</x:v>
       </x:c>
       <x:c r="E62" s="12" t="str">
-        <x:v>maybe-mars-window</x:v>
+        <x:v>why-moon-robot</x:v>
       </x:c>
       <x:c r="F62" s="12" t="str">
-        <x:v>lessons/maybe-mars-window/level-3.txt</x:v>
+        <x:v>lessons/why-moon-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="15" hidden="0" customHeight="1">
       <x:c r="A63" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B63" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C63" s="12" t="str">
         <x:v>SF</x:v>
       </x:c>
       <x:c r="D63" s="12" t="str">
-        <x:v>The Station Was Moved</x:v>
+        <x:v>Maybe at the Mars Window</x:v>
       </x:c>
       <x:c r="E63" s="12" t="str">
-        <x:v>station-was-moved</x:v>
+        <x:v>maybe-mars-window</x:v>
       </x:c>
       <x:c r="F63" s="12" t="str">
-        <x:v>lessons/station-was-moved/level-7.txt</x:v>
+        <x:v>lessons/maybe-mars-window/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
       <x:c r="A64" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B64" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C64" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D64" s="12" t="str">
-        <x:v>Where the Roof Door Opens</x:v>
+        <x:v>The Station Was Moved</x:v>
       </x:c>
       <x:c r="E64" s="12" t="str">
-        <x:v>where-the-roof-door</x:v>
+        <x:v>station-was-moved</x:v>
       </x:c>
       <x:c r="F64" s="12" t="str">
-        <x:v>lessons/where-the-roof-door/level-7.txt</x:v>
+        <x:v>lessons/station-was-moved/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
       <x:c r="A65" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>GDM-37-4</x:v>
       </x:c>
       <x:c r="B65" s="12" t="str">
         <x:v>Long</x:v>
@@ -2471,18 +2471,18 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D65" s="12" t="str">
-        <x:v>The Traveling Shadow Ticket</x:v>
+        <x:v>Where the Roof Door Opens</x:v>
       </x:c>
       <x:c r="E65" s="12" t="str">
-        <x:v>traveling-shadow-ticket</x:v>
+        <x:v>where-the-roof-door</x:v>
       </x:c>
       <x:c r="F65" s="12" t="str">
-        <x:v>lessons/traveling-shadow-ticket/level-7.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66" ht="24" hidden="0" customHeight="1">
+        <x:v>lessons/where-the-roof-door/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="15" hidden="0" customHeight="1">
       <x:c r="A66" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B66" s="12" t="str">
         <x:v>Long</x:v>
@@ -2491,18 +2491,18 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D66" s="12" t="str">
-        <x:v>Because the Wall Listened</x:v>
+        <x:v>The Traveling Shadow Ticket</x:v>
       </x:c>
       <x:c r="E66" s="12" t="str">
-        <x:v>because-the-wall-listened</x:v>
+        <x:v>traveling-shadow-ticket</x:v>
       </x:c>
       <x:c r="F66" s="12" t="str">
-        <x:v>lessons/because-the-wall-listened/level-7.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67" ht="15" hidden="0" customHeight="1">
+        <x:v>lessons/traveling-shadow-ticket/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="24" hidden="0" customHeight="1">
       <x:c r="A67" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B67" s="12" t="str">
         <x:v>Long</x:v>
@@ -2511,18 +2511,18 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D67" s="12" t="str">
-        <x:v>How to Read the Stone</x:v>
+        <x:v>Because the Wall Listened</x:v>
       </x:c>
       <x:c r="E67" s="12" t="str">
-        <x:v>how-to-read-the-stone</x:v>
+        <x:v>because-the-wall-listened</x:v>
       </x:c>
       <x:c r="F67" s="12" t="str">
-        <x:v>lessons/how-to-read-the-stone/level-7.txt</x:v>
+        <x:v>lessons/because-the-wall-listened/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
       <x:c r="A68" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B68" s="12" t="str">
         <x:v>Long</x:v>
@@ -2531,33 +2531,33 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D68" s="12" t="str">
-        <x:v>More Than One Moon</x:v>
+        <x:v>How to Read the Stone</x:v>
       </x:c>
       <x:c r="E68" s="12" t="str">
-        <x:v>more-than-one-moon</x:v>
+        <x:v>how-to-read-the-stone</x:v>
       </x:c>
       <x:c r="F68" s="12" t="str">
-        <x:v>lessons/more-than-one-moon/level-7.txt</x:v>
+        <x:v>lessons/how-to-read-the-stone/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
       <x:c r="A69" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B69" s="12" t="str">
-        <x:v>Very Long</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C69" s="12" t="str">
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D69" s="12" t="str">
-        <x:v>The Locked Umbrella Room</x:v>
+        <x:v>More Than One Moon</x:v>
       </x:c>
       <x:c r="E69" s="12" t="str">
-        <x:v>locked-umbrella-room</x:v>
+        <x:v>more-than-one-moon</x:v>
       </x:c>
       <x:c r="F69" s="12" t="str">
-        <x:v>lessons/locked-umbrella-room/level-8.txt</x:v>
+        <x:v>lessons/more-than-one-moon/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
@@ -2568,16 +2568,16 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C70" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D70" s="12" t="str">
-        <x:v>The Last Seat at the Table</x:v>
+        <x:v>The Locked Umbrella Room</x:v>
       </x:c>
       <x:c r="E70" s="12" t="str">
-        <x:v>last-seat-table</x:v>
+        <x:v>locked-umbrella-room</x:v>
       </x:c>
       <x:c r="F70" s="12" t="str">
-        <x:v>lessons/last-seat-table/level-8.txt</x:v>
+        <x:v>lessons/locked-umbrella-room/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="15" hidden="0" customHeight="1">
@@ -2588,16 +2588,16 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C71" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D71" s="12" t="str">
-        <x:v>The Library That Was Moved</x:v>
+        <x:v>The Last Seat at the Table</x:v>
       </x:c>
       <x:c r="E71" s="12" t="str">
-        <x:v>library-moved</x:v>
+        <x:v>last-seat-table</x:v>
       </x:c>
       <x:c r="F71" s="12" t="str">
-        <x:v>lessons/library-moved/level-8.txt</x:v>
+        <x:v>lessons/last-seat-table/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="15" hidden="0" customHeight="1">
@@ -2608,16 +2608,16 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C72" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D72" s="12" t="str">
-        <x:v>The Moon Lantern Path</x:v>
+        <x:v>The Library That Was Moved</x:v>
       </x:c>
       <x:c r="E72" s="12" t="str">
-        <x:v>moon-lantern-path</x:v>
+        <x:v>library-moved</x:v>
       </x:c>
       <x:c r="F72" s="12" t="str">
-        <x:v>lessons/moon-lantern-path/level-8.txt</x:v>
+        <x:v>lessons/library-moved/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="15" hidden="0" customHeight="1">
@@ -2628,16 +2628,16 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C73" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D73" s="12" t="str">
-        <x:v>The Folded Map Race</x:v>
+        <x:v>The Moon Lantern Path</x:v>
       </x:c>
       <x:c r="E73" s="12" t="str">
-        <x:v>folded-map-race</x:v>
+        <x:v>moon-lantern-path</x:v>
       </x:c>
       <x:c r="F73" s="12" t="str">
-        <x:v>lessons/folded-map-race/level-8.txt</x:v>
+        <x:v>lessons/moon-lantern-path/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="15" hidden="0" customHeight="1">
@@ -2648,15 +2648,35 @@
         <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C74" s="12" t="str">
+        <x:v>Adventure</x:v>
+      </x:c>
+      <x:c r="D74" s="12" t="str">
+        <x:v>The Folded Map Race</x:v>
+      </x:c>
+      <x:c r="E74" s="12" t="str">
+        <x:v>folded-map-race</x:v>
+      </x:c>
+      <x:c r="F74" s="12" t="str">
+        <x:v>lessons/folded-map-race/level-8.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="15" hidden="0" customHeight="1">
+      <x:c r="A75" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B75" s="12" t="str">
+        <x:v>Very Long</x:v>
+      </x:c>
+      <x:c r="C75" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
-      <x:c r="D74" s="12" t="str">
+      <x:c r="D75" s="12" t="str">
         <x:v>The Pudding Case</x:v>
       </x:c>
-      <x:c r="E74" s="12" t="str">
+      <x:c r="E75" s="12" t="str">
         <x:v>jaio-pudding-case</x:v>
       </x:c>
-      <x:c r="F74" s="12" t="str">
+      <x:c r="F75" s="12" t="str">
         <x:v>lessons/jaio-pudding-case/level-8.txt</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Add A-Z title coverage stories
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Rcf972c212868411a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R69ada2d3f23145de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R873d23f339e74af0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R18c6969c95f54d99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Rce026c2334ca4e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R1bd04693db354e22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R0409d47702064355"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="Rd8326c84a5cd4c88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="Ree7ce024b0ca4e46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R3434e8b6e81b432e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2680,6 +2680,326 @@
         <x:v>lessons/jaio-pudding-case/level-8.txt</x:v>
       </x:c>
     </x:row>
+    <x:row r="76" ht="15" hidden="0" customHeight="1">
+      <x:c r="A76" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B76" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C76" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D76" s="12" t="str">
+        <x:v>Another Door Opens</x:v>
+      </x:c>
+      <x:c r="E76" s="12" t="str">
+        <x:v>another-door-opens</x:v>
+      </x:c>
+      <x:c r="F76" s="12" t="str">
+        <x:v>lessons/another-door-opens/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="15" hidden="0" customHeight="1">
+      <x:c r="A77" s="12" t="str">
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
+      </x:c>
+      <x:c r="B77" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C77" s="12" t="str">
+        <x:v>SF</x:v>
+      </x:c>
+      <x:c r="D77" s="12" t="str">
+        <x:v>Echo on the Moon</x:v>
+      </x:c>
+      <x:c r="E77" s="12" t="str">
+        <x:v>echo-on-the-moon</x:v>
+      </x:c>
+      <x:c r="F77" s="12" t="str">
+        <x:v>lessons/echo-on-the-moon/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="15" hidden="0" customHeight="1">
+      <x:c r="A78" s="12" t="str">
+        <x:v>NH1-1-6-V</x:v>
+      </x:c>
+      <x:c r="B78" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C78" s="12" t="str">
+        <x:v>Human Drama</x:v>
+      </x:c>
+      <x:c r="D78" s="12" t="str">
+        <x:v>Inside the Kite</x:v>
+      </x:c>
+      <x:c r="E78" s="12" t="str">
+        <x:v>inside-the-kite</x:v>
+      </x:c>
+      <x:c r="F78" s="12" t="str">
+        <x:v>lessons/inside-the-kite/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="15" hidden="0" customHeight="1">
+      <x:c r="A79" s="12" t="str">
+        <x:v>NH2-2-1-3-SVOO</x:v>
+      </x:c>
+      <x:c r="B79" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C79" s="12" t="str">
+        <x:v>Comedy</x:v>
+      </x:c>
+      <x:c r="D79" s="12" t="str">
+        <x:v>Jiro's Quiet Joke</x:v>
+      </x:c>
+      <x:c r="E79" s="12" t="str">
+        <x:v>jiro-quiet-joke</x:v>
+      </x:c>
+      <x:c r="F79" s="12" t="str">
+        <x:v>lessons/jiro-quiet-joke/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="15" hidden="0" customHeight="1">
+      <x:c r="A80" s="12" t="str">
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
+      </x:c>
+      <x:c r="B80" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C80" s="12" t="str">
+        <x:v>Adventure</x:v>
+      </x:c>
+      <x:c r="D80" s="12" t="str">
+        <x:v>Kaito's Key Map</x:v>
+      </x:c>
+      <x:c r="E80" s="12" t="str">
+        <x:v>kaito-key-map</x:v>
+      </x:c>
+      <x:c r="F80" s="12" t="str">
+        <x:v>lessons/kaito-key-map/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="15" hidden="0" customHeight="1">
+      <x:c r="A81" s="12" t="str">
+        <x:v>NH1-1-11-1-MAYBE</x:v>
+      </x:c>
+      <x:c r="B81" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C81" s="12" t="str">
+        <x:v>Fantasy / Adventure</x:v>
+      </x:c>
+      <x:c r="D81" s="12" t="str">
+        <x:v>Noa and the Night Door</x:v>
+      </x:c>
+      <x:c r="E81" s="12" t="str">
+        <x:v>noa-night-door</x:v>
+      </x:c>
+      <x:c r="F81" s="12" t="str">
+        <x:v>lessons/noa-night-door/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="15" hidden="0" customHeight="1">
+      <x:c r="A82" s="12" t="str">
+        <x:v>NH2-2-3-1-SHOULD</x:v>
+      </x:c>
+      <x:c r="B82" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C82" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D82" s="12" t="str">
+        <x:v>Under the Red Desk</x:v>
+      </x:c>
+      <x:c r="E82" s="12" t="str">
+        <x:v>under-red-desk</x:v>
+      </x:c>
+      <x:c r="F82" s="12" t="str">
+        <x:v>lessons/under-red-desk/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="15" hidden="0" customHeight="1">
+      <x:c r="A83" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B83" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C83" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D83" s="12" t="str">
+        <x:v>Voices in the Wall</x:v>
+      </x:c>
+      <x:c r="E83" s="12" t="str">
+        <x:v>voices-in-wall</x:v>
+      </x:c>
+      <x:c r="F83" s="12" t="str">
+        <x:v>lessons/voices-in-wall/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="15" hidden="0" customHeight="1">
+      <x:c r="A84" s="12" t="str">
+        <x:v>NH2-2-6-MORE-THAN</x:v>
+      </x:c>
+      <x:c r="B84" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C84" s="12" t="str">
+        <x:v>Adventure</x:v>
+      </x:c>
+      <x:c r="D84" s="12" t="str">
+        <x:v>X Marks the Lunch Box</x:v>
+      </x:c>
+      <x:c r="E84" s="12" t="str">
+        <x:v>x-marks-lunch-box</x:v>
+      </x:c>
+      <x:c r="F84" s="12" t="str">
+        <x:v>lessons/x-marks-lunch-box/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="15" hidden="0" customHeight="1">
+      <x:c r="A85" s="12" t="str">
+        <x:v>NH1-0-FAMILY</x:v>
+      </x:c>
+      <x:c r="B85" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C85" s="12" t="str">
+        <x:v>Human Drama</x:v>
+      </x:c>
+      <x:c r="D85" s="12" t="str">
+        <x:v>Yuna's Thank-You Note</x:v>
+      </x:c>
+      <x:c r="E85" s="12" t="str">
+        <x:v>yuna-thank-you-note</x:v>
+      </x:c>
+      <x:c r="F85" s="12" t="str">
+        <x:v>lessons/yuna-thank-you-note/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="15" hidden="0" customHeight="1">
+      <x:c r="A86" s="12" t="str">
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+      </x:c>
+      <x:c r="B86" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C86" s="12" t="str">
+        <x:v>SF</x:v>
+      </x:c>
+      <x:c r="D86" s="12" t="str">
+        <x:v>Zero at the Station</x:v>
+      </x:c>
+      <x:c r="E86" s="12" t="str">
+        <x:v>zero-at-station</x:v>
+      </x:c>
+      <x:c r="F86" s="12" t="str">
+        <x:v>lessons/zero-at-station/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="15" hidden="0" customHeight="1">
+      <x:c r="A87" s="12" t="str">
+        <x:v>GDM-22</x:v>
+      </x:c>
+      <x:c r="B87" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C87" s="12" t="str">
+        <x:v>SF</x:v>
+      </x:c>
+      <x:c r="D87" s="12" t="str">
+        <x:v>Green Glass Signal</x:v>
+      </x:c>
+      <x:c r="E87" s="12" t="str">
+        <x:v>green-glass-signal</x:v>
+      </x:c>
+      <x:c r="F87" s="12" t="str">
+        <x:v>lessons/green-glass-signal/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="15" hidden="0" customHeight="1">
+      <x:c r="A88" s="12" t="str">
+        <x:v>NH1-1-10-V</x:v>
+      </x:c>
+      <x:c r="B88" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C88" s="12" t="str">
+        <x:v>Human Drama</x:v>
+      </x:c>
+      <x:c r="D88" s="12" t="str">
+        <x:v>Lost Library Card</x:v>
+      </x:c>
+      <x:c r="E88" s="12" t="str">
+        <x:v>lost-library-card</x:v>
+      </x:c>
+      <x:c r="F88" s="12" t="str">
+        <x:v>lessons/lost-library-card/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="15" hidden="0" customHeight="1">
+      <x:c r="A89" s="12" t="str">
+        <x:v>NH1-1-5-2-DONTBE</x:v>
+      </x:c>
+      <x:c r="B89" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C89" s="12" t="str">
+        <x:v>Comedy</x:v>
+      </x:c>
+      <x:c r="D89" s="12" t="str">
+        <x:v>Open on Monday</x:v>
+      </x:c>
+      <x:c r="E89" s="12" t="str">
+        <x:v>open-on-monday</x:v>
+      </x:c>
+      <x:c r="F89" s="12" t="str">
+        <x:v>lessons/open-on-monday/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="15" hidden="0" customHeight="1">
+      <x:c r="A90" s="12" t="str">
+        <x:v>NH1-1-3-CAN-Q</x:v>
+      </x:c>
+      <x:c r="B90" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C90" s="12" t="str">
+        <x:v>Fantasy</x:v>
+      </x:c>
+      <x:c r="D90" s="12" t="str">
+        <x:v>Paper Star Plan</x:v>
+      </x:c>
+      <x:c r="E90" s="12" t="str">
+        <x:v>paper-star-plan</x:v>
+      </x:c>
+      <x:c r="F90" s="12" t="str">
+        <x:v>lessons/paper-star-plan/level-3.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="15" hidden="0" customHeight="1">
+      <x:c r="A91" s="12" t="str">
+        <x:v>NH2-2-3-1-SHOULD</x:v>
+      </x:c>
+      <x:c r="B91" s="12" t="str">
+        <x:v>Short</x:v>
+      </x:c>
+      <x:c r="C91" s="12" t="str">
+        <x:v>Mystery</x:v>
+      </x:c>
+      <x:c r="D91" s="12" t="str">
+        <x:v>Quiet Question</x:v>
+      </x:c>
+      <x:c r="E91" s="12" t="str">
+        <x:v>quiet-question</x:v>
+      </x:c>
+      <x:c r="F91" s="12" t="str">
+        <x:v>lessons/quiet-question/level-3.txt</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Clarify Little Door sequence titles
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R1bd04693db354e22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R0409d47702064355"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="Rd8326c84a5cd4c88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="Ree7ce024b0ca4e46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R3434e8b6e81b432e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R4a144bf596c14f58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Refdbeaababc44440"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R2011c0c1baf44959"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R96ee6e5c2f2248f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R2c72a93bb7874bfc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1491,7 +1491,7 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>The Little Door</x:v>
+        <x:v>The Little Door, Part 1</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
         <x:v>graded-story</x:v>

</xml_diff>

<commit_message>
Move water pen trick to make introduction ID
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R4a144bf596c14f58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Refdbeaababc44440"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R2011c0c1baf44959"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R96ee6e5c2f2248f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R2c72a93bb7874bfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Re77bd8b9a8b54217"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R93f39098b1d04297"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R461ffc453757412e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R134f29f6f78b465b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R6f26b0ac8ff54351"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -922,7 +922,7 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH1-1-7-V</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
         <x:v>NH1</x:v>
@@ -931,16 +931,16 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>1-8-3</x:v>
+        <x:v>1-7</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>Why</x:v>
+        <x:v>know / make / buy</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
-        <x:v>疑問詞</x:v>
+        <x:v>一般動詞</x:v>
       </x:c>
       <x:c r="G15" s="12" t="str">
-        <x:v>理由を問うことで次の展開を作る。</x:v>
+        <x:v>知る、作る、買うを使う。</x:v>
       </x:c>
       <x:c r="H15" s="12" t="str">
         <x:v>NH1画像転記</x:v>
@@ -948,7 +948,7 @@
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
         <x:v>NH1</x:v>
@@ -957,16 +957,16 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>1-10</x:v>
+        <x:v>1-8-3</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>travel / visit / listen / spend / stand / feel / get up</x:v>
+        <x:v>Why</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>一般動詞</x:v>
+        <x:v>疑問詞</x:v>
       </x:c>
       <x:c r="G16" s="12" t="str">
-        <x:v>外出・訪問・気持ちを扱う。</x:v>
+        <x:v>理由を問うことで次の展開を作る。</x:v>
       </x:c>
       <x:c r="H16" s="12" t="str">
         <x:v>NH1画像転記</x:v>
@@ -974,7 +974,7 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
         <x:v>NH1</x:v>
@@ -983,16 +983,16 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>1-11-1</x:v>
+        <x:v>1-10</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
-        <x:v>maybe</x:v>
+        <x:v>travel / visit / listen / spend / stand / feel / get up</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
-        <x:v>副詞</x:v>
+        <x:v>一般動詞</x:v>
       </x:c>
       <x:c r="G17" s="12" t="str">
-        <x:v>推測を入れてミステリー感を作る。</x:v>
+        <x:v>外出・訪問・気持ちを扱う。</x:v>
       </x:c>
       <x:c r="H17" s="12" t="str">
         <x:v>NH1画像転記</x:v>
@@ -1000,33 +1000,33 @@
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>NH2</x:v>
+        <x:v>NH1</x:v>
       </x:c>
       <x:c r="C18" s="12" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
-        <x:v>2-1-3</x:v>
+        <x:v>1-11-1</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>SVOO: show / teach / give</x:v>
+        <x:v>maybe</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
-        <x:v>文型</x:v>
+        <x:v>副詞</x:v>
       </x:c>
       <x:c r="G18" s="12" t="str">
-        <x:v>誰が誰に何をするかを明確にする。</x:v>
+        <x:v>推測を入れてミステリー感を作る。</x:v>
       </x:c>
       <x:c r="H18" s="12" t="str">
-        <x:v>NH2画像転記</x:v>
+        <x:v>NH1画像転記</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
         <x:v>NH2</x:v>
@@ -1035,16 +1035,16 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
-        <x:v>2-2-4</x:v>
+        <x:v>2-1-3</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>because</x:v>
+        <x:v>SVOO: show / teach / give</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
-        <x:v>接続詞</x:v>
+        <x:v>文型</x:v>
       </x:c>
       <x:c r="G19" s="12" t="str">
-        <x:v>理由を本文の中で説明する。</x:v>
+        <x:v>誰が誰に何をするかを明確にする。</x:v>
       </x:c>
       <x:c r="H19" s="12" t="str">
         <x:v>NH2画像転記</x:v>
@@ -1052,7 +1052,7 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
         <x:v>NH2</x:v>
@@ -1061,16 +1061,16 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
-        <x:v>2-3-1</x:v>
+        <x:v>2-2-4</x:v>
       </x:c>
       <x:c r="E20" s="12" t="str">
-        <x:v>should</x:v>
+        <x:v>because</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
-        <x:v>助動詞</x:v>
+        <x:v>接続詞</x:v>
       </x:c>
       <x:c r="G20" s="12" t="str">
-        <x:v>助言や判断を話の転機に使う。</x:v>
+        <x:v>理由を本文の中で説明する。</x:v>
       </x:c>
       <x:c r="H20" s="12" t="str">
         <x:v>NH2画像転記</x:v>
@@ -1078,7 +1078,7 @@
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
         <x:v>NH2</x:v>
@@ -1087,16 +1087,16 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="D21" s="12" t="str">
-        <x:v>2-4-1</x:v>
+        <x:v>2-3-1</x:v>
       </x:c>
       <x:c r="E21" s="12" t="str">
-        <x:v>have to</x:v>
+        <x:v>should</x:v>
       </x:c>
       <x:c r="F21" s="12" t="str">
-        <x:v>助動詞相当</x:v>
+        <x:v>助動詞</x:v>
       </x:c>
       <x:c r="G21" s="12" t="str">
-        <x:v>しなければならない理由を作る。</x:v>
+        <x:v>助言や判断を話の転機に使う。</x:v>
       </x:c>
       <x:c r="H21" s="12" t="str">
         <x:v>NH2画像転記</x:v>
@@ -1104,7 +1104,7 @@
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
         <x:v>NH2</x:v>
@@ -1113,16 +1113,16 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>2-5-1</x:v>
+        <x:v>2-4-1</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>how to do</x:v>
+        <x:v>have to</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
-        <x:v>疑問詞 + 不定詞</x:v>
+        <x:v>助動詞相当</x:v>
       </x:c>
       <x:c r="G22" s="12" t="str">
-        <x:v>方法を知ることが解決につながる話。</x:v>
+        <x:v>しなければならない理由を作る。</x:v>
       </x:c>
       <x:c r="H22" s="12" t="str">
         <x:v>NH2画像転記</x:v>
@@ -1130,7 +1130,7 @@
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
         <x:v>NH2</x:v>
@@ -1139,24 +1139,24 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>2-6</x:v>
+        <x:v>2-5-1</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>more than / half</x:v>
+        <x:v>how to do</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
-        <x:v>比較</x:v>
+        <x:v>疑問詞 + 不定詞</x:v>
       </x:c>
       <x:c r="G23" s="12" t="str">
-        <x:v>数や量の比較を使う。</x:v>
+        <x:v>方法を知ることが解決につながる話。</x:v>
       </x:c>
       <x:c r="H23" s="12" t="str">
         <x:v>NH2画像転記</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="24" hidden="0" customHeight="1">
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
         <x:v>NH2</x:v>
@@ -1165,18 +1165,44 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
+        <x:v>2-6</x:v>
+      </x:c>
+      <x:c r="E24" s="12" t="str">
+        <x:v>more than / half</x:v>
+      </x:c>
+      <x:c r="F24" s="12" t="str">
+        <x:v>比較</x:v>
+      </x:c>
+      <x:c r="G24" s="12" t="str">
+        <x:v>数や量の比較を使う。</x:v>
+      </x:c>
+      <x:c r="H24" s="12" t="str">
+        <x:v>NH2画像転記</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="24" hidden="0" customHeight="1">
+      <x:c r="A25" s="12" t="str">
+        <x:v>NH2-2-7-2-VOICE</x:v>
+      </x:c>
+      <x:c r="B25" s="12" t="str">
+        <x:v>NH2</x:v>
+      </x:c>
+      <x:c r="C25" s="12" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D25" s="12" t="str">
         <x:v>2-7-2</x:v>
       </x:c>
-      <x:c r="E24" s="12" t="str">
+      <x:c r="E25" s="12" t="str">
         <x:v>受け身</x:v>
       </x:c>
-      <x:c r="F24" s="12" t="str">
+      <x:c r="F25" s="12" t="str">
         <x:v>何が誰によって行われたかを説明する。</x:v>
       </x:c>
-      <x:c r="G24" s="12" t="str">
+      <x:c r="G25" s="12" t="str">
         <x:v>NH2画像転記</x:v>
       </x:c>
-      <x:c r="H24" s="12"/>
+      <x:c r="H25" s="12"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1442,7 +1468,7 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>NH1-1-7-V</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
         <x:v>Short</x:v>

</xml_diff>

<commit_message>
Handle feedback thank-you and Little Door grading
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Re77bd8b9a8b54217"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R93f39098b1d04297"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R461ffc453757412e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R134f29f6f78b465b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R6f26b0ac8ff54351"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R610307952bbf4b04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R67bf78dec1064379"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R060e6ba424e44d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="Ra18c90a4068b4024"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R42df9717b1fa4c74"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1288,7 +1288,7 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
         <x:v>Very Short</x:v>

</xml_diff>

<commit_message>
Move Red Pin to see introduction ID
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R610307952bbf4b04"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R67bf78dec1064379"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R060e6ba424e44d78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="Ra18c90a4068b4024"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R42df9717b1fa4c74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R48719c8ac9834417"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Ree4264c7f81148b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R6d8e6a99e06c4653"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R77e4e16f70664d44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Ra3ebf699639f4d6a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1428,7 +1428,7 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
         <x:v>Short</x:v>

</xml_diff>

<commit_message>
Add strict grading audit
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R48719c8ac9834417"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Ree4264c7f81148b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R6d8e6a99e06c4653"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R77e4e16f70664d44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Ra3ebf699639f4d6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R793fd7c571cd4e8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R26e033bb70f447a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="Rd0414edad7b54230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="Rea9fcce36adb4077"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R671fbdd41ff64d52"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1308,7 +1308,7 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
         <x:v>Very Short</x:v>
@@ -1328,7 +1328,7 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
         <x:v>Very Short</x:v>
@@ -1348,7 +1348,7 @@
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
         <x:v>Very Short</x:v>
@@ -1368,7 +1368,7 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
         <x:v>Very Short</x:v>
@@ -1388,7 +1388,7 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
         <x:v>Very Short</x:v>
@@ -1408,7 +1408,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
         <x:v>Very Short</x:v>
@@ -1448,7 +1448,7 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>GDM-10</x:v>
+        <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
         <x:v>Short</x:v>
@@ -1488,7 +1488,7 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
         <x:v>Short</x:v>
@@ -1508,7 +1508,7 @@
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
         <x:v>Short</x:v>
@@ -1528,7 +1528,7 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>NH1-0-FAMILY</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
         <x:v>Short</x:v>
@@ -1548,7 +1548,7 @@
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
         <x:v>Short</x:v>
@@ -1568,7 +1568,7 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
         <x:v>Long</x:v>
@@ -1608,7 +1608,7 @@
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
         <x:v>Long</x:v>
@@ -1628,7 +1628,7 @@
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
         <x:v>Long</x:v>
@@ -1648,7 +1648,7 @@
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
         <x:v>Short</x:v>
@@ -1668,7 +1668,7 @@
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
         <x:v>Long</x:v>
@@ -1688,7 +1688,7 @@
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
         <x:v>Short</x:v>
@@ -1708,7 +1708,7 @@
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
         <x:v>Short</x:v>
@@ -1728,7 +1728,7 @@
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
         <x:v>Long</x:v>
@@ -1748,7 +1748,7 @@
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
         <x:v>Long</x:v>
@@ -1768,7 +1768,7 @@
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
         <x:v>Short</x:v>
@@ -1788,7 +1788,7 @@
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
         <x:v>Long</x:v>
@@ -1828,7 +1828,7 @@
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B32" s="12" t="str">
         <x:v>Long</x:v>
@@ -1868,7 +1868,7 @@
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B34" s="12" t="str">
         <x:v>Long</x:v>
@@ -1988,7 +1988,7 @@
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="12" t="str">
-        <x:v>GDM-1</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B40" s="12" t="str">
         <x:v>Long</x:v>
@@ -2008,7 +2008,7 @@
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="12" t="str">
-        <x:v>GDM-10</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B41" s="12" t="str">
         <x:v>Long</x:v>
@@ -2028,7 +2028,7 @@
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B42" s="12" t="str">
         <x:v>Long</x:v>
@@ -2048,7 +2048,7 @@
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B43" s="12" t="str">
         <x:v>Long</x:v>
@@ -2068,7 +2068,7 @@
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B44" s="12" t="str">
         <x:v>Long</x:v>
@@ -2088,7 +2088,7 @@
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="12" t="str">
-        <x:v>NH1-0-FAMILY</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B45" s="12" t="str">
         <x:v>Long</x:v>
@@ -2108,7 +2108,7 @@
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B46" s="12" t="str">
         <x:v>Long</x:v>
@@ -2128,7 +2128,7 @@
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B47" s="12" t="str">
         <x:v>Long</x:v>
@@ -2188,7 +2188,7 @@
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B50" s="12" t="str">
         <x:v>Long</x:v>
@@ -2208,7 +2208,7 @@
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B51" s="12" t="str">
         <x:v>Short</x:v>
@@ -2228,7 +2228,7 @@
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B52" s="12" t="str">
         <x:v>Short</x:v>
@@ -2268,7 +2268,7 @@
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B54" s="12" t="str">
         <x:v>Short</x:v>
@@ -2308,7 +2308,7 @@
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>NH1-1-7-V</x:v>
       </x:c>
       <x:c r="B56" s="12" t="str">
         <x:v>Short</x:v>
@@ -2328,7 +2328,7 @@
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B57" s="12" t="str">
         <x:v>Short</x:v>
@@ -2348,7 +2348,7 @@
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B58" s="12" t="str">
         <x:v>Short</x:v>
@@ -2368,7 +2368,7 @@
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B59" s="12" t="str">
         <x:v>Long</x:v>
@@ -2388,7 +2388,7 @@
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
       <x:c r="A60" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B60" s="12" t="str">
         <x:v>Short</x:v>
@@ -2408,7 +2408,7 @@
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B61" s="12" t="str">
         <x:v>Short</x:v>
@@ -2428,7 +2428,7 @@
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
       <x:c r="A62" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B62" s="12" t="str">
         <x:v>Short</x:v>
@@ -2488,7 +2488,7 @@
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
       <x:c r="A65" s="12" t="str">
-        <x:v>GDM-37-4</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B65" s="12" t="str">
         <x:v>Long</x:v>
@@ -2508,7 +2508,7 @@
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
       <x:c r="A66" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B66" s="12" t="str">
         <x:v>Long</x:v>
@@ -2528,7 +2528,7 @@
     </x:row>
     <x:row r="67" ht="24" hidden="0" customHeight="1">
       <x:c r="A67" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B67" s="12" t="str">
         <x:v>Long</x:v>
@@ -2548,7 +2548,7 @@
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
       <x:c r="A68" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B68" s="12" t="str">
         <x:v>Long</x:v>
@@ -2768,7 +2768,7 @@
     </x:row>
     <x:row r="79" ht="15" hidden="0" customHeight="1">
       <x:c r="A79" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B79" s="12" t="str">
         <x:v>Short</x:v>
@@ -2808,7 +2808,7 @@
     </x:row>
     <x:row r="81" ht="15" hidden="0" customHeight="1">
       <x:c r="A81" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B81" s="12" t="str">
         <x:v>Short</x:v>
@@ -2888,7 +2888,7 @@
     </x:row>
     <x:row r="85" ht="15" hidden="0" customHeight="1">
       <x:c r="A85" s="12" t="str">
-        <x:v>NH1-0-FAMILY</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B85" s="12" t="str">
         <x:v>Short</x:v>
@@ -2928,7 +2928,7 @@
     </x:row>
     <x:row r="87" ht="15" hidden="0" customHeight="1">
       <x:c r="A87" s="12" t="str">
-        <x:v>GDM-22</x:v>
+        <x:v>NH1-1-7-V</x:v>
       </x:c>
       <x:c r="B87" s="12" t="str">
         <x:v>Short</x:v>
@@ -2948,7 +2948,7 @@
     </x:row>
     <x:row r="88" ht="15" hidden="0" customHeight="1">
       <x:c r="A88" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B88" s="12" t="str">
         <x:v>Short</x:v>
@@ -2968,7 +2968,7 @@
     </x:row>
     <x:row r="89" ht="15" hidden="0" customHeight="1">
       <x:c r="A89" s="12" t="str">
-        <x:v>NH1-1-5-2-DONTBE</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B89" s="12" t="str">
         <x:v>Short</x:v>
@@ -2988,7 +2988,7 @@
     </x:row>
     <x:row r="90" ht="15" hidden="0" customHeight="1">
       <x:c r="A90" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>NH1-1-7-V</x:v>
       </x:c>
       <x:c r="B90" s="12" t="str">
         <x:v>Short</x:v>

</xml_diff>

<commit_message>
Remove very short readings
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R793fd7c571cd4e8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R26e033bb70f447a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="Rd0414edad7b54230"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="Rea9fcce36adb4077"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R671fbdd41ff64d52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Ra8f40eb5d7194df3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rb82c59b5f0df4f83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R746569450e604acc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R53414046d44746d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R75d70dcb25e44385"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -365,10 +365,10 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のIDを一本で指定する。本文量はVery Short / Short / Long / Very Longから選ぶ。</x:v>
+        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のIDを一本で指定する。本文量はShort / Long / Very Longから選ぶ。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のIDを一本で指定する。本文量はVery Short / Short / Long / Very Longから選ぶ。</x:v>
+        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のIDを一本で指定する。本文量はShort / Long / Very Longから選ぶ。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -409,7 +409,7 @@
         <x:v>本文量</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>Very Shortはごく短い導入用。Shortは120〜180語程度。Longは300〜450語程度。Very Longは650〜900語程度。UIでは旧段階表記を使わない。</x:v>
+        <x:v>Shortは120〜180語程度。Longは300〜450語程度。Very Longは650〜900語程度。UIでは旧段階表記を使わない。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -496,7 +496,7 @@
         <x:v>このIDまでのGDM/NH項目を使用可</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="24" hidden="0" customHeight="1">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
         <x:v>Length</x:v>
       </x:c>
@@ -504,10 +504,10 @@
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>Very Short / Short / Long / Very Long</x:v>
+        <x:v>Short / Long / Very Long</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>Very Short=ごく短い導入、Short=120〜180語程度、Long=300〜450語程度、Very Long=650〜900語程度</x:v>
+        <x:v>Short=120〜180語程度、Long=300〜450語程度、Very Long=650〜900語程度</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1291,319 +1291,319 @@
         <x:v>GDM-41-10</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>Very Short</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>The Little Door</x:v>
+        <x:v>The Red Pin</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>graded-story</x:v>
+        <x:v>red-pin</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
-        <x:v>lessons/graded-story/level-1.txt</x:v>
+        <x:v>lessons/red-pin/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>NH1-1-1-V</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>Very Short</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>The Blue Lunch Box</x:v>
+        <x:v>The Book Under the Hat</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
-        <x:v>blue-lunch-box</x:v>
+        <x:v>book-under-hat</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
-        <x:v>lessons/blue-lunch-box/level-1.txt</x:v>
+        <x:v>lessons/book-under-hat/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>NH1-1-7-V</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>Very Short</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Water Pen Trick</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>water-pen-trick</x:v>
       </x:c>
       <x:c r="F7" s="12" t="str">
-        <x:v>lessons/bread-shop/level-1.txt</x:v>
+        <x:v>lessons/water-pen-trick/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>Very Short</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>The Star Bus</x:v>
+        <x:v>Where Is the Bell?</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>star-bus</x:v>
+        <x:v>where-is-the-bell</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
-        <x:v>lessons/star-bus/level-1.txt</x:v>
+        <x:v>lessons/where-is-the-bell/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Very Short</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
-        <x:v>The Silver Stone</x:v>
+        <x:v>The Little Door, Part 1</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>silver-stone</x:v>
+        <x:v>graded-story</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
-        <x:v>lessons/silver-stone/level-1.txt</x:v>
+        <x:v>lessons/graded-story/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>Very Short</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C10" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
-        <x:v>The Red Bag Path</x:v>
+        <x:v>Rina's Brother</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>red-bag-path</x:v>
+        <x:v>rina-brother</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
-        <x:v>lessons/red-bag-path/level-1.txt</x:v>
+        <x:v>lessons/rina-brother/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
-        <x:v>NH1-1-8-3-WHY</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>Very Short</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>wrong-robot</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-1.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="12" t="str">
-        <x:v>GDM-41-10</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
-        <x:v>The Red Pin</x:v>
+        <x:v>The Rainy Club Map</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>red-pin</x:v>
+        <x:v>rainy-club-map</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
-        <x:v>lessons/red-pin/level-3.txt</x:v>
+        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="str">
-        <x:v>NH1-1-1-V</x:v>
+        <x:v>NH1-1-3-CAN-Q</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>The Book Under the Hat</x:v>
+        <x:v>The Star Bus</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>book-under-hat</x:v>
+        <x:v>star-bus</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
-        <x:v>lessons/book-under-hat/level-3.txt</x:v>
+        <x:v>lessons/star-bus/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="12" t="str">
-        <x:v>NH1-1-7-V</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C14" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
-        <x:v>The Water Pen Trick</x:v>
+        <x:v>Can the Clock Sing?</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
-        <x:v>water-pen-trick</x:v>
+        <x:v>can-clock-sing</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>lessons/water-pen-trick/level-3.txt</x:v>
+        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C15" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D15" s="12" t="str">
-        <x:v>Where Is the Bell?</x:v>
+        <x:v>Can the Principal Dance?</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>where-is-the-bell</x:v>
+        <x:v>principal-dance</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
-        <x:v>lessons/where-is-the-bell/level-3.txt</x:v>
+        <x:v>lessons/principal-dance/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
-        <x:v>The Little Door, Part 1</x:v>
+        <x:v>The Wrong Robot</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>graded-story</x:v>
+        <x:v>wrong-robot</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>lessons/graded-story/level-3.txt</x:v>
+        <x:v>lessons/wrong-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str">
         <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>Rina's Brother</x:v>
+        <x:v>Don't Be a Hero</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
-        <x:v>rina-brother</x:v>
+        <x:v>dont-be-a-hero</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
-        <x:v>lessons/rina-brother/level-3.txt</x:v>
+        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Window Note</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>window-note</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/window-note/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C19" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
-        <x:v>The Rainy Club Map</x:v>
+        <x:v>The Moon Cup</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>rainy-club-map</x:v>
+        <x:v>moon-cup</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
-        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
+        <x:v>lessons/moon-cup/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="12" t="str">
-        <x:v>NH1-1-3-CAN-Q</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C20" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
-        <x:v>The Star Bus</x:v>
+        <x:v>The Rainy Club Map</x:v>
       </x:c>
       <x:c r="E20" s="12" t="str">
-        <x:v>star-bus</x:v>
+        <x:v>rainy-club-map</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
-        <x:v>lessons/star-bus/level-3.txt</x:v>
+        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -1628,207 +1628,207 @@
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C22" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>Can the Principal Dance?</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>principal-dance</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
-        <x:v>lessons/principal-dance/level-7.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C23" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>wrong-robot</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-3.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C24" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>Don't Be a Hero</x:v>
+        <x:v>The Wrong Robot</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
-        <x:v>dont-be-a-hero</x:v>
+        <x:v>wrong-robot</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
-        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
+        <x:v>lessons/wrong-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
-        <x:v>The Window Note</x:v>
+        <x:v>Because the Hat Said No</x:v>
       </x:c>
       <x:c r="E25" s="12" t="str">
-        <x:v>window-note</x:v>
+        <x:v>hat-said-no</x:v>
       </x:c>
       <x:c r="F25" s="12" t="str">
-        <x:v>lessons/window-note/level-3.txt</x:v>
+        <x:v>lessons/hat-said-no/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C26" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D26" s="12" t="str">
-        <x:v>The Moon Cup</x:v>
+        <x:v>Don't Be a Hero</x:v>
       </x:c>
       <x:c r="E26" s="12" t="str">
-        <x:v>moon-cup</x:v>
+        <x:v>dont-be-a-hero</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
-        <x:v>lessons/moon-cup/level-3.txt</x:v>
+        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C27" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D27" s="12" t="str">
-        <x:v>The Rainy Club Map</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E27" s="12" t="str">
-        <x:v>rainy-club-map</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F27" s="12" t="str">
-        <x:v>lessons/rainy-club-map/level-7.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str">
         <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
-        <x:v>Can the Clock Sing?</x:v>
+        <x:v>The Moon Cup</x:v>
       </x:c>
       <x:c r="E28" s="12" t="str">
-        <x:v>can-clock-sing</x:v>
+        <x:v>moon-cup</x:v>
       </x:c>
       <x:c r="F28" s="12" t="str">
-        <x:v>lessons/can-clock-sing/level-7.txt</x:v>
+        <x:v>lessons/moon-cup/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Fantasy / Adventure</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Dice Gate</x:v>
       </x:c>
       <x:c r="E29" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>dice-gate</x:v>
       </x:c>
       <x:c r="F29" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/dice-gate/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>The Quiet Bread Shop</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>bread-shop</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/bread-shop/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C31" s="12" t="str">
         <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
-        <x:v>The Wrong Robot</x:v>
+        <x:v>The Gift Lesson</x:v>
       </x:c>
       <x:c r="E31" s="12" t="str">
-        <x:v>wrong-robot</x:v>
+        <x:v>gift-lesson</x:v>
       </x:c>
       <x:c r="F31" s="12" t="str">
-        <x:v>lessons/wrong-robot/level-3.txt</x:v>
+        <x:v>lessons/gift-lesson/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B32" s="12" t="str">
         <x:v>Long</x:v>
@@ -1837,158 +1837,158 @@
         <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D32" s="12" t="str">
-        <x:v>Because the Hat Said No</x:v>
+        <x:v>The Cake Was Moved</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
-        <x:v>hat-said-no</x:v>
+        <x:v>cake-was-moved</x:v>
       </x:c>
       <x:c r="F32" s="12" t="str">
-        <x:v>lessons/hat-said-no/level-7.txt</x:v>
+        <x:v>lessons/cake-was-moved/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B33" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C33" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D33" s="12" t="str">
-        <x:v>Don't Be a Hero</x:v>
+        <x:v>The Red Pin Parade</x:v>
       </x:c>
       <x:c r="E33" s="12" t="str">
-        <x:v>dont-be-a-hero</x:v>
+        <x:v>red-pin-parade</x:v>
       </x:c>
       <x:c r="F33" s="12" t="str">
-        <x:v>lessons/dont-be-a-hero/level-7.txt</x:v>
+        <x:v>lessons/red-pin-parade/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B34" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C34" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>The Old Book Signal</x:v>
       </x:c>
       <x:c r="E34" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>old-book-signal</x:v>
       </x:c>
       <x:c r="F34" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/old-book-signal/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B35" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C35" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
-        <x:v>The Moon Cup</x:v>
+        <x:v>The Pens in the Water</x:v>
       </x:c>
       <x:c r="E35" s="12" t="str">
-        <x:v>moon-cup</x:v>
+        <x:v>pens-in-water</x:v>
       </x:c>
       <x:c r="F35" s="12" t="str">
-        <x:v>lessons/moon-cup/level-3.txt</x:v>
+        <x:v>lessons/pens-in-water/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B36" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C36" s="12" t="str">
-        <x:v>Fantasy / Adventure</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D36" s="12" t="str">
-        <x:v>The Dice Gate</x:v>
+        <x:v>The Map Under the Stage</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
-        <x:v>dice-gate</x:v>
+        <x:v>map-under-stage</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
-        <x:v>lessons/dice-gate/level-7.txt</x:v>
+        <x:v>lessons/map-under-stage/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B37" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C37" s="12" t="str">
-        <x:v>Human Drama</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D37" s="12" t="str">
-        <x:v>The Quiet Bread Shop</x:v>
+        <x:v>The Door Under the Stage</x:v>
       </x:c>
       <x:c r="E37" s="12" t="str">
-        <x:v>bread-shop</x:v>
+        <x:v>door-under-stage</x:v>
       </x:c>
       <x:c r="F37" s="12" t="str">
-        <x:v>lessons/bread-shop/level-3.txt</x:v>
+        <x:v>lessons/door-under-stage/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH1-1-10-V</x:v>
       </x:c>
       <x:c r="B38" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C38" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D38" s="12" t="str">
-        <x:v>The Gift Lesson</x:v>
+        <x:v>Family Photo Day</x:v>
       </x:c>
       <x:c r="E38" s="12" t="str">
-        <x:v>gift-lesson</x:v>
+        <x:v>family-photo-day</x:v>
       </x:c>
       <x:c r="F38" s="12" t="str">
-        <x:v>lessons/gift-lesson/level-7.txt</x:v>
+        <x:v>lessons/family-photo-day/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B39" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C39" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D39" s="12" t="str">
-        <x:v>The Cake Was Moved</x:v>
+        <x:v>The Letter Under the Door</x:v>
       </x:c>
       <x:c r="E39" s="12" t="str">
-        <x:v>cake-was-moved</x:v>
+        <x:v>letter-under-door</x:v>
       </x:c>
       <x:c r="F39" s="12" t="str">
-        <x:v>lessons/cake-was-moved/level-7.txt</x:v>
+        <x:v>lessons/letter-under-door/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B40" s="12" t="str">
         <x:v>Long</x:v>
@@ -1997,18 +1997,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D40" s="12" t="str">
-        <x:v>The Red Pin Parade</x:v>
+        <x:v>Why the Lights Blink</x:v>
       </x:c>
       <x:c r="E40" s="12" t="str">
-        <x:v>red-pin-parade</x:v>
+        <x:v>why-lights-blink</x:v>
       </x:c>
       <x:c r="F40" s="12" t="str">
-        <x:v>lessons/red-pin-parade/level-7.txt</x:v>
+        <x:v>lessons/why-lights-blink/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B41" s="12" t="str">
         <x:v>Long</x:v>
@@ -2017,18 +2017,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D41" s="12" t="str">
-        <x:v>The Old Book Signal</x:v>
+        <x:v>Because of the Soup</x:v>
       </x:c>
       <x:c r="E41" s="12" t="str">
-        <x:v>old-book-signal</x:v>
+        <x:v>because-of-soup</x:v>
       </x:c>
       <x:c r="F41" s="12" t="str">
-        <x:v>lessons/old-book-signal/level-7.txt</x:v>
+        <x:v>lessons/because-of-soup/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B42" s="12" t="str">
         <x:v>Long</x:v>
@@ -2037,18 +2037,18 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D42" s="12" t="str">
-        <x:v>The Pens in the Water</x:v>
+        <x:v>How to Open the Box</x:v>
       </x:c>
       <x:c r="E42" s="12" t="str">
-        <x:v>pens-in-water</x:v>
+        <x:v>open-the-box</x:v>
       </x:c>
       <x:c r="F42" s="12" t="str">
-        <x:v>lessons/pens-in-water/level-7.txt</x:v>
+        <x:v>lessons/open-the-box/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B43" s="12" t="str">
         <x:v>Long</x:v>
@@ -2057,13 +2057,13 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D43" s="12" t="str">
-        <x:v>The Map Under the Stage</x:v>
+        <x:v>More Than Half</x:v>
       </x:c>
       <x:c r="E43" s="12" t="str">
-        <x:v>map-under-stage</x:v>
+        <x:v>more-than-half</x:v>
       </x:c>
       <x:c r="F43" s="12" t="str">
-        <x:v>lessons/map-under-stage/level-7.txt</x:v>
+        <x:v>lessons/more-than-half/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
@@ -2071,139 +2071,139 @@
         <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B44" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C44" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D44" s="12" t="str">
-        <x:v>The Door Under the Stage</x:v>
+        <x:v>The Travel Ticket</x:v>
       </x:c>
       <x:c r="E44" s="12" t="str">
-        <x:v>door-under-stage</x:v>
+        <x:v>travel-ticket</x:v>
       </x:c>
       <x:c r="F44" s="12" t="str">
-        <x:v>lessons/door-under-stage/level-7.txt</x:v>
+        <x:v>lessons/travel-ticket/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="12" t="str">
-        <x:v>NH1-1-10-V</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B45" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C45" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D45" s="12" t="str">
-        <x:v>Family Photo Day</x:v>
+        <x:v>Maybe at the Window</x:v>
       </x:c>
       <x:c r="E45" s="12" t="str">
-        <x:v>family-photo-day</x:v>
+        <x:v>maybe-window</x:v>
       </x:c>
       <x:c r="F45" s="12" t="str">
-        <x:v>lessons/family-photo-day/level-7.txt</x:v>
+        <x:v>lessons/maybe-window/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B46" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C46" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D46" s="12" t="str">
-        <x:v>The Letter Under the Door</x:v>
+        <x:v>The Should Sign</x:v>
       </x:c>
       <x:c r="E46" s="12" t="str">
-        <x:v>letter-under-door</x:v>
+        <x:v>should-sign</x:v>
       </x:c>
       <x:c r="F46" s="12" t="str">
-        <x:v>lessons/letter-under-door/level-7.txt</x:v>
+        <x:v>lessons/should-sign/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B47" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C47" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D47" s="12" t="str">
-        <x:v>Why the Lights Blink</x:v>
+        <x:v>The Have-To Key</x:v>
       </x:c>
       <x:c r="E47" s="12" t="str">
-        <x:v>why-lights-blink</x:v>
+        <x:v>have-to-key</x:v>
       </x:c>
       <x:c r="F47" s="12" t="str">
-        <x:v>lessons/why-lights-blink/level-7.txt</x:v>
+        <x:v>lessons/have-to-key/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B48" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C48" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D48" s="12" t="str">
-        <x:v>Because of the Soup</x:v>
+        <x:v>The Poster Was Moved</x:v>
       </x:c>
       <x:c r="E48" s="12" t="str">
-        <x:v>because-of-soup</x:v>
+        <x:v>passive-poster</x:v>
       </x:c>
       <x:c r="F48" s="12" t="str">
-        <x:v>lessons/because-of-soup/level-7.txt</x:v>
+        <x:v>lessons/passive-poster/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH1-1-7-V</x:v>
       </x:c>
       <x:c r="B49" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C49" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D49" s="12" t="str">
-        <x:v>How to Open the Box</x:v>
+        <x:v>The Drink and Read Race</x:v>
       </x:c>
       <x:c r="E49" s="12" t="str">
-        <x:v>open-the-box</x:v>
+        <x:v>drink-read-race</x:v>
       </x:c>
       <x:c r="F49" s="12" t="str">
-        <x:v>lessons/open-the-box/level-7.txt</x:v>
+        <x:v>lessons/drink-read-race/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B50" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C50" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
-        <x:v>More Than Half</x:v>
+        <x:v>Can the Lantern Fly?</x:v>
       </x:c>
       <x:c r="E50" s="12" t="str">
-        <x:v>more-than-half</x:v>
+        <x:v>can-lantern</x:v>
       </x:c>
       <x:c r="F50" s="12" t="str">
-        <x:v>lessons/more-than-half/level-7.txt</x:v>
+        <x:v>lessons/can-lantern/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
@@ -2217,253 +2217,253 @@
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D51" s="12" t="str">
-        <x:v>The Travel Ticket</x:v>
+        <x:v>Don't Be Late</x:v>
       </x:c>
       <x:c r="E51" s="12" t="str">
-        <x:v>travel-ticket</x:v>
+        <x:v>dont-be-late</x:v>
       </x:c>
       <x:c r="F51" s="12" t="str">
-        <x:v>lessons/travel-ticket/level-3.txt</x:v>
+        <x:v>lessons/dont-be-late/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B52" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C52" s="12" t="str">
         <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D52" s="12" t="str">
-        <x:v>Maybe at the Window</x:v>
+        <x:v>Show Me the Seat</x:v>
       </x:c>
       <x:c r="E52" s="12" t="str">
-        <x:v>maybe-window</x:v>
+        <x:v>show-me-the-seat</x:v>
       </x:c>
       <x:c r="F52" s="12" t="str">
-        <x:v>lessons/maybe-window/level-3.txt</x:v>
+        <x:v>lessons/show-me-the-seat/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B53" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C53" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
-        <x:v>The Should Sign</x:v>
+        <x:v>The Signal Under Water</x:v>
       </x:c>
       <x:c r="E53" s="12" t="str">
-        <x:v>should-sign</x:v>
+        <x:v>signal-under-water</x:v>
       </x:c>
       <x:c r="F53" s="12" t="str">
-        <x:v>lessons/should-sign/level-3.txt</x:v>
+        <x:v>lessons/signal-under-water/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B54" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C54" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D54" s="12" t="str">
-        <x:v>The Have-To Key</x:v>
+        <x:v>The Orbit Note</x:v>
       </x:c>
       <x:c r="E54" s="12" t="str">
-        <x:v>have-to-key</x:v>
+        <x:v>orbit-note</x:v>
       </x:c>
       <x:c r="F54" s="12" t="str">
-        <x:v>lessons/have-to-key/level-3.txt</x:v>
+        <x:v>lessons/orbit-note/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B55" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C55" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D55" s="12" t="str">
-        <x:v>The Poster Was Moved</x:v>
+        <x:v>Why the Moon Robot Stops</x:v>
       </x:c>
       <x:c r="E55" s="12" t="str">
-        <x:v>passive-poster</x:v>
+        <x:v>why-moon-robot</x:v>
       </x:c>
       <x:c r="F55" s="12" t="str">
-        <x:v>lessons/passive-poster/level-3.txt</x:v>
+        <x:v>lessons/why-moon-robot/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="12" t="str">
-        <x:v>NH1-1-7-V</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B56" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C56" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D56" s="12" t="str">
-        <x:v>The Drink and Read Race</x:v>
+        <x:v>Maybe at the Mars Window</x:v>
       </x:c>
       <x:c r="E56" s="12" t="str">
-        <x:v>drink-read-race</x:v>
+        <x:v>maybe-mars-window</x:v>
       </x:c>
       <x:c r="F56" s="12" t="str">
-        <x:v>lessons/drink-read-race/level-3.txt</x:v>
+        <x:v>lessons/maybe-mars-window/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B57" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C57" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D57" s="12" t="str">
-        <x:v>Can the Lantern Fly?</x:v>
+        <x:v>The Station Was Moved</x:v>
       </x:c>
       <x:c r="E57" s="12" t="str">
-        <x:v>can-lantern</x:v>
+        <x:v>station-was-moved</x:v>
       </x:c>
       <x:c r="F57" s="12" t="str">
-        <x:v>lessons/can-lantern/level-3.txt</x:v>
+        <x:v>lessons/station-was-moved/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B58" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C58" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D58" s="12" t="str">
-        <x:v>Don't Be Late</x:v>
+        <x:v>Where the Roof Door Opens</x:v>
       </x:c>
       <x:c r="E58" s="12" t="str">
-        <x:v>dont-be-late</x:v>
+        <x:v>where-the-roof-door</x:v>
       </x:c>
       <x:c r="F58" s="12" t="str">
-        <x:v>lessons/dont-be-late/level-3.txt</x:v>
+        <x:v>lessons/where-the-roof-door/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B59" s="12" t="str">
         <x:v>Long</x:v>
       </x:c>
       <x:c r="C59" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D59" s="12" t="str">
-        <x:v>Show Me the Seat</x:v>
+        <x:v>The Traveling Shadow Ticket</x:v>
       </x:c>
       <x:c r="E59" s="12" t="str">
-        <x:v>show-me-the-seat</x:v>
+        <x:v>traveling-shadow-ticket</x:v>
       </x:c>
       <x:c r="F59" s="12" t="str">
-        <x:v>lessons/show-me-the-seat/level-7.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60" ht="15" hidden="0" customHeight="1">
+        <x:v>lessons/traveling-shadow-ticket/level-7.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="24" hidden="0" customHeight="1">
       <x:c r="A60" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B60" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C60" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D60" s="12" t="str">
-        <x:v>The Signal Under Water</x:v>
+        <x:v>Because the Wall Listened</x:v>
       </x:c>
       <x:c r="E60" s="12" t="str">
-        <x:v>signal-under-water</x:v>
+        <x:v>because-the-wall-listened</x:v>
       </x:c>
       <x:c r="F60" s="12" t="str">
-        <x:v>lessons/signal-under-water/level-3.txt</x:v>
+        <x:v>lessons/because-the-wall-listened/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B61" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C61" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D61" s="12" t="str">
-        <x:v>The Orbit Note</x:v>
+        <x:v>How to Read the Stone</x:v>
       </x:c>
       <x:c r="E61" s="12" t="str">
-        <x:v>orbit-note</x:v>
+        <x:v>how-to-read-the-stone</x:v>
       </x:c>
       <x:c r="F61" s="12" t="str">
-        <x:v>lessons/orbit-note/level-3.txt</x:v>
+        <x:v>lessons/how-to-read-the-stone/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
       <x:c r="A62" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B62" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Long</x:v>
       </x:c>
       <x:c r="C62" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D62" s="12" t="str">
-        <x:v>Why the Moon Robot Stops</x:v>
+        <x:v>More Than One Moon</x:v>
       </x:c>
       <x:c r="E62" s="12" t="str">
-        <x:v>why-moon-robot</x:v>
+        <x:v>more-than-one-moon</x:v>
       </x:c>
       <x:c r="F62" s="12" t="str">
-        <x:v>lessons/why-moon-robot/level-3.txt</x:v>
+        <x:v>lessons/more-than-one-moon/level-7.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="15" hidden="0" customHeight="1">
       <x:c r="A63" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B63" s="12" t="str">
-        <x:v>Short</x:v>
+        <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C63" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D63" s="12" t="str">
-        <x:v>Maybe at the Mars Window</x:v>
+        <x:v>The Locked Umbrella Room</x:v>
       </x:c>
       <x:c r="E63" s="12" t="str">
-        <x:v>maybe-mars-window</x:v>
+        <x:v>locked-umbrella-room</x:v>
       </x:c>
       <x:c r="F63" s="12" t="str">
-        <x:v>lessons/maybe-mars-window/level-3.txt</x:v>
+        <x:v>lessons/locked-umbrella-room/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
@@ -2471,79 +2471,79 @@
         <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B64" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C64" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D64" s="12" t="str">
-        <x:v>The Station Was Moved</x:v>
+        <x:v>The Last Seat at the Table</x:v>
       </x:c>
       <x:c r="E64" s="12" t="str">
-        <x:v>station-was-moved</x:v>
+        <x:v>last-seat-table</x:v>
       </x:c>
       <x:c r="F64" s="12" t="str">
-        <x:v>lessons/station-was-moved/level-7.txt</x:v>
+        <x:v>lessons/last-seat-table/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
       <x:c r="A65" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B65" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C65" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D65" s="12" t="str">
-        <x:v>Where the Roof Door Opens</x:v>
+        <x:v>The Library That Was Moved</x:v>
       </x:c>
       <x:c r="E65" s="12" t="str">
-        <x:v>where-the-roof-door</x:v>
+        <x:v>library-moved</x:v>
       </x:c>
       <x:c r="F65" s="12" t="str">
-        <x:v>lessons/where-the-roof-door/level-7.txt</x:v>
+        <x:v>lessons/library-moved/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
       <x:c r="A66" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B66" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C66" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D66" s="12" t="str">
-        <x:v>The Traveling Shadow Ticket</x:v>
+        <x:v>The Moon Lantern Path</x:v>
       </x:c>
       <x:c r="E66" s="12" t="str">
-        <x:v>traveling-shadow-ticket</x:v>
+        <x:v>moon-lantern-path</x:v>
       </x:c>
       <x:c r="F66" s="12" t="str">
-        <x:v>lessons/traveling-shadow-ticket/level-7.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67" ht="24" hidden="0" customHeight="1">
+        <x:v>lessons/moon-lantern-path/level-8.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="15" hidden="0" customHeight="1">
       <x:c r="A67" s="12" t="str">
         <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B67" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C67" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D67" s="12" t="str">
-        <x:v>Because the Wall Listened</x:v>
+        <x:v>The Folded Map Race</x:v>
       </x:c>
       <x:c r="E67" s="12" t="str">
-        <x:v>because-the-wall-listened</x:v>
+        <x:v>folded-map-race</x:v>
       </x:c>
       <x:c r="F67" s="12" t="str">
-        <x:v>lessons/because-the-wall-listened/level-7.txt</x:v>
+        <x:v>lessons/folded-map-race/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
@@ -2551,159 +2551,159 @@
         <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B68" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Very Long</x:v>
       </x:c>
       <x:c r="C68" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D68" s="12" t="str">
-        <x:v>How to Read the Stone</x:v>
+        <x:v>The Pudding Case</x:v>
       </x:c>
       <x:c r="E68" s="12" t="str">
-        <x:v>how-to-read-the-stone</x:v>
+        <x:v>jaio-pudding-case</x:v>
       </x:c>
       <x:c r="F68" s="12" t="str">
-        <x:v>lessons/how-to-read-the-stone/level-7.txt</x:v>
+        <x:v>lessons/jaio-pudding-case/level-8.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
       <x:c r="A69" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-7-2-VOICE</x:v>
       </x:c>
       <x:c r="B69" s="12" t="str">
-        <x:v>Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C69" s="12" t="str">
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D69" s="12" t="str">
-        <x:v>More Than One Moon</x:v>
+        <x:v>Another Door Opens</x:v>
       </x:c>
       <x:c r="E69" s="12" t="str">
-        <x:v>more-than-one-moon</x:v>
+        <x:v>another-door-opens</x:v>
       </x:c>
       <x:c r="F69" s="12" t="str">
-        <x:v>lessons/more-than-one-moon/level-7.txt</x:v>
+        <x:v>lessons/another-door-opens/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
       <x:c r="A70" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B70" s="12" t="str">
-        <x:v>Very Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C70" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D70" s="12" t="str">
-        <x:v>The Locked Umbrella Room</x:v>
+        <x:v>Echo on the Moon</x:v>
       </x:c>
       <x:c r="E70" s="12" t="str">
-        <x:v>locked-umbrella-room</x:v>
+        <x:v>echo-on-the-moon</x:v>
       </x:c>
       <x:c r="F70" s="12" t="str">
-        <x:v>lessons/locked-umbrella-room/level-8.txt</x:v>
+        <x:v>lessons/echo-on-the-moon/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="15" hidden="0" customHeight="1">
       <x:c r="A71" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH1-1-6-V</x:v>
       </x:c>
       <x:c r="B71" s="12" t="str">
-        <x:v>Very Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C71" s="12" t="str">
         <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D71" s="12" t="str">
-        <x:v>The Last Seat at the Table</x:v>
+        <x:v>Inside the Kite</x:v>
       </x:c>
       <x:c r="E71" s="12" t="str">
-        <x:v>last-seat-table</x:v>
+        <x:v>inside-the-kite</x:v>
       </x:c>
       <x:c r="F71" s="12" t="str">
-        <x:v>lessons/last-seat-table/level-8.txt</x:v>
+        <x:v>lessons/inside-the-kite/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="15" hidden="0" customHeight="1">
       <x:c r="A72" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B72" s="12" t="str">
-        <x:v>Very Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C72" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D72" s="12" t="str">
-        <x:v>The Library That Was Moved</x:v>
+        <x:v>Jiro's Quiet Joke</x:v>
       </x:c>
       <x:c r="E72" s="12" t="str">
-        <x:v>library-moved</x:v>
+        <x:v>jiro-quiet-joke</x:v>
       </x:c>
       <x:c r="F72" s="12" t="str">
-        <x:v>lessons/library-moved/level-8.txt</x:v>
+        <x:v>lessons/jiro-quiet-joke/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="15" hidden="0" customHeight="1">
       <x:c r="A73" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-5-1-HOW-TO</x:v>
       </x:c>
       <x:c r="B73" s="12" t="str">
-        <x:v>Very Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C73" s="12" t="str">
-        <x:v>Fantasy</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D73" s="12" t="str">
-        <x:v>The Moon Lantern Path</x:v>
+        <x:v>Kaito's Key Map</x:v>
       </x:c>
       <x:c r="E73" s="12" t="str">
-        <x:v>moon-lantern-path</x:v>
+        <x:v>kaito-key-map</x:v>
       </x:c>
       <x:c r="F73" s="12" t="str">
-        <x:v>lessons/moon-lantern-path/level-8.txt</x:v>
+        <x:v>lessons/kaito-key-map/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="15" hidden="0" customHeight="1">
       <x:c r="A74" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-1-3-SVOO</x:v>
       </x:c>
       <x:c r="B74" s="12" t="str">
-        <x:v>Very Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C74" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Fantasy / Adventure</x:v>
       </x:c>
       <x:c r="D74" s="12" t="str">
-        <x:v>The Folded Map Race</x:v>
+        <x:v>Noa and the Night Door</x:v>
       </x:c>
       <x:c r="E74" s="12" t="str">
-        <x:v>folded-map-race</x:v>
+        <x:v>noa-night-door</x:v>
       </x:c>
       <x:c r="F74" s="12" t="str">
-        <x:v>lessons/folded-map-race/level-8.txt</x:v>
+        <x:v>lessons/noa-night-door/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="15" hidden="0" customHeight="1">
       <x:c r="A75" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B75" s="12" t="str">
-        <x:v>Very Long</x:v>
+        <x:v>Short</x:v>
       </x:c>
       <x:c r="C75" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D75" s="12" t="str">
-        <x:v>The Pudding Case</x:v>
+        <x:v>Under the Red Desk</x:v>
       </x:c>
       <x:c r="E75" s="12" t="str">
-        <x:v>jaio-pudding-case</x:v>
+        <x:v>under-red-desk</x:v>
       </x:c>
       <x:c r="F75" s="12" t="str">
-        <x:v>lessons/jaio-pudding-case/level-8.txt</x:v>
+        <x:v>lessons/under-red-desk/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="15" hidden="0" customHeight="1">
@@ -2717,38 +2717,38 @@
         <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D76" s="12" t="str">
-        <x:v>Another Door Opens</x:v>
+        <x:v>Voices in the Wall</x:v>
       </x:c>
       <x:c r="E76" s="12" t="str">
-        <x:v>another-door-opens</x:v>
+        <x:v>voices-in-wall</x:v>
       </x:c>
       <x:c r="F76" s="12" t="str">
-        <x:v>lessons/another-door-opens/level-3.txt</x:v>
+        <x:v>lessons/voices-in-wall/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="15" hidden="0" customHeight="1">
       <x:c r="A77" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
+        <x:v>NH2-2-6-MORE-THAN</x:v>
       </x:c>
       <x:c r="B77" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C77" s="12" t="str">
-        <x:v>SF</x:v>
+        <x:v>Adventure</x:v>
       </x:c>
       <x:c r="D77" s="12" t="str">
-        <x:v>Echo on the Moon</x:v>
+        <x:v>X Marks the Lunch Box</x:v>
       </x:c>
       <x:c r="E77" s="12" t="str">
-        <x:v>echo-on-the-moon</x:v>
+        <x:v>x-marks-lunch-box</x:v>
       </x:c>
       <x:c r="F77" s="12" t="str">
-        <x:v>lessons/echo-on-the-moon/level-3.txt</x:v>
+        <x:v>lessons/x-marks-lunch-box/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="15" hidden="0" customHeight="1">
       <x:c r="A78" s="12" t="str">
-        <x:v>NH1-1-6-V</x:v>
+        <x:v>NH1-1-11-1-MAYBE</x:v>
       </x:c>
       <x:c r="B78" s="12" t="str">
         <x:v>Short</x:v>
@@ -2757,73 +2757,73 @@
         <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D78" s="12" t="str">
-        <x:v>Inside the Kite</x:v>
+        <x:v>Yuna's Thank-You Note</x:v>
       </x:c>
       <x:c r="E78" s="12" t="str">
-        <x:v>inside-the-kite</x:v>
+        <x:v>yuna-thank-you-note</x:v>
       </x:c>
       <x:c r="F78" s="12" t="str">
-        <x:v>lessons/inside-the-kite/level-3.txt</x:v>
+        <x:v>lessons/yuna-thank-you-note/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="15" hidden="0" customHeight="1">
       <x:c r="A79" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
+        <x:v>NH2-2-4-1-HAVE-TO</x:v>
       </x:c>
       <x:c r="B79" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C79" s="12" t="str">
-        <x:v>Comedy</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D79" s="12" t="str">
-        <x:v>Jiro's Quiet Joke</x:v>
+        <x:v>Zero at the Station</x:v>
       </x:c>
       <x:c r="E79" s="12" t="str">
-        <x:v>jiro-quiet-joke</x:v>
+        <x:v>zero-at-station</x:v>
       </x:c>
       <x:c r="F79" s="12" t="str">
-        <x:v>lessons/jiro-quiet-joke/level-3.txt</x:v>
+        <x:v>lessons/zero-at-station/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="15" hidden="0" customHeight="1">
       <x:c r="A80" s="12" t="str">
-        <x:v>NH2-2-5-1-HOW-TO</x:v>
+        <x:v>NH1-1-7-V</x:v>
       </x:c>
       <x:c r="B80" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C80" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>SF</x:v>
       </x:c>
       <x:c r="D80" s="12" t="str">
-        <x:v>Kaito's Key Map</x:v>
+        <x:v>Green Glass Signal</x:v>
       </x:c>
       <x:c r="E80" s="12" t="str">
-        <x:v>kaito-key-map</x:v>
+        <x:v>green-glass-signal</x:v>
       </x:c>
       <x:c r="F80" s="12" t="str">
-        <x:v>lessons/kaito-key-map/level-3.txt</x:v>
+        <x:v>lessons/green-glass-signal/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15" hidden="0" customHeight="1">
       <x:c r="A81" s="12" t="str">
-        <x:v>NH2-2-1-3-SVOO</x:v>
+        <x:v>NH2-2-2-4-BECAUSE</x:v>
       </x:c>
       <x:c r="B81" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C81" s="12" t="str">
-        <x:v>Fantasy / Adventure</x:v>
+        <x:v>Human Drama</x:v>
       </x:c>
       <x:c r="D81" s="12" t="str">
-        <x:v>Noa and the Night Door</x:v>
+        <x:v>Lost Library Card</x:v>
       </x:c>
       <x:c r="E81" s="12" t="str">
-        <x:v>noa-night-door</x:v>
+        <x:v>lost-library-card</x:v>
       </x:c>
       <x:c r="F81" s="12" t="str">
-        <x:v>lessons/noa-night-door/level-3.txt</x:v>
+        <x:v>lessons/lost-library-card/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="15" hidden="0" customHeight="1">
@@ -2834,195 +2834,55 @@
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C82" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Comedy</x:v>
       </x:c>
       <x:c r="D82" s="12" t="str">
-        <x:v>Under the Red Desk</x:v>
+        <x:v>Open on Monday</x:v>
       </x:c>
       <x:c r="E82" s="12" t="str">
-        <x:v>under-red-desk</x:v>
+        <x:v>open-on-monday</x:v>
       </x:c>
       <x:c r="F82" s="12" t="str">
-        <x:v>lessons/under-red-desk/level-3.txt</x:v>
+        <x:v>lessons/open-on-monday/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="15" hidden="0" customHeight="1">
       <x:c r="A83" s="12" t="str">
-        <x:v>NH2-2-7-2-VOICE</x:v>
+        <x:v>NH1-1-7-V</x:v>
       </x:c>
       <x:c r="B83" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C83" s="12" t="str">
-        <x:v>Mystery</x:v>
+        <x:v>Fantasy</x:v>
       </x:c>
       <x:c r="D83" s="12" t="str">
-        <x:v>Voices in the Wall</x:v>
+        <x:v>Paper Star Plan</x:v>
       </x:c>
       <x:c r="E83" s="12" t="str">
-        <x:v>voices-in-wall</x:v>
+        <x:v>paper-star-plan</x:v>
       </x:c>
       <x:c r="F83" s="12" t="str">
-        <x:v>lessons/voices-in-wall/level-3.txt</x:v>
+        <x:v>lessons/paper-star-plan/level-3.txt</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="15" hidden="0" customHeight="1">
       <x:c r="A84" s="12" t="str">
-        <x:v>NH2-2-6-MORE-THAN</x:v>
+        <x:v>NH2-2-3-1-SHOULD</x:v>
       </x:c>
       <x:c r="B84" s="12" t="str">
         <x:v>Short</x:v>
       </x:c>
       <x:c r="C84" s="12" t="str">
-        <x:v>Adventure</x:v>
+        <x:v>Mystery</x:v>
       </x:c>
       <x:c r="D84" s="12" t="str">
-        <x:v>X Marks the Lunch Box</x:v>
+        <x:v>Quiet Question</x:v>
       </x:c>
       <x:c r="E84" s="12" t="str">
-        <x:v>x-marks-lunch-box</x:v>
+        <x:v>quiet-question</x:v>
       </x:c>
       <x:c r="F84" s="12" t="str">
-        <x:v>lessons/x-marks-lunch-box/level-3.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="85" ht="15" hidden="0" customHeight="1">
-      <x:c r="A85" s="12" t="str">
-        <x:v>NH1-1-11-1-MAYBE</x:v>
-      </x:c>
-      <x:c r="B85" s="12" t="str">
-        <x:v>Short</x:v>
-      </x:c>
-      <x:c r="C85" s="12" t="str">
-        <x:v>Human Drama</x:v>
-      </x:c>
-      <x:c r="D85" s="12" t="str">
-        <x:v>Yuna's Thank-You Note</x:v>
-      </x:c>
-      <x:c r="E85" s="12" t="str">
-        <x:v>yuna-thank-you-note</x:v>
-      </x:c>
-      <x:c r="F85" s="12" t="str">
-        <x:v>lessons/yuna-thank-you-note/level-3.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="86" ht="15" hidden="0" customHeight="1">
-      <x:c r="A86" s="12" t="str">
-        <x:v>NH2-2-4-1-HAVE-TO</x:v>
-      </x:c>
-      <x:c r="B86" s="12" t="str">
-        <x:v>Short</x:v>
-      </x:c>
-      <x:c r="C86" s="12" t="str">
-        <x:v>SF</x:v>
-      </x:c>
-      <x:c r="D86" s="12" t="str">
-        <x:v>Zero at the Station</x:v>
-      </x:c>
-      <x:c r="E86" s="12" t="str">
-        <x:v>zero-at-station</x:v>
-      </x:c>
-      <x:c r="F86" s="12" t="str">
-        <x:v>lessons/zero-at-station/level-3.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="87" ht="15" hidden="0" customHeight="1">
-      <x:c r="A87" s="12" t="str">
-        <x:v>NH1-1-7-V</x:v>
-      </x:c>
-      <x:c r="B87" s="12" t="str">
-        <x:v>Short</x:v>
-      </x:c>
-      <x:c r="C87" s="12" t="str">
-        <x:v>SF</x:v>
-      </x:c>
-      <x:c r="D87" s="12" t="str">
-        <x:v>Green Glass Signal</x:v>
-      </x:c>
-      <x:c r="E87" s="12" t="str">
-        <x:v>green-glass-signal</x:v>
-      </x:c>
-      <x:c r="F87" s="12" t="str">
-        <x:v>lessons/green-glass-signal/level-3.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="88" ht="15" hidden="0" customHeight="1">
-      <x:c r="A88" s="12" t="str">
-        <x:v>NH2-2-2-4-BECAUSE</x:v>
-      </x:c>
-      <x:c r="B88" s="12" t="str">
-        <x:v>Short</x:v>
-      </x:c>
-      <x:c r="C88" s="12" t="str">
-        <x:v>Human Drama</x:v>
-      </x:c>
-      <x:c r="D88" s="12" t="str">
-        <x:v>Lost Library Card</x:v>
-      </x:c>
-      <x:c r="E88" s="12" t="str">
-        <x:v>lost-library-card</x:v>
-      </x:c>
-      <x:c r="F88" s="12" t="str">
-        <x:v>lessons/lost-library-card/level-3.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="89" ht="15" hidden="0" customHeight="1">
-      <x:c r="A89" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
-      </x:c>
-      <x:c r="B89" s="12" t="str">
-        <x:v>Short</x:v>
-      </x:c>
-      <x:c r="C89" s="12" t="str">
-        <x:v>Comedy</x:v>
-      </x:c>
-      <x:c r="D89" s="12" t="str">
-        <x:v>Open on Monday</x:v>
-      </x:c>
-      <x:c r="E89" s="12" t="str">
-        <x:v>open-on-monday</x:v>
-      </x:c>
-      <x:c r="F89" s="12" t="str">
-        <x:v>lessons/open-on-monday/level-3.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="90" ht="15" hidden="0" customHeight="1">
-      <x:c r="A90" s="12" t="str">
-        <x:v>NH1-1-7-V</x:v>
-      </x:c>
-      <x:c r="B90" s="12" t="str">
-        <x:v>Short</x:v>
-      </x:c>
-      <x:c r="C90" s="12" t="str">
-        <x:v>Fantasy</x:v>
-      </x:c>
-      <x:c r="D90" s="12" t="str">
-        <x:v>Paper Star Plan</x:v>
-      </x:c>
-      <x:c r="E90" s="12" t="str">
-        <x:v>paper-star-plan</x:v>
-      </x:c>
-      <x:c r="F90" s="12" t="str">
-        <x:v>lessons/paper-star-plan/level-3.txt</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="91" ht="15" hidden="0" customHeight="1">
-      <x:c r="A91" s="12" t="str">
-        <x:v>NH2-2-3-1-SHOULD</x:v>
-      </x:c>
-      <x:c r="B91" s="12" t="str">
-        <x:v>Short</x:v>
-      </x:c>
-      <x:c r="C91" s="12" t="str">
-        <x:v>Mystery</x:v>
-      </x:c>
-      <x:c r="D91" s="12" t="str">
-        <x:v>Quiet Question</x:v>
-      </x:c>
-      <x:c r="E91" s="12" t="str">
-        <x:v>quiet-question</x:v>
-      </x:c>
-      <x:c r="F91" s="12" t="str">
         <x:v>lessons/quiet-question/level-3.txt</x:v>
       </x:c>
     </x:row>
@@ -3081,7 +2941,7 @@
         <x:v>本文量</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>{Length} で生成する。Very Shortはごく短い導入、Shortは120〜180語程度、Longは300〜450語程度、Very Longは650〜900語程度。</x:v>
+        <x:v>{Length} で生成する。Shortは120〜180語程度、Longは300〜450語程度、Very Longは650〜900語程度。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Rename reading ID label to Grade
</commit_message>
<xml_diff>
--- a/outputs/progress-map/unified_current_id_story_map.xlsx
+++ b/outputs/progress-map/unified_current_id_story_map.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="Ra8f40eb5d7194df3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="Rb82c59b5f0df4f83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="R746569450e604acc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R53414046d44746d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="R75d70dcb25e44385"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_To_Use" sheetId="1" r:id="R3450ddc0cb4d48b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story_Request" sheetId="2" r:id="R099f8e10ae414af2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified_Progress" sheetId="3" r:id="Rd4edd39bddfb42f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content_Map" sheetId="4" r:id="R89ca25df4e874885"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt_Template" sheetId="5" r:id="Rb3db748751f444d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -357,18 +357,18 @@
   <x:sheetData>
     <x:row r="1" ht="19.200000762939453" hidden="0" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>Unified ID 方針</x:v>
+        <x:v>Unified Grade 方針</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>Unified ID 方針</x:v>
+        <x:v>Unified Grade 方針</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のIDを一本で指定する。本文量はShort / Long / Very Longから選ぶ。</x:v>
+        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のGradeを一本で指定する。本文量はShort / Long / Very Longから選ぶ。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のIDを一本で指定する。本文量はShort / Long / Very Longから選ぶ。</x:v>
+        <x:v>GDMは41-10までを橋渡しとして使い、その後はNH1、NH2のGradeを一本で指定する。本文量はShort / Long / Very Longから選ぶ。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -382,10 +382,10 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>ID</x:v>
+        <x:v>Grade</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>GDMとNHを別々に指定しない。ひとつのIDだけを指定する。</x:v>
+        <x:v>GDMとNHを別々に指定しない。ひとつのGradeだけを指定する。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -401,7 +401,7 @@
         <x:v>候補表示</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>サイトでは選択したID以下の近いIDに紐づくコンテンツを最大3件まで表示する。</x:v>
+        <x:v>サイトでは選択したGrade以下の近いGradeに紐づくコンテンツを最大3件まで表示する。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -417,7 +417,7 @@
         <x:v>注意</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>各Lengthは別IDへ紐づける。個別IDの必須語・文法を完全反映する新作本文は今後追加する。</x:v>
+        <x:v>各Lengthは別Gradeへ紐づける。個別Gradeの必須語・文法を完全反映する新作本文は今後追加する。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -455,16 +455,16 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、Lengthで本文量を選ぶ。</x:v>
+        <x:v>本文生成時に使う入力欄。Gradeは1つだけ指定し、Lengthで本文量を選ぶ。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、Lengthで本文量を選ぶ。</x:v>
+        <x:v>本文生成時に使う入力欄。Gradeは1つだけ指定し、Lengthで本文量を選ぶ。</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、Lengthで本文量を選ぶ。</x:v>
+        <x:v>本文生成時に使う入力欄。Gradeは1つだけ指定し、Lengthで本文量を選ぶ。</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>本文生成時に使う入力欄。IDは1つだけ指定し、Lengthで本文量を選ぶ。</x:v>
+        <x:v>本文生成時に使う入力欄。Gradeは1つだけ指定し、Lengthで本文量を選ぶ。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -484,16 +484,16 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>ID</x:v>
+        <x:v>Grade</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
         <x:v>NH1-1-8-3-WHY</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>Unified_ProgressのIDから選ぶ</x:v>
+        <x:v>Unified_ProgressのGradeから選ぶ</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>このIDまでのGDM/NH項目を使用可</x:v>
+        <x:v>このGradeまでのGDM/NH項目を使用可</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -609,34 +609,34 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Gradeの進行表。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Gradeの進行表。</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Gradeの進行表。</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Gradeの進行表。</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Gradeの進行表。</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Gradeの進行表。</x:v>
       </x:c>
       <x:c r="G2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Gradeの進行表。</x:v>
       </x:c>
       <x:c r="H2" s="7" t="str">
-        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一IDの進行表。</x:v>
+        <x:v>GDM合流点以降はNHを中心にNH2まで進める、単一Gradeの進行表。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="16" t="str">
-        <x:v>ID</x:v>
+        <x:v>Grade</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
         <x:v>Series</x:v>
@@ -1247,28 +1247,28 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>既存本文をIDへ紐づけ、Length別に選べるようにした表。LengthごとにIDで管理する。</x:v>
+        <x:v>既存本文をGradeへ紐づけ、Length別に選べるようにした表。LengthごとにGradeで管理する。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>既存本文をIDへ紐づけ、Length別に選べるようにした表。LengthごとにIDで管理する。</x:v>
+        <x:v>既存本文をGradeへ紐づけ、Length別に選べるようにした表。LengthごとにGradeで管理する。</x:v>
       </x:c>
       <x:c r="C2" s="7" t="str">
-        <x:v>既存本文をIDへ紐づけ、Length別に選べるようにした表。LengthごとにIDで管理する。</x:v>
+        <x:v>既存本文をGradeへ紐づけ、Length別に選べるようにした表。LengthごとにGradeで管理する。</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>既存本文をIDへ紐づけ、Length別に選べるようにした表。LengthごとにIDで管理する。</x:v>
+        <x:v>既存本文をGradeへ紐づけ、Length別に選べるようにした表。LengthごとにGradeで管理する。</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>既存本文をIDへ紐づけ、Length別に選べるようにした表。LengthごとにIDで管理する。</x:v>
+        <x:v>既存本文をGradeへ紐づけ、Length別に選べるようにした表。LengthごとにGradeで管理する。</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
-        <x:v>既存本文をIDへ紐づけ、Length別に選べるようにした表。LengthごとにIDで管理する。</x:v>
+        <x:v>既存本文をGradeへ紐づけ、Length別に選べるようにした表。LengthごとにGradeで管理する。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="16" t="str">
-        <x:v>ID</x:v>
+        <x:v>Grade</x:v>
       </x:c>
       <x:c r="B4" s="16" t="str">
         <x:v>Length</x:v>
@@ -2913,10 +2913,10 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>生成時はIDを1つだけ使い、本文量をLengthで指定する。</x:v>
+        <x:v>生成時はGradeを1つだけ使い、本文量をLengthで指定する。</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>生成時はIDを1つだけ使い、本文量をLengthで指定する。</x:v>
+        <x:v>生成時はGradeを1つだけ使い、本文量をLengthで指定する。</x:v>
       </x:c>
     </x:row>
     <x:row r="3"/>
@@ -2933,7 +2933,7 @@
         <x:v>生成指示</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>IDは {ID}。GDM-41-10まではGDMを使い、以降はNH1/NH2の進行順に沿って、このIDまでの語彙・文法を使用する。</x:v>
+        <x:v>Gradeは {Grade}。GDM-41-10まではGDMを使い、以降はNH1/NH2の進行順に沿って、このGradeまでの語彙・文法を使用する。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2949,7 +2949,7 @@
         <x:v>必須項目</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>指定されたIDそのものの導入語・文法は本文に必ず自然に入れる。</x:v>
+        <x:v>指定されたGradeそのものの導入語・文法は本文に必ず自然に入れる。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -2965,7 +2965,7 @@
         <x:v>出力</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Title / ID / Length / Genre / English text / used target items memo</x:v>
+        <x:v>Title / Grade / Length / Genre / English text / used target items memo</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>